<commit_message>
Update NHL stats 2026-10-22 02:53 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -2031,111 +2031,111 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Seattle Kraken</t>
+          <t>Ottawa Senators</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>OTT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>10</v>
       </c>
       <c r="F10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G10" t="n">
         <v>3</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J10" s="1" t="n">
-        <v>0.65</v>
+        <v>0.7</v>
       </c>
       <c r="K10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="N10" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="O10" t="n">
         <v>5</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>3.4</v>
+        <v>2.4</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>26.5</v>
+        <v>23.8</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>31</v>
+        <v>25.5</v>
       </c>
       <c r="T10" s="1" t="n">
-        <v>0.21875</v>
+        <v>0.130434</v>
       </c>
       <c r="U10" s="1" t="n">
-        <v>0.7241379999999999</v>
+        <v>0.794872</v>
       </c>
       <c r="V10" s="1" t="n">
-        <v>0.519736</v>
+        <v>0.524221</v>
       </c>
       <c r="W10" s="1" t="n">
-        <v>0.43788</v>
+        <v>0.4521</v>
       </c>
       <c r="X10" s="1" t="n">
-        <v>0.44142</v>
+        <v>0.46489</v>
       </c>
       <c r="Y10" s="1" t="n">
-        <v>0.48945</v>
+        <v>0.42384</v>
       </c>
       <c r="Z10" s="1" t="n">
-        <v>0.14084</v>
+        <v>0.11042</v>
       </c>
       <c r="AA10" s="1" t="n">
-        <v>0.90946</v>
+        <v>0.92178</v>
       </c>
       <c r="AB10" s="3" t="n">
-        <v>1.0503</v>
+        <v>1.0322</v>
       </c>
       <c r="AC10" s="1" t="n">
-        <v>0.43788</v>
+        <v>0.45833</v>
       </c>
       <c r="AD10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AE10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF10" t="n">
         <v>1</v>
@@ -2144,44 +2144,44 @@
         <v>0</v>
       </c>
       <c r="AH10" t="n">
+        <v>14</v>
+      </c>
+      <c r="AI10" t="n">
         <v>12</v>
       </c>
-      <c r="AI10" t="n">
-        <v>10</v>
-      </c>
       <c r="AJ10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>15</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>12</v>
+      </c>
+      <c r="AP10" t="n">
         <v>7</v>
       </c>
-      <c r="AK10" t="n">
-        <v>4</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>27</v>
-      </c>
-      <c r="AO10" t="n">
+      <c r="AQ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>29</v>
+      </c>
+      <c r="AT10" t="n">
         <v>24</v>
       </c>
-      <c r="AP10" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>3</v>
-      </c>
-      <c r="AR10" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS10" t="n">
-        <v>39</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>34</v>
-      </c>
       <c r="AU10" t="inlineStr">
         <is>
           <t>W1</t>
@@ -2189,33 +2189,33 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ottawa Senators</t>
+          <t>Seattle Kraken</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OTT</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
         <v>6</v>
@@ -2224,106 +2224,106 @@
         <v>3</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" t="n">
+        <v>13</v>
+      </c>
+      <c r="J11" s="1" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4</v>
+      </c>
+      <c r="L11" t="n">
+        <v>4</v>
+      </c>
+      <c r="M11" t="n">
+        <v>39</v>
+      </c>
+      <c r="N11" t="n">
+        <v>34</v>
+      </c>
+      <c r="O11" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="T11" s="1" t="n">
+        <v>0.21875</v>
+      </c>
+      <c r="U11" s="1" t="n">
+        <v>0.7241379999999999</v>
+      </c>
+      <c r="V11" s="1" t="n">
+        <v>0.519736</v>
+      </c>
+      <c r="W11" s="1" t="n">
+        <v>0.43788</v>
+      </c>
+      <c r="X11" s="1" t="n">
+        <v>0.44142</v>
+      </c>
+      <c r="Y11" s="1" t="n">
+        <v>0.48945</v>
+      </c>
+      <c r="Z11" s="1" t="n">
+        <v>0.14084</v>
+      </c>
+      <c r="AA11" s="1" t="n">
+        <v>0.90946</v>
+      </c>
+      <c r="AB11" s="3" t="n">
+        <v>1.0503</v>
+      </c>
+      <c r="AC11" s="1" t="n">
+        <v>0.43788</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="n">
         <v>12</v>
       </c>
-      <c r="J11" s="1" t="n">
-        <v>0.666667</v>
-      </c>
-      <c r="K11" t="n">
-        <v>4</v>
-      </c>
-      <c r="L11" t="n">
-        <v>4</v>
-      </c>
-      <c r="M11" t="n">
+      <c r="AI11" t="n">
+        <v>10</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>27</v>
+      </c>
+      <c r="AO11" t="n">
         <v>24</v>
-      </c>
-      <c r="N11" t="n">
-        <v>23</v>
-      </c>
-      <c r="O11" t="n">
-        <v>1</v>
-      </c>
-      <c r="P11" s="2" t="n">
-        <v>2.6667</v>
-      </c>
-      <c r="Q11" s="2" t="n">
-        <v>2.5556</v>
-      </c>
-      <c r="R11" s="2" t="n">
-        <v>23.11111</v>
-      </c>
-      <c r="S11" s="2" t="n">
-        <v>26.22222</v>
-      </c>
-      <c r="T11" s="1" t="n">
-        <v>0.128205</v>
-      </c>
-      <c r="U11" s="1" t="n">
-        <v>0.794118</v>
-      </c>
-      <c r="V11" s="1" t="n">
-        <v>0.514285</v>
-      </c>
-      <c r="W11" s="1" t="n">
-        <v>0.44351</v>
-      </c>
-      <c r="X11" s="1" t="n">
-        <v>0.45041</v>
-      </c>
-      <c r="Y11" s="1" t="n">
-        <v>0.41787</v>
-      </c>
-      <c r="Z11" s="1" t="n">
-        <v>0.09722</v>
-      </c>
-      <c r="AA11" s="1" t="n">
-        <v>0.91666</v>
-      </c>
-      <c r="AB11" s="3" t="n">
-        <v>1.01388</v>
-      </c>
-      <c r="AC11" s="1" t="n">
-        <v>0.45161</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH11" t="n">
-        <v>9</v>
-      </c>
-      <c r="AI11" t="n">
-        <v>11</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>15</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>12</v>
       </c>
       <c r="AP11" t="n">
         <v>6</v>
@@ -2332,22 +2332,22 @@
         <v>3</v>
       </c>
       <c r="AR11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS11" t="n">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="AT11" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -2373,13 +2373,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
         <v>5</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
@@ -2388,7 +2388,7 @@
         <v>12</v>
       </c>
       <c r="J12" s="1" t="n">
-        <v>0.666667</v>
+        <v>0.6</v>
       </c>
       <c r="K12" t="n">
         <v>3</v>
@@ -2397,55 +2397,55 @@
         <v>5</v>
       </c>
       <c r="M12" t="n">
+        <v>31</v>
+      </c>
+      <c r="N12" t="n">
         <v>30</v>
       </c>
-      <c r="N12" t="n">
-        <v>25</v>
-      </c>
       <c r="O12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>3.3333</v>
+        <v>3.1</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>2.7778</v>
+        <v>3</v>
       </c>
       <c r="R12" s="2" t="n">
-        <v>29.33333</v>
+        <v>28.3</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>24</v>
+        <v>24.6</v>
       </c>
       <c r="T12" s="1" t="n">
-        <v>0.209302</v>
+        <v>0.208333</v>
       </c>
       <c r="U12" s="1" t="n">
-        <v>0.805556</v>
+        <v>0.813954</v>
       </c>
       <c r="V12" s="1" t="n">
-        <v>0.463551</v>
+        <v>0.455782</v>
       </c>
       <c r="W12" s="1" t="n">
-        <v>0.57402</v>
+        <v>0.56393</v>
       </c>
       <c r="X12" s="1" t="n">
-        <v>0.56116</v>
+        <v>0.54659</v>
       </c>
       <c r="Y12" s="1" t="n">
-        <v>0.59574</v>
+        <v>0.58874</v>
       </c>
       <c r="Z12" s="1" t="n">
-        <v>0.09195</v>
+        <v>0.08648</v>
       </c>
       <c r="AA12" s="1" t="n">
-        <v>0.90277</v>
+        <v>0.88957</v>
       </c>
       <c r="AB12" s="3" t="n">
-        <v>0.99472</v>
+        <v>0.97605</v>
       </c>
       <c r="AC12" s="1" t="n">
-        <v>0.58771</v>
+        <v>0.57786</v>
       </c>
       <c r="AD12" t="n">
         <v>3</v>
@@ -2466,46 +2466,46 @@
         <v>9</v>
       </c>
       <c r="AJ12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AK12" t="n">
         <v>3</v>
       </c>
       <c r="AL12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM12" t="n">
         <v>2</v>
       </c>
       <c r="AN12" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AO12" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="AP12" t="n">
         <v>5</v>
       </c>
       <c r="AQ12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR12" t="n">
         <v>2</v>
       </c>
       <c r="AS12" t="n">
+        <v>31</v>
+      </c>
+      <c r="AT12" t="n">
         <v>30</v>
       </c>
-      <c r="AT12" t="n">
-        <v>25</v>
-      </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -3769,19 +3769,19 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Buffalo Sabres</t>
+          <t>Montréal Canadiens</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3813,64 +3813,64 @@
         <v>0.555556</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M21" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="N21" t="n">
         <v>34</v>
       </c>
       <c r="O21" t="n">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="P21" s="2" t="n">
-        <v>3</v>
+        <v>3.3333</v>
       </c>
       <c r="Q21" s="2" t="n">
         <v>3.7778</v>
       </c>
       <c r="R21" s="2" t="n">
-        <v>26.77777</v>
+        <v>29.66666</v>
       </c>
       <c r="S21" s="2" t="n">
-        <v>25.66666</v>
+        <v>26.33333</v>
       </c>
       <c r="T21" s="1" t="n">
-        <v>0.090909</v>
+        <v>0.137931</v>
       </c>
       <c r="U21" s="1" t="n">
-        <v>0.645162</v>
+        <v>0.783784</v>
       </c>
       <c r="V21" s="1" t="n">
-        <v>0.461824</v>
+        <v>0.525423</v>
       </c>
       <c r="W21" s="1" t="n">
-        <v>0.52727</v>
+        <v>0.56701</v>
       </c>
       <c r="X21" s="1" t="n">
-        <v>0.5222</v>
+        <v>0.55789</v>
       </c>
       <c r="Y21" s="1" t="n">
-        <v>0.49259</v>
+        <v>0.57046</v>
       </c>
       <c r="Z21" s="1" t="n">
-        <v>0.10106</v>
+        <v>0.09182999999999999</v>
       </c>
       <c r="AA21" s="1" t="n">
-        <v>0.87577</v>
+        <v>0.88235</v>
       </c>
       <c r="AB21" s="3" t="n">
-        <v>0.97683</v>
+        <v>0.97418</v>
       </c>
       <c r="AC21" s="1" t="n">
-        <v>0.52059</v>
+        <v>0.5641</v>
       </c>
       <c r="AD21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE21" t="n">
         <v>3</v>
@@ -3879,32 +3879,32 @@
         <v>2</v>
       </c>
       <c r="AG21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH21" t="n">
+        <v>18</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>21</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>12</v>
+      </c>
+      <c r="AO21" t="n">
         <v>13</v>
       </c>
-      <c r="AI21" t="n">
-        <v>16</v>
-      </c>
-      <c r="AJ21" t="n">
-        <v>4</v>
-      </c>
-      <c r="AK21" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL21" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM21" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN21" t="n">
-        <v>14</v>
-      </c>
-      <c r="AO21" t="n">
-        <v>18</v>
-      </c>
       <c r="AP21" t="n">
         <v>4</v>
       </c>
@@ -3915,7 +3915,7 @@
         <v>2</v>
       </c>
       <c r="AS21" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="AT21" t="n">
         <v>34</v>
@@ -3927,19 +3927,19 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Montréal Canadiens</t>
+          <t>Buffalo Sabres</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MTL</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3953,13 +3953,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F22" t="n">
         <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H22" t="n">
         <v>2</v>
@@ -3968,64 +3968,64 @@
         <v>10</v>
       </c>
       <c r="J22" s="1" t="n">
-        <v>0.555556</v>
+        <v>0.5</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M22" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N22" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="O22" t="n">
-        <v>-4</v>
+        <v>-9</v>
       </c>
       <c r="P22" s="2" t="n">
-        <v>3.3333</v>
+        <v>2.8</v>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>3.7778</v>
+        <v>3.7</v>
       </c>
       <c r="R22" s="2" t="n">
-        <v>29.66666</v>
+        <v>26.9</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>26.33333</v>
+        <v>25.7</v>
       </c>
       <c r="T22" s="1" t="n">
-        <v>0.137931</v>
+        <v>0.111111</v>
       </c>
       <c r="U22" s="1" t="n">
-        <v>0.783784</v>
+        <v>0.666667</v>
       </c>
       <c r="V22" s="1" t="n">
-        <v>0.525423</v>
+        <v>0.470085</v>
       </c>
       <c r="W22" s="1" t="n">
-        <v>0.56701</v>
+        <v>0.52606</v>
       </c>
       <c r="X22" s="1" t="n">
-        <v>0.55789</v>
+        <v>0.5211</v>
       </c>
       <c r="Y22" s="1" t="n">
-        <v>0.57046</v>
+        <v>0.49477</v>
       </c>
       <c r="Z22" s="1" t="n">
-        <v>0.09182999999999999</v>
+        <v>0.09268</v>
       </c>
       <c r="AA22" s="1" t="n">
-        <v>0.88235</v>
+        <v>0.8764</v>
       </c>
       <c r="AB22" s="3" t="n">
-        <v>0.97418</v>
+        <v>0.9690800000000001</v>
       </c>
       <c r="AC22" s="1" t="n">
-        <v>0.5641</v>
+        <v>0.51557</v>
       </c>
       <c r="AD22" t="n">
         <v>6</v>
@@ -4034,58 +4034,58 @@
         <v>3</v>
       </c>
       <c r="AF22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH22" t="n">
+        <v>14</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>19</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>14</v>
+      </c>
+      <c r="AO22" t="n">
         <v>18</v>
       </c>
-      <c r="AI22" t="n">
-        <v>21</v>
-      </c>
-      <c r="AJ22" t="n">
-        <v>3</v>
-      </c>
-      <c r="AK22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN22" t="n">
-        <v>12</v>
-      </c>
-      <c r="AO22" t="n">
-        <v>13</v>
-      </c>
       <c r="AP22" t="n">
         <v>4</v>
       </c>
       <c r="AQ22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR22" t="n">
         <v>2</v>
       </c>
       <c r="AS22" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="AT22" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="AU22" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -4559,315 +4559,315 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Anaheim Ducks</t>
+          <t>Philadelphia Flyers</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ANA</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E26" t="n">
+        <v>12</v>
+      </c>
+      <c r="F26" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" t="n">
         <v>9</v>
       </c>
-      <c r="F26" t="n">
-        <v>4</v>
-      </c>
-      <c r="G26" t="n">
-        <v>5</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>8</v>
-      </c>
       <c r="J26" s="1" t="n">
-        <v>0.444444</v>
+        <v>0.375</v>
       </c>
       <c r="K26" t="n">
         <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M26" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="N26" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="O26" t="n">
-        <v>-3</v>
+        <v>-17</v>
       </c>
       <c r="P26" s="2" t="n">
-        <v>2.8889</v>
+        <v>1.6667</v>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>3.2222</v>
+        <v>3.0833</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>24.11111</v>
+        <v>21.83333</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>26.55555</v>
+        <v>31.91666</v>
       </c>
       <c r="T26" s="1" t="n">
-        <v>0.225806</v>
+        <v>0.138888</v>
       </c>
       <c r="U26" s="1" t="n">
-        <v>0.787879</v>
+        <v>0.833334</v>
       </c>
       <c r="V26" s="1" t="n">
-        <v>0.43217</v>
+        <v>0.509246</v>
       </c>
       <c r="W26" s="1" t="n">
-        <v>0.48104</v>
+        <v>0.41227</v>
       </c>
       <c r="X26" s="1" t="n">
-        <v>0.48469</v>
+        <v>0.39664</v>
       </c>
       <c r="Y26" s="1" t="n">
-        <v>0.46393</v>
+        <v>0.40745</v>
       </c>
       <c r="Z26" s="1" t="n">
-        <v>0.08522</v>
+        <v>0.06349</v>
       </c>
       <c r="AA26" s="1" t="n">
-        <v>0.89617</v>
+        <v>0.91245</v>
       </c>
       <c r="AB26" s="3" t="n">
-        <v>0.98139</v>
+        <v>0.97594</v>
       </c>
       <c r="AC26" s="1" t="n">
-        <v>0.498</v>
+        <v>0.39215</v>
       </c>
       <c r="AD26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AE26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AH26" t="n">
+        <v>11</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>20</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN26" t="n">
         <v>9</v>
       </c>
-      <c r="AI26" t="n">
-        <v>15</v>
-      </c>
-      <c r="AJ26" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL26" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN26" t="n">
+      <c r="AO26" t="n">
         <v>17</v>
       </c>
-      <c r="AO26" t="n">
-        <v>14</v>
-      </c>
       <c r="AP26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AQ26" t="n">
         <v>5</v>
       </c>
       <c r="AR26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS26" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="AT26" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="AU26" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pittsburgh Penguins</t>
+          <t>Anaheim Ducks</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>ANA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J27" s="1" t="n">
-        <v>0.35</v>
+        <v>0.444444</v>
       </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M27" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="N27" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="O27" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="P27" s="2" t="n">
-        <v>3.3</v>
+        <v>2.8889</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>3.8</v>
+        <v>3.2222</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>27.4</v>
+        <v>24.11111</v>
       </c>
       <c r="S27" s="2" t="n">
-        <v>27.8</v>
+        <v>26.55555</v>
       </c>
       <c r="T27" s="1" t="n">
-        <v>0.233333</v>
+        <v>0.225806</v>
       </c>
       <c r="U27" s="1" t="n">
-        <v>0.807693</v>
+        <v>0.787879</v>
       </c>
       <c r="V27" s="1" t="n">
-        <v>0.446236</v>
+        <v>0.43217</v>
       </c>
       <c r="W27" s="1" t="n">
-        <v>0.50781</v>
+        <v>0.48104</v>
       </c>
       <c r="X27" s="1" t="n">
-        <v>0.51588</v>
+        <v>0.48469</v>
       </c>
       <c r="Y27" s="1" t="n">
-        <v>0.48703</v>
+        <v>0.46393</v>
       </c>
       <c r="Z27" s="1" t="n">
-        <v>0.1055</v>
+        <v>0.08522</v>
       </c>
       <c r="AA27" s="1" t="n">
-        <v>0.87793</v>
+        <v>0.89617</v>
       </c>
       <c r="AB27" s="3" t="n">
-        <v>0.98343</v>
+        <v>0.98139</v>
       </c>
       <c r="AC27" s="1" t="n">
-        <v>0.54577</v>
+        <v>0.498</v>
       </c>
       <c r="AD27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AG27" t="n">
         <v>0</v>
       </c>
       <c r="AH27" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AI27" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="AJ27" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AK27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AL27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>17</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>14</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>4</v>
+      </c>
+      <c r="AQ27" t="n">
         <v>5</v>
       </c>
-      <c r="AM27" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN27" t="n">
-        <v>23</v>
-      </c>
-      <c r="AO27" t="n">
+      <c r="AR27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>26</v>
+      </c>
+      <c r="AT27" t="n">
         <v>29</v>
       </c>
-      <c r="AP27" t="n">
-        <v>3</v>
-      </c>
-      <c r="AQ27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AR27" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS27" t="n">
-        <v>33</v>
-      </c>
-      <c r="AT27" t="n">
-        <v>38</v>
-      </c>
       <c r="AU27" t="inlineStr">
         <is>
           <t>L4</t>
@@ -4875,19 +4875,19 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Philadelphia Flyers</t>
+          <t>Pittsburgh Penguins</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4901,139 +4901,139 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G28" t="n">
         <v>6</v>
       </c>
       <c r="H28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
         <v>7</v>
       </c>
       <c r="J28" s="1" t="n">
-        <v>0.318182</v>
+        <v>0.35</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
         <v>2</v>
       </c>
       <c r="M28" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="N28" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O28" t="n">
-        <v>-19</v>
+        <v>-5</v>
       </c>
       <c r="P28" s="2" t="n">
-        <v>1.5455</v>
+        <v>3.3</v>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>3.2727</v>
+        <v>3.8</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>21.45454</v>
+        <v>27.4</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>32.27272</v>
+        <v>27.8</v>
       </c>
       <c r="T28" s="1" t="n">
-        <v>0.129032</v>
+        <v>0.233333</v>
       </c>
       <c r="U28" s="1" t="n">
-        <v>0.846154</v>
+        <v>0.807693</v>
       </c>
       <c r="V28" s="1" t="n">
-        <v>0.514503</v>
+        <v>0.446236</v>
       </c>
       <c r="W28" s="1" t="n">
-        <v>0.4066</v>
+        <v>0.50781</v>
       </c>
       <c r="X28" s="1" t="n">
-        <v>0.38914</v>
+        <v>0.51588</v>
       </c>
       <c r="Y28" s="1" t="n">
-        <v>0.40434</v>
+        <v>0.48703</v>
       </c>
       <c r="Z28" s="1" t="n">
-        <v>0.05813</v>
+        <v>0.1055</v>
       </c>
       <c r="AA28" s="1" t="n">
-        <v>0.9071399999999999</v>
+        <v>0.87793</v>
       </c>
       <c r="AB28" s="3" t="n">
-        <v>0.96527</v>
+        <v>0.98343</v>
       </c>
       <c r="AC28" s="1" t="n">
-        <v>0.38208</v>
+        <v>0.54577</v>
       </c>
       <c r="AD28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>9</v>
+      </c>
+      <c r="AJ28" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>23</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>29</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AQ28" t="n">
         <v>6</v>
       </c>
-      <c r="AE28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH28" t="n">
-        <v>11</v>
-      </c>
-      <c r="AI28" t="n">
-        <v>20</v>
-      </c>
-      <c r="AJ28" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL28" t="n">
-        <v>4</v>
-      </c>
-      <c r="AM28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN28" t="n">
-        <v>6</v>
-      </c>
-      <c r="AO28" t="n">
-        <v>16</v>
-      </c>
-      <c r="AP28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AQ28" t="n">
-        <v>5</v>
-      </c>
       <c r="AR28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AS28" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="AT28" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="AU28" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>L4</t>
         </is>
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-21 16:42</t>
+          <t>2026-10-22 02:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-22 08:16 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-22 02:53</t>
+          <t>2026-10-22 08:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-23 08:11 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-23 02:52</t>
+          <t>2026-10-23 08:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-24 02:49 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -847,13 +847,13 @@
         <v>0.501408</v>
       </c>
       <c r="W2" s="1" t="n">
-        <v>0.59396</v>
+        <v>0.59454</v>
       </c>
       <c r="X2" s="1" t="n">
-        <v>0.60686</v>
+        <v>0.60766</v>
       </c>
       <c r="Y2" s="1" t="n">
-        <v>0.59307</v>
+        <v>0.59393</v>
       </c>
       <c r="Z2" s="1" t="n">
         <v>0.10333</v>
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -1005,13 +1005,13 @@
         <v>0.501706</v>
       </c>
       <c r="W3" s="1" t="n">
-        <v>0.47337</v>
+        <v>0.47274</v>
       </c>
       <c r="X3" s="1" t="n">
-        <v>0.47203</v>
+        <v>0.47116</v>
       </c>
       <c r="Y3" s="1" t="n">
-        <v>0.51502</v>
+        <v>0.51397</v>
       </c>
       <c r="Z3" s="1" t="n">
         <v>0.15254</v>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1306,7 @@
         <v>3</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>30.08333</v>
+        <v>30</v>
       </c>
       <c r="S5" s="2" t="n">
         <v>25.5</v>
@@ -1330,13 +1330,13 @@
         <v>0.5375</v>
       </c>
       <c r="Z5" s="1" t="n">
-        <v>0.10211</v>
+        <v>0.10247</v>
       </c>
       <c r="AA5" s="1" t="n">
         <v>0.90123</v>
       </c>
       <c r="AB5" s="3" t="n">
-        <v>1.00334</v>
+        <v>1.0037</v>
       </c>
       <c r="AC5" s="1" t="n">
         <v>0.53369</v>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
         <v>3.3636</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>26.18181</v>
+        <v>26.36363</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>31.45454</v>
@@ -1479,22 +1479,22 @@
         <v>0.503681</v>
       </c>
       <c r="W6" s="1" t="n">
-        <v>0.43222</v>
+        <v>0.43263</v>
       </c>
       <c r="X6" s="1" t="n">
-        <v>0.43415</v>
+        <v>0.43472</v>
       </c>
       <c r="Y6" s="1" t="n">
-        <v>0.49015</v>
+        <v>0.49112</v>
       </c>
       <c r="Z6" s="1" t="n">
-        <v>0.14035</v>
+        <v>0.13973</v>
       </c>
       <c r="AA6" s="1" t="n">
         <v>0.91544</v>
       </c>
       <c r="AB6" s="3" t="n">
-        <v>1.05579</v>
+        <v>1.05517</v>
       </c>
       <c r="AC6" s="1" t="n">
         <v>0.43526</v>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -1741,13 +1741,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
         <v>7</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -1756,7 +1756,7 @@
         <v>14</v>
       </c>
       <c r="J8" s="1" t="n">
-        <v>0.777778</v>
+        <v>0.7</v>
       </c>
       <c r="K8" t="n">
         <v>6</v>
@@ -1765,55 +1765,55 @@
         <v>7</v>
       </c>
       <c r="M8" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="N8" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="O8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>3.4444</v>
+        <v>3.4</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>2.5556</v>
+        <v>2.9</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>29.77777</v>
+        <v>30.2</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>24.22222</v>
+        <v>24.2</v>
       </c>
       <c r="T8" s="1" t="n">
-        <v>0.129032</v>
+        <v>0.135135</v>
       </c>
       <c r="U8" s="1" t="n">
-        <v>0.791667</v>
+        <v>0.777778</v>
       </c>
       <c r="V8" s="1" t="n">
-        <v>0.484848</v>
+        <v>0.497316</v>
       </c>
       <c r="W8" s="1" t="n">
-        <v>0.55764</v>
+        <v>0.5604</v>
       </c>
       <c r="X8" s="1" t="n">
-        <v>0.5567299999999999</v>
+        <v>0.5622</v>
       </c>
       <c r="Y8" s="1" t="n">
-        <v>0.56192</v>
+        <v>0.5625</v>
       </c>
       <c r="Z8" s="1" t="n">
-        <v>0.11219</v>
+        <v>0.10822</v>
       </c>
       <c r="AA8" s="1" t="n">
-        <v>0.90909</v>
+        <v>0.89617</v>
       </c>
       <c r="AB8" s="3" t="n">
-        <v>1.02128</v>
+        <v>1.00439</v>
       </c>
       <c r="AC8" s="1" t="n">
-        <v>0.59523</v>
+        <v>0.59498</v>
       </c>
       <c r="AD8" t="n">
         <v>5</v>
@@ -1834,46 +1834,46 @@
         <v>9</v>
       </c>
       <c r="AJ8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AK8" t="n">
         <v>2</v>
       </c>
       <c r="AL8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM8" t="n">
         <v>0</v>
       </c>
       <c r="AN8" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="AO8" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="AP8" t="n">
         <v>7</v>
       </c>
       <c r="AQ8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR8" t="n">
         <v>0</v>
       </c>
       <c r="AS8" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="AT8" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="AU8" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
         <v>30.63636</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>22.54545</v>
+        <v>22.72727</v>
       </c>
       <c r="T9" s="1" t="n">
         <v>0.384615</v>
@@ -1953,22 +1953,22 @@
         <v>0.533639</v>
       </c>
       <c r="W9" s="1" t="n">
-        <v>0.57313</v>
+        <v>0.5727100000000001</v>
       </c>
       <c r="X9" s="1" t="n">
-        <v>0.5795</v>
+        <v>0.57891</v>
       </c>
       <c r="Y9" s="1" t="n">
-        <v>0.572</v>
+        <v>0.57113</v>
       </c>
       <c r="Z9" s="1" t="n">
         <v>0.09118</v>
       </c>
       <c r="AA9" s="1" t="n">
-        <v>0.8930399999999999</v>
+        <v>0.89361</v>
       </c>
       <c r="AB9" s="3" t="n">
-        <v>0.98422</v>
+        <v>0.9847900000000001</v>
       </c>
       <c r="AC9" s="1" t="n">
         <v>0.51497</v>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
         <v>2.4545</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>30.45454</v>
+        <v>30.63636</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>25.72727</v>
@@ -2111,22 +2111,22 @@
         <v>0.524409</v>
       </c>
       <c r="W10" s="1" t="n">
-        <v>0.5267500000000001</v>
+        <v>0.52725</v>
       </c>
       <c r="X10" s="1" t="n">
-        <v>0.54597</v>
+        <v>0.54662</v>
       </c>
       <c r="Y10" s="1" t="n">
-        <v>0.5285</v>
+        <v>0.5306999999999999</v>
       </c>
       <c r="Z10" s="1" t="n">
-        <v>0.08064</v>
+        <v>0.08032</v>
       </c>
       <c r="AA10" s="1" t="n">
         <v>0.92647</v>
       </c>
       <c r="AB10" s="3" t="n">
-        <v>1.00711</v>
+        <v>1.00679</v>
       </c>
       <c r="AC10" s="1" t="n">
         <v>0.55263</v>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -2663,19 +2663,19 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>San Jose Sharks</t>
+          <t>Colorado Avalanche</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SJS</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -2707,97 +2707,97 @@
         <v>0.590909</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L14" t="n">
+        <v>6</v>
+      </c>
+      <c r="M14" t="n">
+        <v>47</v>
+      </c>
+      <c r="N14" t="n">
+        <v>34</v>
+      </c>
+      <c r="O14" t="n">
+        <v>13</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>4.2727</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>3.0909</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>27.90909</v>
+      </c>
+      <c r="T14" s="1" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="U14" s="1" t="n">
+        <v>0.827587</v>
+      </c>
+      <c r="V14" s="1" t="n">
+        <v>0.471556</v>
+      </c>
+      <c r="W14" s="1" t="n">
+        <v>0.51595</v>
+      </c>
+      <c r="X14" s="1" t="n">
+        <v>0.51351</v>
+      </c>
+      <c r="Y14" s="1" t="n">
+        <v>0.52679</v>
+      </c>
+      <c r="Z14" s="1" t="n">
+        <v>0.14843</v>
+      </c>
+      <c r="AA14" s="1" t="n">
+        <v>0.91164</v>
+      </c>
+      <c r="AB14" s="3" t="n">
+        <v>1.06007</v>
+      </c>
+      <c r="AC14" s="1" t="n">
+        <v>0.49554</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>19</v>
+      </c>
+      <c r="AJ14" t="n">
         <v>5</v>
       </c>
-      <c r="M14" t="n">
-        <v>33</v>
-      </c>
-      <c r="N14" t="n">
-        <v>37</v>
-      </c>
-      <c r="O14" t="n">
-        <v>-4</v>
-      </c>
-      <c r="P14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q14" s="2" t="n">
-        <v>3.3636</v>
-      </c>
-      <c r="R14" s="2" t="n">
-        <v>28.18181</v>
-      </c>
-      <c r="S14" s="2" t="n">
-        <v>29.90909</v>
-      </c>
-      <c r="T14" s="1" t="n">
-        <v>0.257142</v>
-      </c>
-      <c r="U14" s="1" t="n">
-        <v>0.805556</v>
-      </c>
-      <c r="V14" s="1" t="n">
-        <v>0.470676</v>
-      </c>
-      <c r="W14" s="1" t="n">
-        <v>0.45731</v>
-      </c>
-      <c r="X14" s="1" t="n">
-        <v>0.46266</v>
-      </c>
-      <c r="Y14" s="1" t="n">
-        <v>0.48953</v>
-      </c>
-      <c r="Z14" s="1" t="n">
-        <v>0.06808</v>
-      </c>
-      <c r="AA14" s="1" t="n">
-        <v>0.90495</v>
-      </c>
-      <c r="AB14" s="3" t="n">
-        <v>0.97303</v>
-      </c>
-      <c r="AC14" s="1" t="n">
-        <v>0.4494</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>13</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>16</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>7</v>
-      </c>
       <c r="AK14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AL14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN14" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AO14" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="AP14" t="n">
         <v>5</v>
@@ -2809,189 +2809,189 @@
         <v>1</v>
       </c>
       <c r="AS14" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="AT14" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>New York Islanders</t>
+          <t>San Jose Sharks</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NYI</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J15" s="1" t="n">
-        <v>0.6</v>
+        <v>0.590909</v>
       </c>
       <c r="K15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
         <v>5</v>
       </c>
       <c r="M15" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="N15" t="n">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="O15" t="n">
-        <v>6</v>
+        <v>-4</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>2.3</v>
+        <v>3.3636</v>
       </c>
       <c r="R15" s="2" t="n">
-        <v>26.7</v>
+        <v>28.18181</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>25.5</v>
+        <v>29.90909</v>
       </c>
       <c r="T15" s="1" t="n">
-        <v>0.2</v>
+        <v>0.257142</v>
       </c>
       <c r="U15" s="1" t="n">
-        <v>0.8823530000000001</v>
+        <v>0.805556</v>
       </c>
       <c r="V15" s="1" t="n">
-        <v>0.547388</v>
+        <v>0.470676</v>
       </c>
       <c r="W15" s="1" t="n">
-        <v>0.53278</v>
+        <v>0.45731</v>
       </c>
       <c r="X15" s="1" t="n">
-        <v>0.5238</v>
+        <v>0.46266</v>
       </c>
       <c r="Y15" s="1" t="n">
-        <v>0.56179</v>
+        <v>0.48953</v>
       </c>
       <c r="Z15" s="1" t="n">
-        <v>0.09134</v>
+        <v>0.06808</v>
       </c>
       <c r="AA15" s="1" t="n">
-        <v>0.93548</v>
+        <v>0.90495</v>
       </c>
       <c r="AB15" s="3" t="n">
-        <v>1.02682</v>
+        <v>0.97303</v>
       </c>
       <c r="AC15" s="1" t="n">
-        <v>0.5289199999999999</v>
+        <v>0.4494</v>
       </c>
       <c r="AD15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AE15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AF15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH15" t="n">
+        <v>13</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>16</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>20</v>
+      </c>
+      <c r="AO15" t="n">
         <v>21</v>
-      </c>
-      <c r="AI15" t="n">
-        <v>13</v>
-      </c>
-      <c r="AJ15" t="n">
-        <v>4</v>
-      </c>
-      <c r="AK15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>8</v>
-      </c>
-      <c r="AO15" t="n">
-        <v>10</v>
       </c>
       <c r="AP15" t="n">
         <v>5</v>
       </c>
       <c r="AQ15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS15" t="n">
         <v>29</v>
       </c>
       <c r="AT15" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>New Jersey Devils</t>
+          <t>New York Islanders</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NJD</t>
+          <t>NYI</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3008,13 +3008,13 @@
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I16" t="n">
         <v>12</v>
@@ -3023,133 +3023,133 @@
         <v>0.6</v>
       </c>
       <c r="K16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L16" t="n">
+        <v>5</v>
+      </c>
+      <c r="M16" t="n">
+        <v>29</v>
+      </c>
+      <c r="N16" t="n">
+        <v>23</v>
+      </c>
+      <c r="O16" t="n">
         <v>6</v>
       </c>
-      <c r="M16" t="n">
-        <v>33</v>
-      </c>
-      <c r="N16" t="n">
-        <v>31</v>
-      </c>
-      <c r="O16" t="n">
-        <v>2</v>
-      </c>
       <c r="P16" s="2" t="n">
-        <v>3.3</v>
+        <v>2.9</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>3.1</v>
+        <v>2.3</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>35</v>
+        <v>26.7</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>25.1</v>
+        <v>25.5</v>
       </c>
       <c r="T16" s="1" t="n">
-        <v>0.21875</v>
+        <v>0.2</v>
       </c>
       <c r="U16" s="1" t="n">
-        <v>0.72</v>
+        <v>0.8823530000000001</v>
       </c>
       <c r="V16" s="1" t="n">
-        <v>0.513043</v>
+        <v>0.545454</v>
       </c>
       <c r="W16" s="1" t="n">
-        <v>0.59574</v>
+        <v>0.53278</v>
       </c>
       <c r="X16" s="1" t="n">
-        <v>0.58933</v>
+        <v>0.5238</v>
       </c>
       <c r="Y16" s="1" t="n">
-        <v>0.59459</v>
+        <v>0.56179</v>
       </c>
       <c r="Z16" s="1" t="n">
-        <v>0.07446</v>
+        <v>0.09134</v>
       </c>
       <c r="AA16" s="1" t="n">
-        <v>0.89847</v>
+        <v>0.93548</v>
       </c>
       <c r="AB16" s="3" t="n">
-        <v>0.97293</v>
+        <v>1.02682</v>
       </c>
       <c r="AC16" s="1" t="n">
-        <v>0.5647799999999999</v>
+        <v>0.5289199999999999</v>
       </c>
       <c r="AD16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AE16" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>21</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>13</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>8</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>10</v>
+      </c>
+      <c r="AP16" t="n">
         <v>5</v>
       </c>
-      <c r="AF16" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH16" t="n">
-        <v>26</v>
-      </c>
-      <c r="AI16" t="n">
-        <v>17</v>
-      </c>
-      <c r="AJ16" t="n">
-        <v>3</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL16" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN16" t="n">
-        <v>7</v>
-      </c>
-      <c r="AO16" t="n">
-        <v>14</v>
-      </c>
-      <c r="AP16" t="n">
-        <v>6</v>
-      </c>
       <c r="AQ16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS16" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="AT16" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>OT1</t>
         </is>
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Florida Panthers</t>
+          <t>New Jersey Devils</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>NJD</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3159,165 +3159,165 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G17" t="n">
         <v>4</v>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>12</v>
       </c>
       <c r="J17" s="1" t="n">
-        <v>0.545455</v>
+        <v>0.6</v>
       </c>
       <c r="K17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L17" t="n">
+        <v>6</v>
+      </c>
+      <c r="M17" t="n">
+        <v>33</v>
+      </c>
+      <c r="N17" t="n">
+        <v>31</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="T17" s="1" t="n">
+        <v>0.21875</v>
+      </c>
+      <c r="U17" s="1" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="V17" s="1" t="n">
+        <v>0.513043</v>
+      </c>
+      <c r="W17" s="1" t="n">
+        <v>0.59593</v>
+      </c>
+      <c r="X17" s="1" t="n">
+        <v>0.5895899999999999</v>
+      </c>
+      <c r="Y17" s="1" t="n">
+        <v>0.59459</v>
+      </c>
+      <c r="Z17" s="1" t="n">
+        <v>0.07473</v>
+      </c>
+      <c r="AA17" s="1" t="n">
+        <v>0.89796</v>
+      </c>
+      <c r="AB17" s="3" t="n">
+        <v>0.9726900000000001</v>
+      </c>
+      <c r="AC17" s="1" t="n">
+        <v>0.5647799999999999</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE17" t="n">
         <v>5</v>
       </c>
-      <c r="M17" t="n">
+      <c r="AF17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>26</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>17</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>7</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>14</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>33</v>
+      </c>
+      <c r="AT17" t="n">
         <v>31</v>
       </c>
-      <c r="N17" t="n">
-        <v>34</v>
-      </c>
-      <c r="O17" t="n">
-        <v>-3</v>
-      </c>
-      <c r="P17" s="2" t="n">
-        <v>2.8182</v>
-      </c>
-      <c r="Q17" s="2" t="n">
-        <v>3.0909</v>
-      </c>
-      <c r="R17" s="2" t="n">
-        <v>28.0909</v>
-      </c>
-      <c r="S17" s="2" t="n">
-        <v>24.27272</v>
-      </c>
-      <c r="T17" s="1" t="n">
-        <v>0.192307</v>
-      </c>
-      <c r="U17" s="1" t="n">
-        <v>0.826087</v>
-      </c>
-      <c r="V17" s="1" t="n">
-        <v>0.455384</v>
-      </c>
-      <c r="W17" s="1" t="n">
-        <v>0.55775</v>
-      </c>
-      <c r="X17" s="1" t="n">
-        <v>0.54397</v>
-      </c>
-      <c r="Y17" s="1" t="n">
-        <v>0.58333</v>
-      </c>
-      <c r="Z17" s="1" t="n">
-        <v>0.07843</v>
-      </c>
-      <c r="AA17" s="1" t="n">
-        <v>0.88397</v>
-      </c>
-      <c r="AB17" s="3" t="n">
-        <v>0.9624</v>
-      </c>
-      <c r="AC17" s="1" t="n">
-        <v>0.57347</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH17" t="n">
-        <v>12</v>
-      </c>
-      <c r="AI17" t="n">
-        <v>9</v>
-      </c>
-      <c r="AJ17" t="n">
-        <v>8</v>
-      </c>
-      <c r="AK17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN17" t="n">
-        <v>19</v>
-      </c>
-      <c r="AO17" t="n">
-        <v>25</v>
-      </c>
-      <c r="AP17" t="n">
-        <v>4</v>
-      </c>
-      <c r="AQ17" t="n">
-        <v>4</v>
-      </c>
-      <c r="AR17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS17" t="n">
-        <v>30</v>
-      </c>
-      <c r="AT17" t="n">
-        <v>34</v>
-      </c>
       <c r="AU17" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Colorado Avalanche</t>
+          <t>Montréal Canadiens</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -3327,159 +3327,159 @@
         <v>5</v>
       </c>
       <c r="G18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J18" s="1" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="K18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M18" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="N18" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="O18" t="n">
-        <v>10</v>
+        <v>-1</v>
       </c>
       <c r="P18" s="2" t="n">
-        <v>4.1</v>
+        <v>3.4</v>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="R18" s="2" t="n">
-        <v>30.6</v>
+        <v>29.5</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>27.3</v>
+        <v>25.8</v>
       </c>
       <c r="T18" s="1" t="n">
-        <v>0.1875</v>
+        <v>0.125</v>
       </c>
       <c r="U18" s="1" t="n">
-        <v>0.826087</v>
+        <v>0.809524</v>
       </c>
       <c r="V18" s="1" t="n">
-        <v>0.478476</v>
+        <v>0.536789</v>
       </c>
       <c r="W18" s="1" t="n">
-        <v>0.52547</v>
+        <v>0.57125</v>
       </c>
       <c r="X18" s="1" t="n">
-        <v>0.52549</v>
+        <v>0.5657</v>
       </c>
       <c r="Y18" s="1" t="n">
-        <v>0.52886</v>
+        <v>0.5721000000000001</v>
       </c>
       <c r="Z18" s="1" t="n">
-        <v>0.14285</v>
+        <v>0.09216000000000001</v>
       </c>
       <c r="AA18" s="1" t="n">
-        <v>0.91031</v>
+        <v>0.88648</v>
       </c>
       <c r="AB18" s="3" t="n">
-        <v>1.05316</v>
+        <v>0.97864</v>
       </c>
       <c r="AC18" s="1" t="n">
-        <v>0.50322</v>
+        <v>0.58113</v>
       </c>
       <c r="AD18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE18" t="n">
         <v>3</v>
       </c>
       <c r="AF18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG18" t="n">
         <v>1</v>
       </c>
       <c r="AH18" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="AI18" t="n">
+        <v>21</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN18" t="n">
         <v>16</v>
       </c>
-      <c r="AJ18" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK18" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL18" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN18" t="n">
-        <v>17</v>
-      </c>
       <c r="AO18" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AP18" t="n">
         <v>5</v>
       </c>
       <c r="AQ18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS18" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="AT18" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>St. Louis Blues</t>
+          <t>Florida Panthers</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F19" t="n">
         <v>5</v>
@@ -3488,142 +3488,142 @@
         <v>4</v>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J19" s="1" t="n">
-        <v>0.55</v>
+        <v>0.545455</v>
       </c>
       <c r="K19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L19" t="n">
         <v>5</v>
       </c>
       <c r="M19" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N19" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O19" t="n">
-        <v>4</v>
+        <v>-3</v>
       </c>
       <c r="P19" s="2" t="n">
-        <v>3.5</v>
+        <v>2.8182</v>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>3.1</v>
+        <v>3.0909</v>
       </c>
       <c r="R19" s="2" t="n">
-        <v>26.7</v>
+        <v>28.0909</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>27.5</v>
+        <v>24.36363</v>
       </c>
       <c r="T19" s="1" t="n">
-        <v>0.25</v>
+        <v>0.192307</v>
       </c>
       <c r="U19" s="1" t="n">
-        <v>0.857143</v>
+        <v>0.826087</v>
       </c>
       <c r="V19" s="1" t="n">
-        <v>0.489898</v>
+        <v>0.455384</v>
       </c>
       <c r="W19" s="1" t="n">
-        <v>0.50114</v>
+        <v>0.55775</v>
       </c>
       <c r="X19" s="1" t="n">
-        <v>0.47702</v>
+        <v>0.54397</v>
       </c>
       <c r="Y19" s="1" t="n">
-        <v>0.50481</v>
+        <v>0.58333</v>
       </c>
       <c r="Z19" s="1" t="n">
-        <v>0.09755999999999999</v>
+        <v>0.07843</v>
       </c>
       <c r="AA19" s="1" t="n">
-        <v>0.8878</v>
+        <v>0.88461</v>
       </c>
       <c r="AB19" s="3" t="n">
-        <v>0.98536</v>
+        <v>0.96304</v>
       </c>
       <c r="AC19" s="1" t="n">
-        <v>0.52525</v>
+        <v>0.57347</v>
       </c>
       <c r="AD19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH19" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AI19" t="n">
         <v>9</v>
       </c>
       <c r="AJ19" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AK19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AM19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AN19" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AO19" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="AP19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AQ19" t="n">
         <v>4</v>
       </c>
       <c r="AR19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS19" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="AT19" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="AU19" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Winnipeg Jets</t>
+          <t>St. Louis Blues</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>WPG</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3640,13 +3640,13 @@
         <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
         <v>11</v>
@@ -3655,143 +3655,143 @@
         <v>0.55</v>
       </c>
       <c r="K20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M20" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="N20" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="O20" t="n">
-        <v>-3</v>
+        <v>4</v>
       </c>
       <c r="P20" s="2" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="R20" s="2" t="n">
-        <v>26.5</v>
+        <v>26.7</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>30</v>
+        <v>27.4</v>
       </c>
       <c r="T20" s="1" t="n">
-        <v>0.222222</v>
+        <v>0.25</v>
       </c>
       <c r="U20" s="1" t="n">
-        <v>0.807693</v>
+        <v>0.857143</v>
       </c>
       <c r="V20" s="1" t="n">
-        <v>0.450354</v>
+        <v>0.489898</v>
       </c>
       <c r="W20" s="1" t="n">
-        <v>0.47516</v>
+        <v>0.50114</v>
       </c>
       <c r="X20" s="1" t="n">
-        <v>0.47126</v>
+        <v>0.47702</v>
       </c>
       <c r="Y20" s="1" t="n">
-        <v>0.48442</v>
+        <v>0.50481</v>
       </c>
       <c r="Z20" s="1" t="n">
-        <v>0.09569</v>
+        <v>0.09755999999999999</v>
       </c>
       <c r="AA20" s="1" t="n">
-        <v>0.92796</v>
+        <v>0.88725</v>
       </c>
       <c r="AB20" s="3" t="n">
-        <v>1.02365</v>
+        <v>0.98481</v>
       </c>
       <c r="AC20" s="1" t="n">
-        <v>0.44444</v>
+        <v>0.52525</v>
       </c>
       <c r="AD20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>15</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>9</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>22</v>
+      </c>
+      <c r="AP20" t="n">
         <v>5</v>
       </c>
-      <c r="AE20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH20" t="n">
-        <v>14</v>
-      </c>
-      <c r="AI20" t="n">
-        <v>16</v>
-      </c>
-      <c r="AJ20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>12</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>13</v>
-      </c>
-      <c r="AP20" t="n">
-        <v>4</v>
-      </c>
       <c r="AQ20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AS20" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="AT20" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="AU20" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Detroit Red Wings</t>
+          <t>Winnipeg Jets</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -3813,97 +3813,97 @@
         <v>0.55</v>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M21" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N21" t="n">
+        <v>29</v>
+      </c>
+      <c r="O21" t="n">
+        <v>-3</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="R21" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="S21" s="2" t="n">
         <v>30</v>
-      </c>
-      <c r="O21" t="n">
-        <v>-2</v>
-      </c>
-      <c r="P21" s="2" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="Q21" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="R21" s="2" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="S21" s="2" t="n">
-        <v>25.6</v>
       </c>
       <c r="T21" s="1" t="n">
         <v>0.222222</v>
       </c>
       <c r="U21" s="1" t="n">
-        <v>0.694445</v>
+        <v>0.807693</v>
       </c>
       <c r="V21" s="1" t="n">
-        <v>0.496632</v>
+        <v>0.450354</v>
       </c>
       <c r="W21" s="1" t="n">
-        <v>0.52993</v>
+        <v>0.47516</v>
       </c>
       <c r="X21" s="1" t="n">
-        <v>0.5488</v>
+        <v>0.47126</v>
       </c>
       <c r="Y21" s="1" t="n">
-        <v>0.50375</v>
+        <v>0.48442</v>
       </c>
       <c r="Z21" s="1" t="n">
-        <v>0.08108</v>
+        <v>0.09569</v>
       </c>
       <c r="AA21" s="1" t="n">
-        <v>0.9206299999999999</v>
+        <v>0.92796</v>
       </c>
       <c r="AB21" s="3" t="n">
-        <v>1.00171</v>
+        <v>1.02365</v>
       </c>
       <c r="AC21" s="1" t="n">
-        <v>0.51063</v>
+        <v>0.44444</v>
       </c>
       <c r="AD21" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AE21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG21" t="n">
         <v>1</v>
       </c>
       <c r="AH21" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="AI21" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="AJ21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AK21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM21" t="n">
         <v>2</v>
       </c>
       <c r="AN21" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AO21" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="AP21" t="n">
         <v>4</v>
@@ -3915,31 +3915,31 @@
         <v>3</v>
       </c>
       <c r="AS21" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="AT21" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AU21" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>OT1</t>
         </is>
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Washington Capitals</t>
+          <t>Detroit Red Wings</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3949,101 +3949,101 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J22" s="1" t="n">
-        <v>0.555556</v>
+        <v>0.55</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M22" t="n">
+        <v>28</v>
+      </c>
+      <c r="N22" t="n">
         <v>30</v>
       </c>
-      <c r="N22" t="n">
-        <v>29</v>
-      </c>
       <c r="O22" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="P22" s="2" t="n">
-        <v>3.3333</v>
+        <v>2.8</v>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>3.2222</v>
+        <v>3</v>
       </c>
       <c r="R22" s="2" t="n">
-        <v>26.77777</v>
+        <v>29.9</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>29.22222</v>
+        <v>25.6</v>
       </c>
       <c r="T22" s="1" t="n">
-        <v>0.2</v>
+        <v>0.222222</v>
       </c>
       <c r="U22" s="1" t="n">
-        <v>0.8</v>
+        <v>0.694445</v>
       </c>
       <c r="V22" s="1" t="n">
-        <v>0.508806</v>
+        <v>0.496632</v>
       </c>
       <c r="W22" s="1" t="n">
-        <v>0.46558</v>
+        <v>0.52993</v>
       </c>
       <c r="X22" s="1" t="n">
-        <v>0.47368</v>
+        <v>0.5488</v>
       </c>
       <c r="Y22" s="1" t="n">
-        <v>0.47216</v>
+        <v>0.50375</v>
       </c>
       <c r="Z22" s="1" t="n">
-        <v>0.12707</v>
+        <v>0.08108</v>
       </c>
       <c r="AA22" s="1" t="n">
-        <v>0.89847</v>
+        <v>0.9206299999999999</v>
       </c>
       <c r="AB22" s="3" t="n">
-        <v>1.02554</v>
+        <v>1.00171</v>
       </c>
       <c r="AC22" s="1" t="n">
-        <v>0.43319</v>
+        <v>0.51063</v>
       </c>
       <c r="AD22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AE22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH22" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="AI22" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="AJ22" t="n">
         <v>3</v>
@@ -4052,52 +4052,52 @@
         <v>1</v>
       </c>
       <c r="AL22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AN22" t="n">
         <v>8</v>
       </c>
       <c r="AO22" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AP22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AQ22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS22" t="n">
+        <v>28</v>
+      </c>
+      <c r="AT22" t="n">
         <v>30</v>
       </c>
-      <c r="AT22" t="n">
-        <v>29</v>
-      </c>
       <c r="AU22" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Montréal Canadiens</t>
+          <t>Washington Capitals</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MTL</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4107,20 +4107,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>9</v>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
         <v>10</v>
@@ -4129,79 +4129,79 @@
         <v>0.555556</v>
       </c>
       <c r="K23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M23" t="n">
         <v>30</v>
       </c>
       <c r="N23" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="O23" t="n">
-        <v>-4</v>
+        <v>1</v>
       </c>
       <c r="P23" s="2" t="n">
         <v>3.3333</v>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>3.7778</v>
+        <v>3.2222</v>
       </c>
       <c r="R23" s="2" t="n">
-        <v>29.66666</v>
+        <v>26.77777</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>26.33333</v>
+        <v>29.22222</v>
       </c>
       <c r="T23" s="1" t="n">
-        <v>0.137931</v>
+        <v>0.2</v>
       </c>
       <c r="U23" s="1" t="n">
-        <v>0.783784</v>
+        <v>0.8</v>
       </c>
       <c r="V23" s="1" t="n">
-        <v>0.525423</v>
+        <v>0.508806</v>
       </c>
       <c r="W23" s="1" t="n">
-        <v>0.56701</v>
+        <v>0.46558</v>
       </c>
       <c r="X23" s="1" t="n">
-        <v>0.55789</v>
+        <v>0.47368</v>
       </c>
       <c r="Y23" s="1" t="n">
-        <v>0.57046</v>
+        <v>0.47216</v>
       </c>
       <c r="Z23" s="1" t="n">
-        <v>0.09182999999999999</v>
+        <v>0.12707</v>
       </c>
       <c r="AA23" s="1" t="n">
-        <v>0.88235</v>
+        <v>0.89847</v>
       </c>
       <c r="AB23" s="3" t="n">
-        <v>0.97418</v>
+        <v>1.02554</v>
       </c>
       <c r="AC23" s="1" t="n">
-        <v>0.5641</v>
+        <v>0.43319</v>
       </c>
       <c r="AD23" t="n">
         <v>6</v>
       </c>
       <c r="AE23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF23" t="n">
         <v>2</v>
       </c>
       <c r="AG23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH23" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="AI23" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AJ23" t="n">
         <v>3</v>
@@ -4210,40 +4210,40 @@
         <v>1</v>
       </c>
       <c r="AL23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN23" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AO23" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="AP23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AQ23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS23" t="n">
         <v>30</v>
       </c>
       <c r="AT23" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="AU23" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
         <v>3.4545</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>26.81818</v>
+        <v>26.90909</v>
       </c>
       <c r="S26" s="2" t="n">
         <v>27.63636</v>
@@ -4648,13 +4648,13 @@
         <v>0.48625</v>
       </c>
       <c r="Z26" s="1" t="n">
-        <v>0.11016</v>
+        <v>0.1097</v>
       </c>
       <c r="AA26" s="1" t="n">
         <v>0.88793</v>
       </c>
       <c r="AB26" s="3" t="n">
-        <v>0.99809</v>
+        <v>0.99763</v>
       </c>
       <c r="AC26" s="1" t="n">
         <v>0.53605</v>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -4940,10 +4940,10 @@
         <v>3.3</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>23.4</v>
+        <v>23.3</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>26.8</v>
+        <v>26.7</v>
       </c>
       <c r="T28" s="1" t="n">
         <v>0.21875</v>
@@ -4955,22 +4955,22 @@
         <v>0.437168</v>
       </c>
       <c r="W28" s="1" t="n">
-        <v>0.48081</v>
+        <v>0.48076</v>
       </c>
       <c r="X28" s="1" t="n">
-        <v>0.48323</v>
+        <v>0.48318</v>
       </c>
       <c r="Y28" s="1" t="n">
         <v>0.46182</v>
       </c>
       <c r="Z28" s="1" t="n">
-        <v>0.0829</v>
+        <v>0.08333</v>
       </c>
       <c r="AA28" s="1" t="n">
-        <v>0.89952</v>
+        <v>0.89903</v>
       </c>
       <c r="AB28" s="3" t="n">
-        <v>0.98242</v>
+        <v>0.98236</v>
       </c>
       <c r="AC28" s="1" t="n">
         <v>0.51612</v>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -5268,7 +5268,7 @@
         <v>0.62963</v>
       </c>
       <c r="V30" s="1" t="n">
-        <v>0.507494</v>
+        <v>0.5096349999999999</v>
       </c>
       <c r="W30" s="1" t="n">
         <v>0.49455</v>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -5417,7 +5417,7 @@
         <v>29.11111</v>
       </c>
       <c r="S31" s="2" t="n">
-        <v>30.44444</v>
+        <v>30.66666</v>
       </c>
       <c r="T31" s="1" t="n">
         <v>0.260869</v>
@@ -5429,22 +5429,22 @@
         <v>0.499085</v>
       </c>
       <c r="W31" s="1" t="n">
-        <v>0.51793</v>
+        <v>0.51738</v>
       </c>
       <c r="X31" s="1" t="n">
-        <v>0.50149</v>
+        <v>0.50074</v>
       </c>
       <c r="Y31" s="1" t="n">
-        <v>0.5158700000000001</v>
+        <v>0.51388</v>
       </c>
       <c r="Z31" s="1" t="n">
         <v>0.05116</v>
       </c>
       <c r="AA31" s="1" t="n">
-        <v>0.87096</v>
+        <v>0.87156</v>
       </c>
       <c r="AB31" s="3" t="n">
-        <v>0.9221200000000001</v>
+        <v>0.92272</v>
       </c>
       <c r="AC31" s="1" t="n">
         <v>0.50349</v>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F32" t="n">
         <v>3</v>
       </c>
       <c r="G32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -5548,7 +5548,7 @@
         <v>6</v>
       </c>
       <c r="J32" s="1" t="n">
-        <v>0.333333</v>
+        <v>0.3</v>
       </c>
       <c r="K32" t="n">
         <v>2</v>
@@ -5557,73 +5557,73 @@
         <v>3</v>
       </c>
       <c r="M32" t="n">
+        <v>22</v>
+      </c>
+      <c r="N32" t="n">
+        <v>40</v>
+      </c>
+      <c r="O32" t="n">
+        <v>-18</v>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="T32" s="1" t="n">
+        <v>0.103448</v>
+      </c>
+      <c r="U32" s="1" t="n">
+        <v>0.766667</v>
+      </c>
+      <c r="V32" s="1" t="n">
+        <v>0.423407</v>
+      </c>
+      <c r="W32" s="1" t="n">
+        <v>0.42687</v>
+      </c>
+      <c r="X32" s="1" t="n">
+        <v>0.41121</v>
+      </c>
+      <c r="Y32" s="1" t="n">
+        <v>0.41628</v>
+      </c>
+      <c r="Z32" s="1" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="AA32" s="1" t="n">
+        <v>0.88607</v>
+      </c>
+      <c r="AB32" s="3" t="n">
+        <v>0.9694</v>
+      </c>
+      <c r="AC32" s="1" t="n">
+        <v>0.46551</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH32" t="n">
+        <v>16</v>
+      </c>
+      <c r="AI32" t="n">
         <v>21</v>
-      </c>
-      <c r="N32" t="n">
-        <v>36</v>
-      </c>
-      <c r="O32" t="n">
-        <v>-15</v>
-      </c>
-      <c r="P32" s="2" t="n">
-        <v>2.3333</v>
-      </c>
-      <c r="Q32" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="R32" s="2" t="n">
-        <v>21.44444</v>
-      </c>
-      <c r="S32" s="2" t="n">
-        <v>30.55555</v>
-      </c>
-      <c r="T32" s="1" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="U32" s="1" t="n">
-        <v>0.740741</v>
-      </c>
-      <c r="V32" s="1" t="n">
-        <v>0.429961</v>
-      </c>
-      <c r="W32" s="1" t="n">
-        <v>0.43096</v>
-      </c>
-      <c r="X32" s="1" t="n">
-        <v>0.41666</v>
-      </c>
-      <c r="Y32" s="1" t="n">
-        <v>0.4175</v>
-      </c>
-      <c r="Z32" s="1" t="n">
-        <v>0.08495999999999999</v>
-      </c>
-      <c r="AA32" s="1" t="n">
-        <v>0.88426</v>
-      </c>
-      <c r="AB32" s="3" t="n">
-        <v>0.96922</v>
-      </c>
-      <c r="AC32" s="1" t="n">
-        <v>0.48648</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>5</v>
-      </c>
-      <c r="AE32" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF32" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH32" t="n">
-        <v>15</v>
-      </c>
-      <c r="AI32" t="n">
-        <v>17</v>
       </c>
       <c r="AJ32" t="n">
         <v>4</v>
@@ -5647,25 +5647,25 @@
         <v>3</v>
       </c>
       <c r="AQ32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AR32" t="n">
         <v>0</v>
       </c>
       <c r="AS32" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AT32" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="AU32" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-23 08:11</t>
+          <t>2026-10-24 02:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-24 08:09 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-24 02:49</t>
+          <t>2026-10-24 08:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-25 08:08 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-25 02:50</t>
+          <t>2026-10-25 08:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-26 02:57 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -1083,19 +1083,19 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Edmonton Oilers</t>
+          <t>Minnesota Wild</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1105,155 +1105,155 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F4" t="n">
         <v>8</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J4" s="1" t="n">
-        <v>0.7727270000000001</v>
+        <v>0.692308</v>
       </c>
       <c r="K4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M4" t="n">
+        <v>41</v>
+      </c>
+      <c r="N4" t="n">
+        <v>30</v>
+      </c>
+      <c r="O4" t="n">
+        <v>11</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>3.1538</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>2.3077</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>31.30769</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>24.92307</v>
+      </c>
+      <c r="T4" s="1" t="n">
+        <v>0.261904</v>
+      </c>
+      <c r="U4" s="1" t="n">
+        <v>0.804879</v>
+      </c>
+      <c r="V4" s="1" t="n">
+        <v>0.506056</v>
+      </c>
+      <c r="W4" s="1" t="n">
+        <v>0.53764</v>
+      </c>
+      <c r="X4" s="1" t="n">
+        <v>0.5569</v>
+      </c>
+      <c r="Y4" s="1" t="n">
+        <v>0.52141</v>
+      </c>
+      <c r="Z4" s="1" t="n">
+        <v>0.0858</v>
+      </c>
+      <c r="AA4" s="1" t="n">
+        <v>0.92405</v>
+      </c>
+      <c r="AB4" s="3" t="n">
+        <v>1.00985</v>
+      </c>
+      <c r="AC4" s="1" t="n">
+        <v>0.55337</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>9</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>26</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>22</v>
+      </c>
+      <c r="AP4" t="n">
         <v>6</v>
       </c>
-      <c r="L4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M4" t="n">
-        <v>49</v>
-      </c>
-      <c r="N4" t="n">
-        <v>39</v>
-      </c>
-      <c r="O4" t="n">
-        <v>10</v>
-      </c>
-      <c r="P4" s="2" t="n">
-        <v>4.4545</v>
-      </c>
-      <c r="Q4" s="2" t="n">
-        <v>3.5455</v>
-      </c>
-      <c r="R4" s="2" t="n">
-        <v>25.45454</v>
-      </c>
-      <c r="S4" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="T4" s="1" t="n">
-        <v>0.351351</v>
-      </c>
-      <c r="U4" s="1" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="V4" s="1" t="n">
-        <v>0.501572</v>
-      </c>
-      <c r="W4" s="1" t="n">
-        <v>0.47523</v>
-      </c>
-      <c r="X4" s="1" t="n">
-        <v>0.47299</v>
-      </c>
-      <c r="Y4" s="1" t="n">
-        <v>0.51568</v>
-      </c>
-      <c r="Z4" s="1" t="n">
-        <v>0.135</v>
-      </c>
-      <c r="AA4" s="1" t="n">
-        <v>0.88983</v>
-      </c>
-      <c r="AB4" s="3" t="n">
-        <v>1.02483</v>
-      </c>
-      <c r="AC4" s="1" t="n">
-        <v>0.51228</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>22</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>26</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>27</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>13</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>8</v>
-      </c>
       <c r="AQ4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS4" t="n">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="AT4" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Vegas Golden Knights</t>
+          <t>Edmonton Oilers</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>VGK</t>
+          <t>EDM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1267,13 +1267,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
         <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
@@ -1282,7 +1282,7 @@
         <v>17</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>0.653846</v>
+        <v>0.7727270000000001</v>
       </c>
       <c r="K5" t="n">
         <v>6</v>
@@ -1291,127 +1291,127 @@
         <v>7</v>
       </c>
       <c r="M5" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="N5" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>3.6154</v>
+        <v>4.4545</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>2.9231</v>
+        <v>3.5455</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>29.76923</v>
+        <v>25.45454</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>25.07692</v>
+        <v>27</v>
       </c>
       <c r="T5" s="1" t="n">
-        <v>0.243902</v>
+        <v>0.351351</v>
       </c>
       <c r="U5" s="1" t="n">
-        <v>0.67742</v>
+        <v>0.7</v>
       </c>
       <c r="V5" s="1" t="n">
-        <v>0.506056</v>
+        <v>0.501572</v>
       </c>
       <c r="W5" s="1" t="n">
-        <v>0.5244799999999999</v>
+        <v>0.47523</v>
       </c>
       <c r="X5" s="1" t="n">
-        <v>0.53517</v>
+        <v>0.47299</v>
       </c>
       <c r="Y5" s="1" t="n">
-        <v>0.53846</v>
+        <v>0.51568</v>
       </c>
       <c r="Z5" s="1" t="n">
-        <v>0.09771000000000001</v>
+        <v>0.135</v>
       </c>
       <c r="AA5" s="1" t="n">
-        <v>0.9031</v>
+        <v>0.88983</v>
       </c>
       <c r="AB5" s="3" t="n">
-        <v>1.00081</v>
+        <v>1.02483</v>
       </c>
       <c r="AC5" s="1" t="n">
-        <v>0.52058</v>
+        <v>0.51228</v>
       </c>
       <c r="AD5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AE5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>22</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>26</v>
+      </c>
+      <c r="AJ5" t="n">
         <v>5</v>
       </c>
-      <c r="AF5" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>28</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>20</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>6</v>
-      </c>
       <c r="AK5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AL5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN5" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="AO5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="AP5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AQ5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AR5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS5" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="AT5" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Utah Mammoth</t>
+          <t>Vegas Golden Knights</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UTA</t>
+          <t>VGK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1421,11 +1421,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F6" t="n">
         <v>8</v>
@@ -1434,142 +1434,142 @@
         <v>4</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J6" s="1" t="n">
-        <v>0.666667</v>
+        <v>0.653846</v>
       </c>
       <c r="K6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" t="n">
         <v>7</v>
       </c>
-      <c r="L6" t="n">
-        <v>8</v>
-      </c>
       <c r="M6" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N6" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="O6" t="n">
+        <v>9</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>3.6154</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>2.9231</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>29.76923</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>25.07692</v>
+      </c>
+      <c r="T6" s="1" t="n">
+        <v>0.243902</v>
+      </c>
+      <c r="U6" s="1" t="n">
+        <v>0.67742</v>
+      </c>
+      <c r="V6" s="1" t="n">
+        <v>0.506056</v>
+      </c>
+      <c r="W6" s="1" t="n">
+        <v>0.5244799999999999</v>
+      </c>
+      <c r="X6" s="1" t="n">
+        <v>0.53517</v>
+      </c>
+      <c r="Y6" s="1" t="n">
+        <v>0.53846</v>
+      </c>
+      <c r="Z6" s="1" t="n">
+        <v>0.09771000000000001</v>
+      </c>
+      <c r="AA6" s="1" t="n">
+        <v>0.9031</v>
+      </c>
+      <c r="AB6" s="3" t="n">
+        <v>1.00081</v>
+      </c>
+      <c r="AC6" s="1" t="n">
+        <v>0.52058</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>28</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>20</v>
+      </c>
+      <c r="AJ6" t="n">
         <v>6</v>
       </c>
-      <c r="P6" s="2" t="n">
-        <v>3.8333</v>
-      </c>
-      <c r="Q6" s="2" t="n">
-        <v>3.3333</v>
-      </c>
-      <c r="R6" s="2" t="n">
-        <v>30.41666</v>
-      </c>
-      <c r="S6" s="2" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="T6" s="1" t="n">
-        <v>0.380952</v>
-      </c>
-      <c r="U6" s="1" t="n">
-        <v>0.666667</v>
-      </c>
-      <c r="V6" s="1" t="n">
-        <v>0.541208</v>
-      </c>
-      <c r="W6" s="1" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="X6" s="1" t="n">
-        <v>0.57298</v>
-      </c>
-      <c r="Y6" s="1" t="n">
-        <v>0.56414</v>
-      </c>
-      <c r="Z6" s="1" t="n">
-        <v>0.09533</v>
-      </c>
-      <c r="AA6" s="1" t="n">
-        <v>0.89302</v>
-      </c>
-      <c r="AB6" s="3" t="n">
-        <v>0.98835</v>
-      </c>
-      <c r="AC6" s="1" t="n">
-        <v>0.51474</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>5</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>4</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>23</v>
-      </c>
-      <c r="AI6" t="n">
+      <c r="AK6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>19</v>
+      </c>
+      <c r="AO6" t="n">
         <v>18</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>4</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>23</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>22</v>
       </c>
       <c r="AP6" t="n">
         <v>6</v>
       </c>
       <c r="AQ6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS6" t="n">
         <v>36</v>
       </c>
       <c r="AT6" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>OT1</t>
         </is>
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Minnesota Wild</t>
+          <t>Utah Mammoth</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>UTA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1586,13 +1586,13 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>16</v>
@@ -1604,109 +1604,109 @@
         <v>7</v>
       </c>
       <c r="L7" t="n">
+        <v>8</v>
+      </c>
+      <c r="M7" t="n">
+        <v>46</v>
+      </c>
+      <c r="N7" t="n">
+        <v>40</v>
+      </c>
+      <c r="O7" t="n">
+        <v>6</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>3.8333</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>3.3333</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>30.41666</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="T7" s="1" t="n">
+        <v>0.380952</v>
+      </c>
+      <c r="U7" s="1" t="n">
+        <v>0.666667</v>
+      </c>
+      <c r="V7" s="1" t="n">
+        <v>0.541208</v>
+      </c>
+      <c r="W7" s="1" t="n">
+        <v>0.5685</v>
+      </c>
+      <c r="X7" s="1" t="n">
+        <v>0.57298</v>
+      </c>
+      <c r="Y7" s="1" t="n">
+        <v>0.56414</v>
+      </c>
+      <c r="Z7" s="1" t="n">
+        <v>0.09533</v>
+      </c>
+      <c r="AA7" s="1" t="n">
+        <v>0.89302</v>
+      </c>
+      <c r="AB7" s="3" t="n">
+        <v>0.98835</v>
+      </c>
+      <c r="AC7" s="1" t="n">
+        <v>0.51474</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>23</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>18</v>
+      </c>
+      <c r="AJ7" t="n">
         <v>7</v>
       </c>
-      <c r="M7" t="n">
-        <v>37</v>
-      </c>
-      <c r="N7" t="n">
-        <v>28</v>
-      </c>
-      <c r="O7" t="n">
-        <v>9</v>
-      </c>
-      <c r="P7" s="2" t="n">
-        <v>3.0833</v>
-      </c>
-      <c r="Q7" s="2" t="n">
-        <v>2.3333</v>
-      </c>
-      <c r="R7" s="2" t="n">
-        <v>31.08333</v>
-      </c>
-      <c r="S7" s="2" t="n">
-        <v>25.58333</v>
-      </c>
-      <c r="T7" s="1" t="n">
-        <v>0.243243</v>
-      </c>
-      <c r="U7" s="1" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="V7" s="1" t="n">
-        <v>0.508595</v>
-      </c>
-      <c r="W7" s="1" t="n">
-        <v>0.5325</v>
-      </c>
-      <c r="X7" s="1" t="n">
-        <v>0.55249</v>
-      </c>
-      <c r="Y7" s="1" t="n">
-        <v>0.53187</v>
-      </c>
-      <c r="Z7" s="1" t="n">
-        <v>0.08633</v>
-      </c>
-      <c r="AA7" s="1" t="n">
-        <v>0.92825</v>
-      </c>
-      <c r="AB7" s="3" t="n">
-        <v>1.01458</v>
-      </c>
-      <c r="AC7" s="1" t="n">
-        <v>0.55325</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>4</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH7" t="n">
-        <v>15</v>
-      </c>
-      <c r="AI7" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>8</v>
-      </c>
       <c r="AK7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AL7" t="n">
         <v>3</v>
       </c>
       <c r="AM7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AN7" t="n">
+        <v>23</v>
+      </c>
+      <c r="AO7" t="n">
         <v>22</v>
       </c>
-      <c r="AO7" t="n">
-        <v>20</v>
-      </c>
       <c r="AP7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AQ7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS7" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="AT7" t="n">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="AU7" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -2189,19 +2189,19 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Seattle Kraken</t>
+          <t>Dallas Stars</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2211,17 +2211,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F11" t="n">
         <v>7</v>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
         <v>1</v>
@@ -2230,156 +2230,156 @@
         <v>15</v>
       </c>
       <c r="J11" s="1" t="n">
-        <v>0.625</v>
+        <v>0.681818</v>
       </c>
       <c r="K11" t="n">
+        <v>4</v>
+      </c>
+      <c r="L11" t="n">
+        <v>6</v>
+      </c>
+      <c r="M11" t="n">
+        <v>32</v>
+      </c>
+      <c r="N11" t="n">
+        <v>20</v>
+      </c>
+      <c r="O11" t="n">
+        <v>12</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>2.9091</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>1.8182</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>27.72727</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>21.81818</v>
+      </c>
+      <c r="T11" s="1" t="n">
+        <v>0.185185</v>
+      </c>
+      <c r="U11" s="1" t="n">
+        <v>0.923077</v>
+      </c>
+      <c r="V11" s="1" t="n">
+        <v>0.562814</v>
+      </c>
+      <c r="W11" s="1" t="n">
+        <v>0.52852</v>
+      </c>
+      <c r="X11" s="1" t="n">
+        <v>0.5438499999999999</v>
+      </c>
+      <c r="Y11" s="1" t="n">
+        <v>0.53228</v>
+      </c>
+      <c r="Z11" s="1" t="n">
+        <v>0.09132</v>
+      </c>
+      <c r="AA11" s="1" t="n">
+        <v>0.92655</v>
+      </c>
+      <c r="AB11" s="3" t="n">
+        <v>1.01787</v>
+      </c>
+      <c r="AC11" s="1" t="n">
+        <v>0.49038</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>19</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>14</v>
+      </c>
+      <c r="AJ11" t="n">
         <v>5</v>
       </c>
-      <c r="L11" t="n">
-        <v>5</v>
-      </c>
-      <c r="M11" t="n">
-        <v>45</v>
-      </c>
-      <c r="N11" t="n">
-        <v>42</v>
-      </c>
-      <c r="O11" t="n">
-        <v>3</v>
-      </c>
-      <c r="P11" s="2" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="Q11" s="2" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="R11" s="2" t="n">
-        <v>26.16666</v>
-      </c>
-      <c r="S11" s="2" t="n">
-        <v>31.83333</v>
-      </c>
-      <c r="T11" s="1" t="n">
-        <v>0.230769</v>
-      </c>
-      <c r="U11" s="1" t="n">
-        <v>0.705883</v>
-      </c>
-      <c r="V11" s="1" t="n">
-        <v>0.516172</v>
-      </c>
-      <c r="W11" s="1" t="n">
-        <v>0.43106</v>
-      </c>
-      <c r="X11" s="1" t="n">
-        <v>0.4308</v>
-      </c>
-      <c r="Y11" s="1" t="n">
-        <v>0.48824</v>
-      </c>
-      <c r="Z11" s="1" t="n">
-        <v>0.13306</v>
-      </c>
-      <c r="AA11" s="1" t="n">
-        <v>0.9103</v>
-      </c>
-      <c r="AB11" s="3" t="n">
-        <v>1.04336</v>
-      </c>
-      <c r="AC11" s="1" t="n">
-        <v>0.43576</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>5</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH11" t="n">
-        <v>18</v>
-      </c>
-      <c r="AI11" t="n">
-        <v>18</v>
-      </c>
-      <c r="AJ11" t="n">
+      <c r="AK11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>13</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AP11" t="n">
         <v>7</v>
       </c>
-      <c r="AK11" t="n">
-        <v>4</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>27</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>24</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>6</v>
-      </c>
       <c r="AQ11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AR11" t="n">
         <v>1</v>
       </c>
       <c r="AS11" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="AT11" t="n">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>New York Rangers</t>
+          <t>Seattle Kraken</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NYR</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F12" t="n">
         <v>7</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H12" t="n">
         <v>1</v>
@@ -2388,136 +2388,136 @@
         <v>15</v>
       </c>
       <c r="J12" s="1" t="n">
-        <v>0.576923</v>
+        <v>0.625</v>
       </c>
       <c r="K12" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L12" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M12" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="N12" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="O12" t="n">
+        <v>3</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>26.16666</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>31.83333</v>
+      </c>
+      <c r="T12" s="1" t="n">
+        <v>0.230769</v>
+      </c>
+      <c r="U12" s="1" t="n">
+        <v>0.705883</v>
+      </c>
+      <c r="V12" s="1" t="n">
+        <v>0.516172</v>
+      </c>
+      <c r="W12" s="1" t="n">
+        <v>0.43106</v>
+      </c>
+      <c r="X12" s="1" t="n">
+        <v>0.4308</v>
+      </c>
+      <c r="Y12" s="1" t="n">
+        <v>0.48824</v>
+      </c>
+      <c r="Z12" s="1" t="n">
+        <v>0.13306</v>
+      </c>
+      <c r="AA12" s="1" t="n">
+        <v>0.9103</v>
+      </c>
+      <c r="AB12" s="3" t="n">
+        <v>1.04336</v>
+      </c>
+      <c r="AC12" s="1" t="n">
+        <v>0.43576</v>
+      </c>
+      <c r="AD12" t="n">
         <v>5</v>
       </c>
-      <c r="P12" s="2" t="n">
-        <v>3.1538</v>
-      </c>
-      <c r="Q12" s="2" t="n">
-        <v>2.7692</v>
-      </c>
-      <c r="R12" s="2" t="n">
-        <v>24.53846</v>
-      </c>
-      <c r="S12" s="2" t="n">
-        <v>26.30769</v>
-      </c>
-      <c r="T12" s="1" t="n">
-        <v>0.189189</v>
-      </c>
-      <c r="U12" s="1" t="n">
-        <v>0.923077</v>
-      </c>
-      <c r="V12" s="1" t="n">
-        <v>0.53412</v>
-      </c>
-      <c r="W12" s="1" t="n">
-        <v>0.47627</v>
-      </c>
-      <c r="X12" s="1" t="n">
-        <v>0.465</v>
-      </c>
-      <c r="Y12" s="1" t="n">
-        <v>0.46656</v>
-      </c>
-      <c r="Z12" s="1" t="n">
-        <v>0.10569</v>
-      </c>
-      <c r="AA12" s="1" t="n">
-        <v>0.90334</v>
-      </c>
-      <c r="AB12" s="3" t="n">
-        <v>1.00903</v>
-      </c>
-      <c r="AC12" s="1" t="n">
-        <v>0.47244</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>6</v>
-      </c>
       <c r="AE12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AF12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AG12" t="n">
         <v>0</v>
       </c>
       <c r="AH12" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="AI12" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="AJ12" t="n">
         <v>7</v>
       </c>
       <c r="AK12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AL12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AM12" t="n">
         <v>1</v>
       </c>
       <c r="AN12" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="AO12" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="AP12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AQ12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR12" t="n">
         <v>1</v>
       </c>
       <c r="AS12" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="AT12" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>New Jersey Devils</t>
+          <t>New York Rangers</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NJD</t>
+          <t>NYR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2531,88 +2531,88 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F13" t="n">
         <v>7</v>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J13" s="1" t="n">
-        <v>0.636364</v>
+        <v>0.576923</v>
       </c>
       <c r="K13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L13" t="n">
         <v>7</v>
       </c>
       <c r="M13" t="n">
+        <v>41</v>
+      </c>
+      <c r="N13" t="n">
         <v>36</v>
       </c>
-      <c r="N13" t="n">
-        <v>32</v>
-      </c>
       <c r="O13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>3.2727</v>
+        <v>3.1538</v>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>2.9091</v>
+        <v>2.7692</v>
       </c>
       <c r="R13" s="2" t="n">
-        <v>34.0909</v>
+        <v>24.53846</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>23.90909</v>
+        <v>26.30769</v>
       </c>
       <c r="T13" s="1" t="n">
-        <v>0.205882</v>
+        <v>0.189189</v>
       </c>
       <c r="U13" s="1" t="n">
-        <v>0.740741</v>
+        <v>0.923077</v>
       </c>
       <c r="V13" s="1" t="n">
-        <v>0.511475</v>
+        <v>0.53412</v>
       </c>
       <c r="W13" s="1" t="n">
-        <v>0.59774</v>
+        <v>0.47627</v>
       </c>
       <c r="X13" s="1" t="n">
-        <v>0.59491</v>
+        <v>0.465</v>
       </c>
       <c r="Y13" s="1" t="n">
-        <v>0.60273</v>
+        <v>0.46656</v>
       </c>
       <c r="Z13" s="1" t="n">
-        <v>0.07692</v>
+        <v>0.10569</v>
       </c>
       <c r="AA13" s="1" t="n">
-        <v>0.89952</v>
+        <v>0.90334</v>
       </c>
       <c r="AB13" s="3" t="n">
-        <v>0.97644</v>
+        <v>1.00903</v>
       </c>
       <c r="AC13" s="1" t="n">
-        <v>0.56962</v>
+        <v>0.47244</v>
       </c>
       <c r="AD13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AE13" t="n">
         <v>6</v>
       </c>
       <c r="AF13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AG13" t="n">
         <v>0</v>
@@ -2621,154 +2621,154 @@
         <v>29</v>
       </c>
       <c r="AI13" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="AJ13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AK13" t="n">
         <v>1</v>
       </c>
       <c r="AL13" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AM13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN13" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="AO13" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="AP13" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ13" t="n">
         <v>4</v>
       </c>
       <c r="AR13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS13" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="AT13" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dallas Stars</t>
+          <t>New Jersey Devils</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>NJD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>14</v>
+      </c>
+      <c r="J14" s="1" t="n">
+        <v>0.636364</v>
+      </c>
+      <c r="K14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" t="n">
+        <v>7</v>
+      </c>
+      <c r="M14" t="n">
+        <v>36</v>
+      </c>
+      <c r="N14" t="n">
+        <v>32</v>
+      </c>
+      <c r="O14" t="n">
+        <v>4</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>3.2727</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>2.9091</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>34.0909</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>23.90909</v>
+      </c>
+      <c r="T14" s="1" t="n">
+        <v>0.205882</v>
+      </c>
+      <c r="U14" s="1" t="n">
+        <v>0.740741</v>
+      </c>
+      <c r="V14" s="1" t="n">
+        <v>0.511475</v>
+      </c>
+      <c r="W14" s="1" t="n">
+        <v>0.59774</v>
+      </c>
+      <c r="X14" s="1" t="n">
+        <v>0.59491</v>
+      </c>
+      <c r="Y14" s="1" t="n">
+        <v>0.60273</v>
+      </c>
+      <c r="Z14" s="1" t="n">
+        <v>0.07692</v>
+      </c>
+      <c r="AA14" s="1" t="n">
+        <v>0.89952</v>
+      </c>
+      <c r="AB14" s="3" t="n">
+        <v>0.97644</v>
+      </c>
+      <c r="AC14" s="1" t="n">
+        <v>0.56962</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE14" t="n">
         <v>6</v>
       </c>
-      <c r="G14" t="n">
-        <v>3</v>
-      </c>
-      <c r="H14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" t="n">
-        <v>13</v>
-      </c>
-      <c r="J14" s="1" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="K14" t="n">
-        <v>3</v>
-      </c>
-      <c r="L14" t="n">
-        <v>5</v>
-      </c>
-      <c r="M14" t="n">
-        <v>26</v>
-      </c>
-      <c r="N14" t="n">
-        <v>17</v>
-      </c>
-      <c r="O14" t="n">
-        <v>9</v>
-      </c>
-      <c r="P14" s="2" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="Q14" s="2" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="R14" s="2" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="S14" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="T14" s="1" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U14" s="1" t="n">
-        <v>0.916667</v>
-      </c>
-      <c r="V14" s="1" t="n">
-        <v>0.570915</v>
-      </c>
-      <c r="W14" s="1" t="n">
-        <v>0.5185999999999999</v>
-      </c>
-      <c r="X14" s="1" t="n">
-        <v>0.53046</v>
-      </c>
-      <c r="Y14" s="1" t="n">
-        <v>0.52566</v>
-      </c>
-      <c r="Z14" s="1" t="n">
-        <v>0.08695</v>
-      </c>
-      <c r="AA14" s="1" t="n">
-        <v>0.93167</v>
-      </c>
-      <c r="AB14" s="3" t="n">
-        <v>1.01862</v>
-      </c>
-      <c r="AC14" s="1" t="n">
-        <v>0.47635</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>5</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>3</v>
-      </c>
       <c r="AF14" t="n">
         <v>2</v>
       </c>
@@ -2776,74 +2776,74 @@
         <v>0</v>
       </c>
       <c r="AH14" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="AI14" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="AJ14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AK14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AL14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN14" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="AO14" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="AP14" t="n">
         <v>6</v>
       </c>
       <c r="AQ14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS14" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="AT14" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Colorado Avalanche</t>
+          <t>Montréal Canadiens</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -2853,106 +2853,106 @@
         <v>6</v>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J15" s="1" t="n">
-        <v>0.590909</v>
+        <v>0.636364</v>
       </c>
       <c r="K15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M15" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="N15" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O15" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>4.2727</v>
+        <v>3.2727</v>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>3.0909</v>
+        <v>3.2727</v>
       </c>
       <c r="R15" s="2" t="n">
-        <v>30</v>
+        <v>28.72727</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>27.90909</v>
+        <v>26.54545</v>
       </c>
       <c r="T15" s="1" t="n">
-        <v>0.2</v>
+        <v>0.125</v>
       </c>
       <c r="U15" s="1" t="n">
-        <v>0.827587</v>
+        <v>0.826087</v>
       </c>
       <c r="V15" s="1" t="n">
-        <v>0.471556</v>
+        <v>0.534246</v>
       </c>
       <c r="W15" s="1" t="n">
-        <v>0.51595</v>
+        <v>0.56269</v>
       </c>
       <c r="X15" s="1" t="n">
-        <v>0.51351</v>
+        <v>0.5601699999999999</v>
       </c>
       <c r="Y15" s="1" t="n">
-        <v>0.52679</v>
+        <v>0.57122</v>
       </c>
       <c r="Z15" s="1" t="n">
-        <v>0.14843</v>
+        <v>0.09322</v>
       </c>
       <c r="AA15" s="1" t="n">
-        <v>0.91164</v>
+        <v>0.89473</v>
       </c>
       <c r="AB15" s="3" t="n">
-        <v>1.06007</v>
+        <v>0.98795</v>
       </c>
       <c r="AC15" s="1" t="n">
-        <v>0.49554</v>
+        <v>0.55518</v>
       </c>
       <c r="AD15" t="n">
         <v>6</v>
       </c>
       <c r="AE15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG15" t="n">
         <v>1</v>
       </c>
       <c r="AH15" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="AI15" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="AJ15" t="n">
         <v>5</v>
       </c>
       <c r="AK15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AM15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AO15" t="n">
         <v>15</v>
@@ -2961,47 +2961,47 @@
         <v>5</v>
       </c>
       <c r="AQ15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS15" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="AT15" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>San Jose Sharks</t>
+          <t>Florida Panthers</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SJS</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -3011,94 +3011,94 @@
         <v>6</v>
       </c>
       <c r="G16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J16" s="1" t="n">
-        <v>0.541667</v>
+        <v>0.583333</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M16" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="O16" t="n">
-        <v>-6</v>
+        <v>-2</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>3.0833</v>
+        <v>2.8333</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>3.5833</v>
+        <v>3</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>28.08333</v>
+        <v>28.5</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>30.33333</v>
+        <v>24.08333</v>
       </c>
       <c r="T16" s="1" t="n">
-        <v>0.268292</v>
+        <v>0.196428</v>
       </c>
       <c r="U16" s="1" t="n">
-        <v>0.804879</v>
+        <v>0.849057</v>
       </c>
       <c r="V16" s="1" t="n">
-        <v>0.463748</v>
+        <v>0.461756</v>
       </c>
       <c r="W16" s="1" t="n">
-        <v>0.44931</v>
+        <v>0.56055</v>
       </c>
       <c r="X16" s="1" t="n">
-        <v>0.45185</v>
+        <v>0.54977</v>
       </c>
       <c r="Y16" s="1" t="n">
-        <v>0.47254</v>
+        <v>0.5837599999999999</v>
       </c>
       <c r="Z16" s="1" t="n">
-        <v>0.064</v>
+        <v>0.07826</v>
       </c>
       <c r="AA16" s="1" t="n">
-        <v>0.89925</v>
+        <v>0.88083</v>
       </c>
       <c r="AB16" s="3" t="n">
-        <v>0.9632500000000001</v>
+        <v>0.95909</v>
       </c>
       <c r="AC16" s="1" t="n">
-        <v>0.45081</v>
+        <v>0.57859</v>
       </c>
       <c r="AD16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE16" t="n">
         <v>2</v>
       </c>
       <c r="AF16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG16" t="n">
         <v>0</v>
       </c>
       <c r="AH16" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AI16" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="AJ16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AK16" t="n">
         <v>4</v>
@@ -3107,365 +3107,365 @@
         <v>3</v>
       </c>
       <c r="AM16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN16" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="AO16" t="n">
         <v>27</v>
       </c>
       <c r="AP16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AQ16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AR16" t="n">
         <v>1</v>
       </c>
       <c r="AS16" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="AT16" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Washington Capitals</t>
+          <t>Colorado Avalanche</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F17" t="n">
         <v>6</v>
       </c>
       <c r="G17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J17" s="1" t="n">
-        <v>0.6</v>
+        <v>0.541667</v>
       </c>
       <c r="K17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L17" t="n">
         <v>6</v>
       </c>
       <c r="M17" t="n">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="N17" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="O17" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="P17" s="2" t="n">
-        <v>3.4</v>
+        <v>4.0833</v>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>3.2</v>
+        <v>3.3333</v>
       </c>
       <c r="R17" s="2" t="n">
-        <v>27.5</v>
+        <v>29.25</v>
       </c>
       <c r="S17" s="2" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
       <c r="T17" s="1" t="n">
-        <v>0.178571</v>
+        <v>0.179487</v>
       </c>
       <c r="U17" s="1" t="n">
-        <v>0.8125</v>
+        <v>0.75</v>
       </c>
       <c r="V17" s="1" t="n">
-        <v>0.501773</v>
+        <v>0.464285</v>
       </c>
       <c r="W17" s="1" t="n">
-        <v>0.46959</v>
+        <v>0.5144300000000001</v>
       </c>
       <c r="X17" s="1" t="n">
-        <v>0.48387</v>
+        <v>0.50954</v>
       </c>
       <c r="Y17" s="1" t="n">
-        <v>0.47993</v>
+        <v>0.52615</v>
       </c>
       <c r="Z17" s="1" t="n">
-        <v>0.12745</v>
+        <v>0.14233</v>
       </c>
       <c r="AA17" s="1" t="n">
-        <v>0.89201</v>
+        <v>0.91208</v>
       </c>
       <c r="AB17" s="3" t="n">
-        <v>1.01946</v>
+        <v>1.05441</v>
       </c>
       <c r="AC17" s="1" t="n">
-        <v>0.42804</v>
+        <v>0.50552</v>
       </c>
       <c r="AD17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AE17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>19</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>19</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>21</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AQ17" t="n">
         <v>5</v>
       </c>
-      <c r="AF17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH17" t="n">
-        <v>26</v>
-      </c>
-      <c r="AI17" t="n">
-        <v>23</v>
-      </c>
-      <c r="AJ17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AK17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN17" t="n">
-        <v>8</v>
-      </c>
-      <c r="AO17" t="n">
-        <v>9</v>
-      </c>
-      <c r="AP17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AQ17" t="n">
-        <v>4</v>
-      </c>
       <c r="AR17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS17" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AT17" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="AU17" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>New York Islanders</t>
+          <t>San Jose Sharks</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>NYI</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F18" t="n">
+        <v>6</v>
+      </c>
+      <c r="G18" t="n">
         <v>5</v>
       </c>
-      <c r="G18" t="n">
-        <v>3</v>
-      </c>
       <c r="H18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J18" s="1" t="n">
-        <v>0.6</v>
+        <v>0.541667</v>
       </c>
       <c r="K18" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
         <v>5</v>
       </c>
       <c r="M18" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="N18" t="n">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="O18" t="n">
-        <v>6</v>
+        <v>-6</v>
       </c>
       <c r="P18" s="2" t="n">
-        <v>2.9</v>
+        <v>3.0833</v>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>2.3</v>
+        <v>3.5833</v>
       </c>
       <c r="R18" s="2" t="n">
-        <v>26.7</v>
+        <v>28.08333</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>25.5</v>
+        <v>30.33333</v>
       </c>
       <c r="T18" s="1" t="n">
-        <v>0.2</v>
+        <v>0.268292</v>
       </c>
       <c r="U18" s="1" t="n">
-        <v>0.8823530000000001</v>
+        <v>0.804879</v>
       </c>
       <c r="V18" s="1" t="n">
-        <v>0.545454</v>
+        <v>0.463748</v>
       </c>
       <c r="W18" s="1" t="n">
-        <v>0.53278</v>
+        <v>0.44931</v>
       </c>
       <c r="X18" s="1" t="n">
-        <v>0.5238</v>
+        <v>0.45185</v>
       </c>
       <c r="Y18" s="1" t="n">
-        <v>0.56179</v>
+        <v>0.47254</v>
       </c>
       <c r="Z18" s="1" t="n">
-        <v>0.09134</v>
+        <v>0.064</v>
       </c>
       <c r="AA18" s="1" t="n">
-        <v>0.93548</v>
+        <v>0.89925</v>
       </c>
       <c r="AB18" s="3" t="n">
-        <v>1.02682</v>
+        <v>0.9632500000000001</v>
       </c>
       <c r="AC18" s="1" t="n">
-        <v>0.5289199999999999</v>
+        <v>0.45081</v>
       </c>
       <c r="AD18" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AE18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AF18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH18" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="AI18" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="AJ18" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AK18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AL18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM18" t="n">
         <v>1</v>
       </c>
       <c r="AN18" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="AO18" t="n">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="AP18" t="n">
+        <v>4</v>
+      </c>
+      <c r="AQ18" t="n">
         <v>5</v>
       </c>
-      <c r="AQ18" t="n">
-        <v>3</v>
-      </c>
       <c r="AR18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS18" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AT18" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Montréal Canadiens</t>
+          <t>Washington Capitals</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MTL</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3475,20 +3475,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E19" t="n">
         <v>10</v>
       </c>
       <c r="F19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
         <v>12</v>
@@ -3497,112 +3497,112 @@
         <v>0.6</v>
       </c>
       <c r="K19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M19" t="n">
         <v>34</v>
       </c>
       <c r="N19" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="O19" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="P19" s="2" t="n">
         <v>3.4</v>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="R19" s="2" t="n">
-        <v>29.5</v>
+        <v>27.5</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>25.8</v>
+        <v>28.4</v>
       </c>
       <c r="T19" s="1" t="n">
-        <v>0.125</v>
+        <v>0.178571</v>
       </c>
       <c r="U19" s="1" t="n">
-        <v>0.809524</v>
+        <v>0.8125</v>
       </c>
       <c r="V19" s="1" t="n">
-        <v>0.536789</v>
+        <v>0.501773</v>
       </c>
       <c r="W19" s="1" t="n">
-        <v>0.57125</v>
+        <v>0.46959</v>
       </c>
       <c r="X19" s="1" t="n">
-        <v>0.5657</v>
+        <v>0.48387</v>
       </c>
       <c r="Y19" s="1" t="n">
-        <v>0.5721000000000001</v>
+        <v>0.47993</v>
       </c>
       <c r="Z19" s="1" t="n">
-        <v>0.09216000000000001</v>
+        <v>0.12745</v>
       </c>
       <c r="AA19" s="1" t="n">
-        <v>0.88648</v>
+        <v>0.89201</v>
       </c>
       <c r="AB19" s="3" t="n">
-        <v>0.97864</v>
+        <v>1.01946</v>
       </c>
       <c r="AC19" s="1" t="n">
-        <v>0.58113</v>
+        <v>0.42804</v>
       </c>
       <c r="AD19" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>26</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>23</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>8</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>9</v>
+      </c>
+      <c r="AP19" t="n">
         <v>6</v>
       </c>
-      <c r="AE19" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF19" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH19" t="n">
-        <v>18</v>
-      </c>
-      <c r="AI19" t="n">
-        <v>21</v>
-      </c>
-      <c r="AJ19" t="n">
-        <v>4</v>
-      </c>
-      <c r="AK19" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN19" t="n">
-        <v>16</v>
-      </c>
-      <c r="AO19" t="n">
-        <v>14</v>
-      </c>
-      <c r="AP19" t="n">
-        <v>5</v>
-      </c>
       <c r="AQ19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS19" t="n">
         <v>34</v>
       </c>
       <c r="AT19" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AU19" t="inlineStr">
         <is>
@@ -3611,19 +3611,19 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Florida Panthers</t>
+          <t>New York Islanders</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>NYI</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -3655,133 +3655,133 @@
         <v>0.545455</v>
       </c>
       <c r="K20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L20" t="n">
         <v>5</v>
       </c>
       <c r="M20" t="n">
+        <v>32</v>
+      </c>
+      <c r="N20" t="n">
+        <v>29</v>
+      </c>
+      <c r="O20" t="n">
+        <v>3</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>2.9091</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>2.6364</v>
+      </c>
+      <c r="R20" s="2" t="n">
+        <v>26.0909</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>26.63636</v>
+      </c>
+      <c r="T20" s="1" t="n">
+        <v>0.181818</v>
+      </c>
+      <c r="U20" s="1" t="n">
+        <v>0.861112</v>
+      </c>
+      <c r="V20" s="1" t="n">
+        <v>0.54578</v>
+      </c>
+      <c r="W20" s="1" t="n">
+        <v>0.51789</v>
+      </c>
+      <c r="X20" s="1" t="n">
+        <v>0.50589</v>
+      </c>
+      <c r="Y20" s="1" t="n">
+        <v>0.54174</v>
+      </c>
+      <c r="Z20" s="1" t="n">
+        <v>0.09375</v>
+      </c>
+      <c r="AA20" s="1" t="n">
+        <v>0.9276</v>
+      </c>
+      <c r="AB20" s="3" t="n">
+        <v>1.02135</v>
+      </c>
+      <c r="AC20" s="1" t="n">
+        <v>0.51162</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>21</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>13</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>11</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>16</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS20" t="n">
         <v>31</v>
       </c>
-      <c r="N20" t="n">
-        <v>34</v>
-      </c>
-      <c r="O20" t="n">
-        <v>-3</v>
-      </c>
-      <c r="P20" s="2" t="n">
-        <v>2.8182</v>
-      </c>
-      <c r="Q20" s="2" t="n">
-        <v>3.0909</v>
-      </c>
-      <c r="R20" s="2" t="n">
-        <v>28.0909</v>
-      </c>
-      <c r="S20" s="2" t="n">
-        <v>24.36363</v>
-      </c>
-      <c r="T20" s="1" t="n">
-        <v>0.192307</v>
-      </c>
-      <c r="U20" s="1" t="n">
-        <v>0.826087</v>
-      </c>
-      <c r="V20" s="1" t="n">
-        <v>0.455384</v>
-      </c>
-      <c r="W20" s="1" t="n">
-        <v>0.55775</v>
-      </c>
-      <c r="X20" s="1" t="n">
-        <v>0.54397</v>
-      </c>
-      <c r="Y20" s="1" t="n">
-        <v>0.58333</v>
-      </c>
-      <c r="Z20" s="1" t="n">
-        <v>0.07843</v>
-      </c>
-      <c r="AA20" s="1" t="n">
-        <v>0.88461</v>
-      </c>
-      <c r="AB20" s="3" t="n">
-        <v>0.96304</v>
-      </c>
-      <c r="AC20" s="1" t="n">
-        <v>0.57347</v>
-      </c>
-      <c r="AD20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH20" t="n">
-        <v>12</v>
-      </c>
-      <c r="AI20" t="n">
-        <v>9</v>
-      </c>
-      <c r="AJ20" t="n">
-        <v>8</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>19</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>25</v>
-      </c>
-      <c r="AP20" t="n">
-        <v>4</v>
-      </c>
-      <c r="AQ20" t="n">
-        <v>4</v>
-      </c>
-      <c r="AR20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS20" t="n">
-        <v>30</v>
-      </c>
       <c r="AT20" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="AU20" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Winnipeg Jets</t>
+          <t>Nashville Predators</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>WPG</t>
+          <t>NSH</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F21" t="n">
         <v>4</v>
@@ -3804,13 +3804,13 @@
         <v>3</v>
       </c>
       <c r="H21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I21" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J21" s="1" t="n">
-        <v>0.55</v>
+        <v>0.545455</v>
       </c>
       <c r="K21" t="n">
         <v>4</v>
@@ -3819,61 +3819,61 @@
         <v>4</v>
       </c>
       <c r="M21" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="N21" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="O21" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="P21" s="2" t="n">
-        <v>2.6</v>
+        <v>2.8182</v>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>2.9</v>
+        <v>3.1818</v>
       </c>
       <c r="R21" s="2" t="n">
-        <v>26.5</v>
+        <v>25.81818</v>
       </c>
       <c r="S21" s="2" t="n">
-        <v>30</v>
+        <v>29.27272</v>
       </c>
       <c r="T21" s="1" t="n">
-        <v>0.222222</v>
+        <v>0.333333</v>
       </c>
       <c r="U21" s="1" t="n">
-        <v>0.807693</v>
+        <v>0.857143</v>
       </c>
       <c r="V21" s="1" t="n">
-        <v>0.450354</v>
+        <v>0.505511</v>
       </c>
       <c r="W21" s="1" t="n">
-        <v>0.47516</v>
+        <v>0.44533</v>
       </c>
       <c r="X21" s="1" t="n">
-        <v>0.47126</v>
+        <v>0.45765</v>
       </c>
       <c r="Y21" s="1" t="n">
-        <v>0.48442</v>
+        <v>0.42446</v>
       </c>
       <c r="Z21" s="1" t="n">
-        <v>0.09569</v>
+        <v>0.06829</v>
       </c>
       <c r="AA21" s="1" t="n">
-        <v>0.92796</v>
+        <v>0.91304</v>
       </c>
       <c r="AB21" s="3" t="n">
-        <v>1.02365</v>
+        <v>0.98133</v>
       </c>
       <c r="AC21" s="1" t="n">
-        <v>0.44444</v>
+        <v>0.45859</v>
       </c>
       <c r="AD21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF21" t="n">
         <v>2</v>
@@ -3882,7 +3882,7 @@
         <v>1</v>
       </c>
       <c r="AH21" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="AI21" t="n">
         <v>16</v>
@@ -3891,43 +3891,43 @@
         <v>5</v>
       </c>
       <c r="AK21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AL21" t="n">
         <v>1</v>
       </c>
       <c r="AM21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN21" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AO21" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="AP21" t="n">
         <v>4</v>
       </c>
       <c r="AQ21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AR21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AS21" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="AT21" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="AU21" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -4085,29 +4085,29 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Detroit Red Wings</t>
+          <t>Winnipeg Jets</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -4129,67 +4129,67 @@
         <v>0.5</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M23" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="N23" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O23" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="P23" s="2" t="n">
-        <v>2.6364</v>
+        <v>2.4545</v>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>3.0909</v>
+        <v>2.8182</v>
       </c>
       <c r="R23" s="2" t="n">
-        <v>29.81818</v>
+        <v>27.18181</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>25.54545</v>
+        <v>29.18181</v>
       </c>
       <c r="T23" s="1" t="n">
-        <v>0.210526</v>
+        <v>0.193548</v>
       </c>
       <c r="U23" s="1" t="n">
-        <v>0.657895</v>
+        <v>0.807693</v>
       </c>
       <c r="V23" s="1" t="n">
-        <v>0.500777</v>
+        <v>0.454253</v>
       </c>
       <c r="W23" s="1" t="n">
-        <v>0.53407</v>
+        <v>0.47821</v>
       </c>
       <c r="X23" s="1" t="n">
-        <v>0.5497</v>
+        <v>0.47272</v>
       </c>
       <c r="Y23" s="1" t="n">
-        <v>0.50946</v>
+        <v>0.48068</v>
       </c>
       <c r="Z23" s="1" t="n">
-        <v>0.07722999999999999</v>
+        <v>0.09012000000000001</v>
       </c>
       <c r="AA23" s="1" t="n">
-        <v>0.91866</v>
+        <v>0.92549</v>
       </c>
       <c r="AB23" s="3" t="n">
-        <v>0.9958900000000001</v>
+        <v>1.01561</v>
       </c>
       <c r="AC23" s="1" t="n">
-        <v>0.51935</v>
+        <v>0.46418</v>
       </c>
       <c r="AD23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AE23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF23" t="n">
         <v>3</v>
@@ -4198,16 +4198,16 @@
         <v>1</v>
       </c>
       <c r="AH23" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="AI23" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="AJ23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AK23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL23" t="n">
         <v>1</v>
@@ -4216,25 +4216,25 @@
         <v>2</v>
       </c>
       <c r="AN23" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="AO23" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AP23" t="n">
         <v>4</v>
       </c>
       <c r="AQ23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AS23" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="AT23" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="AU23" t="inlineStr">
         <is>
@@ -4243,19 +4243,19 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Buffalo Sabres</t>
+          <t>Detroit Red Wings</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4287,64 +4287,64 @@
         <v>0.5</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M24" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="N24" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="O24" t="n">
-        <v>-10</v>
+        <v>-5</v>
       </c>
       <c r="P24" s="2" t="n">
-        <v>2.8182</v>
+        <v>2.6364</v>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>3.7273</v>
+        <v>3.0909</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>26.36363</v>
+        <v>29.81818</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>26.54545</v>
+        <v>25.54545</v>
       </c>
       <c r="T24" s="1" t="n">
-        <v>0.105263</v>
+        <v>0.210526</v>
       </c>
       <c r="U24" s="1" t="n">
-        <v>0.692308</v>
+        <v>0.657895</v>
       </c>
       <c r="V24" s="1" t="n">
-        <v>0.478056</v>
+        <v>0.500777</v>
       </c>
       <c r="W24" s="1" t="n">
-        <v>0.5230399999999999</v>
+        <v>0.53407</v>
       </c>
       <c r="X24" s="1" t="n">
-        <v>0.51179</v>
+        <v>0.5497</v>
       </c>
       <c r="Y24" s="1" t="n">
-        <v>0.49155</v>
+        <v>0.50946</v>
       </c>
       <c r="Z24" s="1" t="n">
-        <v>0.09954</v>
+        <v>0.07722999999999999</v>
       </c>
       <c r="AA24" s="1" t="n">
-        <v>0.87623</v>
+        <v>0.91866</v>
       </c>
       <c r="AB24" s="3" t="n">
-        <v>0.97577</v>
+        <v>0.9958900000000001</v>
       </c>
       <c r="AC24" s="1" t="n">
-        <v>0.52396</v>
+        <v>0.51935</v>
       </c>
       <c r="AD24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AE24" t="n">
         <v>3</v>
@@ -4353,16 +4353,16 @@
         <v>3</v>
       </c>
       <c r="AG24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH24" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="AI24" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="AJ24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AK24" t="n">
         <v>1</v>
@@ -4371,13 +4371,13 @@
         <v>1</v>
       </c>
       <c r="AM24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AN24" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AO24" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="AP24" t="n">
         <v>4</v>
@@ -4389,31 +4389,31 @@
         <v>3</v>
       </c>
       <c r="AS24" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="AT24" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AU24" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Pittsburgh Penguins</t>
+          <t>Buffalo Sabres</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4423,26 +4423,26 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I25" t="n">
         <v>11</v>
       </c>
       <c r="J25" s="1" t="n">
-        <v>0.458333</v>
+        <v>0.5</v>
       </c>
       <c r="K25" t="n">
         <v>2</v>
@@ -4451,273 +4451,273 @@
         <v>4</v>
       </c>
       <c r="M25" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="N25" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="P25" s="2" t="n">
-        <v>3.3333</v>
+        <v>2.8182</v>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>3.3333</v>
+        <v>3.7273</v>
       </c>
       <c r="R25" s="2" t="n">
-        <v>27.75</v>
+        <v>26.36363</v>
       </c>
       <c r="S25" s="2" t="n">
-        <v>27.5</v>
+        <v>26.54545</v>
       </c>
       <c r="T25" s="1" t="n">
-        <v>0.205882</v>
+        <v>0.105263</v>
       </c>
       <c r="U25" s="1" t="n">
-        <v>0.83871</v>
+        <v>0.692308</v>
       </c>
       <c r="V25" s="1" t="n">
-        <v>0.455882</v>
+        <v>0.478056</v>
       </c>
       <c r="W25" s="1" t="n">
-        <v>0.51813</v>
+        <v>0.5230399999999999</v>
       </c>
       <c r="X25" s="1" t="n">
-        <v>0.5201</v>
+        <v>0.51179</v>
       </c>
       <c r="Y25" s="1" t="n">
-        <v>0.50532</v>
+        <v>0.49155</v>
       </c>
       <c r="Z25" s="1" t="n">
-        <v>0.10074</v>
+        <v>0.09954</v>
       </c>
       <c r="AA25" s="1" t="n">
-        <v>0.89105</v>
+        <v>0.87623</v>
       </c>
       <c r="AB25" s="3" t="n">
-        <v>0.9917899999999999</v>
+        <v>0.97577</v>
       </c>
       <c r="AC25" s="1" t="n">
-        <v>0.525</v>
+        <v>0.52396</v>
       </c>
       <c r="AD25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>14</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>19</v>
+      </c>
+      <c r="AJ25" t="n">
         <v>5</v>
       </c>
-      <c r="AE25" t="n">
-        <v>4</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH25" t="n">
+      <c r="AK25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN25" t="n">
         <v>17</v>
       </c>
-      <c r="AI25" t="n">
-        <v>11</v>
-      </c>
-      <c r="AJ25" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL25" t="n">
-        <v>5</v>
-      </c>
-      <c r="AM25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN25" t="n">
-        <v>23</v>
-      </c>
       <c r="AO25" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="AP25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AQ25" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AR25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS25" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AT25" t="n">
         <v>35</v>
       </c>
       <c r="AU25" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>OT1</t>
         </is>
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Nashville Predators</t>
+          <t>Pittsburgh Penguins</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>NSH</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J26" s="1" t="n">
-        <v>0.5</v>
+        <v>0.458333</v>
       </c>
       <c r="K26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M26" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="N26" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="O26" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="P26" s="2" t="n">
-        <v>2.5</v>
+        <v>3.3333</v>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>3.3</v>
+        <v>3.3333</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>24.9</v>
+        <v>27.75</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>30.1</v>
+        <v>27.5</v>
       </c>
       <c r="T26" s="1" t="n">
-        <v>0.275862</v>
+        <v>0.205882</v>
       </c>
       <c r="U26" s="1" t="n">
         <v>0.83871</v>
       </c>
       <c r="V26" s="1" t="n">
-        <v>0.493913</v>
+        <v>0.455882</v>
       </c>
       <c r="W26" s="1" t="n">
-        <v>0.43995</v>
+        <v>0.51813</v>
       </c>
       <c r="X26" s="1" t="n">
-        <v>0.45007</v>
+        <v>0.5201</v>
       </c>
       <c r="Y26" s="1" t="n">
-        <v>0.42222</v>
+        <v>0.50532</v>
       </c>
       <c r="Z26" s="1" t="n">
-        <v>0.06629</v>
+        <v>0.10074</v>
       </c>
       <c r="AA26" s="1" t="n">
-        <v>0.9106300000000001</v>
+        <v>0.89105</v>
       </c>
       <c r="AB26" s="3" t="n">
-        <v>0.97692</v>
+        <v>0.9917899999999999</v>
       </c>
       <c r="AC26" s="1" t="n">
-        <v>0.46712</v>
+        <v>0.525</v>
       </c>
       <c r="AD26" t="n">
         <v>5</v>
       </c>
       <c r="AE26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH26" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="AI26" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="AJ26" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL26" t="n">
         <v>5</v>
       </c>
-      <c r="AK26" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL26" t="n">
-        <v>1</v>
-      </c>
       <c r="AM26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AN26" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="AO26" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="AP26" t="n">
         <v>3</v>
       </c>
       <c r="AQ26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AR26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AS26" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="AT26" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AU26" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F32" t="n">
         <v>3</v>
       </c>
       <c r="G32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -5548,7 +5548,7 @@
         <v>6</v>
       </c>
       <c r="J32" s="1" t="n">
-        <v>0.3</v>
+        <v>0.272727</v>
       </c>
       <c r="K32" t="n">
         <v>2</v>
@@ -5557,73 +5557,73 @@
         <v>3</v>
       </c>
       <c r="M32" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="N32" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="O32" t="n">
-        <v>-18</v>
+        <v>-19</v>
       </c>
       <c r="P32" s="2" t="n">
-        <v>2.2</v>
+        <v>2.1818</v>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>4</v>
+        <v>3.9091</v>
       </c>
       <c r="R32" s="2" t="n">
-        <v>21.4</v>
+        <v>21.36363</v>
       </c>
       <c r="S32" s="2" t="n">
-        <v>30.3</v>
+        <v>30.54545</v>
       </c>
       <c r="T32" s="1" t="n">
-        <v>0.103448</v>
+        <v>0.083333</v>
       </c>
       <c r="U32" s="1" t="n">
-        <v>0.766667</v>
+        <v>0.764706</v>
       </c>
       <c r="V32" s="1" t="n">
-        <v>0.423407</v>
+        <v>0.427001</v>
       </c>
       <c r="W32" s="1" t="n">
-        <v>0.42687</v>
+        <v>0.42529</v>
       </c>
       <c r="X32" s="1" t="n">
-        <v>0.41121</v>
+        <v>0.40941</v>
       </c>
       <c r="Y32" s="1" t="n">
-        <v>0.41628</v>
+        <v>0.41586</v>
       </c>
       <c r="Z32" s="1" t="n">
-        <v>0.08333</v>
+        <v>0.08938</v>
       </c>
       <c r="AA32" s="1" t="n">
-        <v>0.88607</v>
+        <v>0.88973</v>
       </c>
       <c r="AB32" s="3" t="n">
-        <v>0.9694</v>
+        <v>0.97911</v>
       </c>
       <c r="AC32" s="1" t="n">
-        <v>0.46551</v>
+        <v>0.45806</v>
       </c>
       <c r="AD32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AE32" t="n">
         <v>3</v>
       </c>
       <c r="AF32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG32" t="n">
         <v>0</v>
       </c>
       <c r="AH32" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="AI32" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="AJ32" t="n">
         <v>4</v>
@@ -5656,16 +5656,16 @@
         <v>22</v>
       </c>
       <c r="AT32" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="AU32" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>
@@ -5691,13 +5691,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F33" t="n">
         <v>2</v>
       </c>
       <c r="G33" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
@@ -5706,7 +5706,7 @@
         <v>5</v>
       </c>
       <c r="J33" s="1" t="n">
-        <v>0.208333</v>
+        <v>0.192308</v>
       </c>
       <c r="K33" t="n">
         <v>1</v>
@@ -5715,73 +5715,73 @@
         <v>2</v>
       </c>
       <c r="M33" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N33" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="O33" t="n">
-        <v>-21</v>
+        <v>-23</v>
       </c>
       <c r="P33" s="2" t="n">
-        <v>2.9167</v>
+        <v>2.8462</v>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>4.6667</v>
+        <v>4.6154</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>20.08333</v>
+        <v>19.84615</v>
       </c>
       <c r="S33" s="2" t="n">
-        <v>33.5</v>
+        <v>33.53846</v>
       </c>
       <c r="T33" s="1" t="n">
-        <v>0.222222</v>
+        <v>0.216216</v>
       </c>
       <c r="U33" s="1" t="n">
-        <v>0.65</v>
+        <v>0.644445</v>
       </c>
       <c r="V33" s="1" t="n">
-        <v>0.473684</v>
+        <v>0.477568</v>
       </c>
       <c r="W33" s="1" t="n">
-        <v>0.41045</v>
+        <v>0.40949</v>
       </c>
       <c r="X33" s="1" t="n">
-        <v>0.39973</v>
+        <v>0.39901</v>
       </c>
       <c r="Y33" s="1" t="n">
-        <v>0.40106</v>
+        <v>0.41442</v>
       </c>
       <c r="Z33" s="1" t="n">
-        <v>0.1117</v>
+        <v>0.11386</v>
       </c>
       <c r="AA33" s="1" t="n">
-        <v>0.88607</v>
+        <v>0.88856</v>
       </c>
       <c r="AB33" s="3" t="n">
-        <v>0.99777</v>
+        <v>1.00242</v>
       </c>
       <c r="AC33" s="1" t="n">
-        <v>0.40728</v>
+        <v>0.40937</v>
       </c>
       <c r="AD33" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF33" t="n">
         <v>5</v>
       </c>
-      <c r="AE33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF33" t="n">
-        <v>4</v>
-      </c>
       <c r="AG33" t="n">
         <v>0</v>
       </c>
       <c r="AH33" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="AI33" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="AJ33" t="n">
         <v>7</v>
@@ -5802,28 +5802,28 @@
         <v>32</v>
       </c>
       <c r="AP33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ33" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AR33" t="n">
         <v>1</v>
       </c>
       <c r="AS33" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="AT33" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="AU33" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L4</t>
         </is>
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-25 08:08</t>
+          <t>2026-10-26 02:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-26 10:07 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-26 02:57</t>
+          <t>2026-10-26 10:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-27 02:52 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -1005,13 +1005,13 @@
         <v>0.535014</v>
       </c>
       <c r="W3" s="1" t="n">
-        <v>0.4954</v>
+        <v>0.49448</v>
       </c>
       <c r="X3" s="1" t="n">
-        <v>0.5057</v>
+        <v>0.50507</v>
       </c>
       <c r="Y3" s="1" t="n">
-        <v>0.49507</v>
+        <v>0.49436</v>
       </c>
       <c r="Z3" s="1" t="n">
         <v>0.12643</v>
@@ -1083,19 +1083,19 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Minnesota Wild</t>
+          <t>Edmonton Oilers</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>EDM</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1105,17 +1105,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
         <v>8</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
         <v>2</v>
@@ -1124,136 +1124,136 @@
         <v>18</v>
       </c>
       <c r="J4" s="1" t="n">
-        <v>0.692308</v>
+        <v>0.75</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M4" t="n">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="N4" t="n">
+        <v>43</v>
+      </c>
+      <c r="O4" t="n">
+        <v>9</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>4.3333</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>3.5833</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>25.66666</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>27.16666</v>
+      </c>
+      <c r="T4" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="U4" s="1" t="n">
+        <v>0.705883</v>
+      </c>
+      <c r="V4" s="1" t="n">
+        <v>0.496413</v>
+      </c>
+      <c r="W4" s="1" t="n">
+        <v>0.47558</v>
+      </c>
+      <c r="X4" s="1" t="n">
+        <v>0.47375</v>
+      </c>
+      <c r="Y4" s="1" t="n">
+        <v>0.51202</v>
+      </c>
+      <c r="Z4" s="1" t="n">
+        <v>0.13364</v>
+      </c>
+      <c r="AA4" s="1" t="n">
+        <v>0.89494</v>
+      </c>
+      <c r="AB4" s="3" t="n">
+        <v>1.02858</v>
+      </c>
+      <c r="AC4" s="1" t="n">
+        <v>0.52076</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>25</v>
+      </c>
+      <c r="AI4" t="n">
         <v>30</v>
       </c>
-      <c r="O4" t="n">
-        <v>11</v>
-      </c>
-      <c r="P4" s="2" t="n">
-        <v>3.1538</v>
-      </c>
-      <c r="Q4" s="2" t="n">
-        <v>2.3077</v>
-      </c>
-      <c r="R4" s="2" t="n">
-        <v>31.30769</v>
-      </c>
-      <c r="S4" s="2" t="n">
-        <v>24.92307</v>
-      </c>
-      <c r="T4" s="1" t="n">
-        <v>0.261904</v>
-      </c>
-      <c r="U4" s="1" t="n">
-        <v>0.804879</v>
-      </c>
-      <c r="V4" s="1" t="n">
-        <v>0.506056</v>
-      </c>
-      <c r="W4" s="1" t="n">
-        <v>0.53764</v>
-      </c>
-      <c r="X4" s="1" t="n">
-        <v>0.5569</v>
-      </c>
-      <c r="Y4" s="1" t="n">
-        <v>0.52141</v>
-      </c>
-      <c r="Z4" s="1" t="n">
-        <v>0.0858</v>
-      </c>
-      <c r="AA4" s="1" t="n">
-        <v>0.92405</v>
-      </c>
-      <c r="AB4" s="3" t="n">
-        <v>1.00985</v>
-      </c>
-      <c r="AC4" s="1" t="n">
-        <v>0.55337</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AF4" t="n">
+      <c r="AJ4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL4" t="n">
         <v>0</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="AM4" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" t="n">
-        <v>15</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>2</v>
-      </c>
       <c r="AN4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AO4" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="AP4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AQ4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AR4" t="n">
         <v>1</v>
       </c>
       <c r="AS4" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="AT4" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>OT1</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Edmonton Oilers</t>
+          <t>Minnesota Wild</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1263,143 +1263,143 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F5" t="n">
         <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>0.7727270000000001</v>
+        <v>0.692308</v>
       </c>
       <c r="K5" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" t="n">
+        <v>8</v>
+      </c>
+      <c r="M5" t="n">
+        <v>41</v>
+      </c>
+      <c r="N5" t="n">
+        <v>30</v>
+      </c>
+      <c r="O5" t="n">
+        <v>11</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>3.1538</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>2.3077</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>31.30769</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>24.92307</v>
+      </c>
+      <c r="T5" s="1" t="n">
+        <v>0.261904</v>
+      </c>
+      <c r="U5" s="1" t="n">
+        <v>0.804879</v>
+      </c>
+      <c r="V5" s="1" t="n">
+        <v>0.507402</v>
+      </c>
+      <c r="W5" s="1" t="n">
+        <v>0.53764</v>
+      </c>
+      <c r="X5" s="1" t="n">
+        <v>0.5569</v>
+      </c>
+      <c r="Y5" s="1" t="n">
+        <v>0.52141</v>
+      </c>
+      <c r="Z5" s="1" t="n">
+        <v>0.0858</v>
+      </c>
+      <c r="AA5" s="1" t="n">
+        <v>0.92405</v>
+      </c>
+      <c r="AB5" s="3" t="n">
+        <v>1.00985</v>
+      </c>
+      <c r="AC5" s="1" t="n">
+        <v>0.55337</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>15</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>9</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>26</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>22</v>
+      </c>
+      <c r="AP5" t="n">
         <v>6</v>
       </c>
-      <c r="L5" t="n">
-        <v>7</v>
-      </c>
-      <c r="M5" t="n">
-        <v>49</v>
-      </c>
-      <c r="N5" t="n">
-        <v>39</v>
-      </c>
-      <c r="O5" t="n">
-        <v>10</v>
-      </c>
-      <c r="P5" s="2" t="n">
-        <v>4.4545</v>
-      </c>
-      <c r="Q5" s="2" t="n">
-        <v>3.5455</v>
-      </c>
-      <c r="R5" s="2" t="n">
-        <v>25.45454</v>
-      </c>
-      <c r="S5" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="T5" s="1" t="n">
-        <v>0.351351</v>
-      </c>
-      <c r="U5" s="1" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="V5" s="1" t="n">
-        <v>0.501572</v>
-      </c>
-      <c r="W5" s="1" t="n">
-        <v>0.47523</v>
-      </c>
-      <c r="X5" s="1" t="n">
-        <v>0.47299</v>
-      </c>
-      <c r="Y5" s="1" t="n">
-        <v>0.51568</v>
-      </c>
-      <c r="Z5" s="1" t="n">
-        <v>0.135</v>
-      </c>
-      <c r="AA5" s="1" t="n">
-        <v>0.88983</v>
-      </c>
-      <c r="AB5" s="3" t="n">
-        <v>1.02483</v>
-      </c>
-      <c r="AC5" s="1" t="n">
-        <v>0.51228</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>22</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>26</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>27</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>13</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>8</v>
-      </c>
       <c r="AQ5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS5" t="n">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="AT5" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -1479,13 +1479,13 @@
         <v>0.506056</v>
       </c>
       <c r="W6" s="1" t="n">
-        <v>0.5244799999999999</v>
+        <v>0.52491</v>
       </c>
       <c r="X6" s="1" t="n">
-        <v>0.53517</v>
+        <v>0.53579</v>
       </c>
       <c r="Y6" s="1" t="n">
-        <v>0.53846</v>
+        <v>0.5394</v>
       </c>
       <c r="Z6" s="1" t="n">
         <v>0.09771000000000001</v>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
         <v>25.41666</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>25.91666</v>
+        <v>26</v>
       </c>
       <c r="T8" s="1" t="n">
         <v>0.115384</v>
@@ -1807,10 +1807,10 @@
         <v>0.11162</v>
       </c>
       <c r="AA8" s="1" t="n">
-        <v>0.91855</v>
+        <v>0.91891</v>
       </c>
       <c r="AB8" s="3" t="n">
-        <v>1.03017</v>
+        <v>1.03053</v>
       </c>
       <c r="AC8" s="1" t="n">
         <v>0.48502</v>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -1899,13 +1899,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F9" t="n">
         <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
@@ -1914,7 +1914,7 @@
         <v>16</v>
       </c>
       <c r="J9" s="1" t="n">
-        <v>0.615385</v>
+        <v>0.571429</v>
       </c>
       <c r="K9" t="n">
         <v>6</v>
@@ -1923,55 +1923,55 @@
         <v>7</v>
       </c>
       <c r="M9" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="N9" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="O9" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>3.8462</v>
+        <v>3.7143</v>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>3.1538</v>
+        <v>3.2857</v>
       </c>
       <c r="R9" s="2" t="n">
-        <v>28.61538</v>
+        <v>28.57142</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>30</v>
+        <v>30.28571</v>
       </c>
       <c r="T9" s="1" t="n">
-        <v>0.302325</v>
+        <v>0.288888</v>
       </c>
       <c r="U9" s="1" t="n">
-        <v>0.952381</v>
+        <v>0.936171</v>
       </c>
       <c r="V9" s="1" t="n">
-        <v>0.517473</v>
+        <v>0.522443</v>
       </c>
       <c r="W9" s="1" t="n">
-        <v>0.47038</v>
+        <v>0.46367</v>
       </c>
       <c r="X9" s="1" t="n">
-        <v>0.48045</v>
+        <v>0.47526</v>
       </c>
       <c r="Y9" s="1" t="n">
-        <v>0.49232</v>
+        <v>0.49186</v>
       </c>
       <c r="Z9" s="1" t="n">
-        <v>0.11071</v>
+        <v>0.11111</v>
       </c>
       <c r="AA9" s="1" t="n">
-        <v>0.89152</v>
+        <v>0.89341</v>
       </c>
       <c r="AB9" s="3" t="n">
-        <v>1.00223</v>
+        <v>1.00452</v>
       </c>
       <c r="AC9" s="1" t="n">
-        <v>0.50146</v>
+        <v>0.49175</v>
       </c>
       <c r="AD9" t="n">
         <v>8</v>
@@ -1992,46 +1992,46 @@
         <v>25</v>
       </c>
       <c r="AJ9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK9" t="n">
         <v>3</v>
       </c>
       <c r="AL9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM9" t="n">
         <v>1</v>
       </c>
       <c r="AN9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="AO9" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="AP9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR9" t="n">
         <v>2</v>
       </c>
       <c r="AS9" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="AT9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AU9" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
         <v>27.72727</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>21.81818</v>
+        <v>21.72727</v>
       </c>
       <c r="T11" s="1" t="n">
         <v>0.185185</v>
@@ -2281,10 +2281,10 @@
         <v>0.09132</v>
       </c>
       <c r="AA11" s="1" t="n">
-        <v>0.92655</v>
+        <v>0.92613</v>
       </c>
       <c r="AB11" s="3" t="n">
-        <v>1.01787</v>
+        <v>1.01745</v>
       </c>
       <c r="AC11" s="1" t="n">
         <v>0.49038</v>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -2531,13 +2531,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F13" t="n">
         <v>7</v>
       </c>
       <c r="G13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
@@ -2546,7 +2546,7 @@
         <v>15</v>
       </c>
       <c r="J13" s="1" t="n">
-        <v>0.576923</v>
+        <v>0.535714</v>
       </c>
       <c r="K13" t="n">
         <v>7</v>
@@ -2555,73 +2555,73 @@
         <v>7</v>
       </c>
       <c r="M13" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="N13" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="O13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>3.1538</v>
+        <v>3.1429</v>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>2.7692</v>
+        <v>3</v>
       </c>
       <c r="R13" s="2" t="n">
-        <v>24.53846</v>
+        <v>24.71428</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>26.30769</v>
+        <v>26.28571</v>
       </c>
       <c r="T13" s="1" t="n">
-        <v>0.189189</v>
+        <v>0.210526</v>
       </c>
       <c r="U13" s="1" t="n">
-        <v>0.923077</v>
+        <v>0.904762</v>
       </c>
       <c r="V13" s="1" t="n">
-        <v>0.53412</v>
+        <v>0.538274</v>
       </c>
       <c r="W13" s="1" t="n">
-        <v>0.47627</v>
+        <v>0.48139</v>
       </c>
       <c r="X13" s="1" t="n">
-        <v>0.465</v>
+        <v>0.47289</v>
       </c>
       <c r="Y13" s="1" t="n">
-        <v>0.46656</v>
+        <v>0.47323</v>
       </c>
       <c r="Z13" s="1" t="n">
-        <v>0.10569</v>
+        <v>0.1</v>
       </c>
       <c r="AA13" s="1" t="n">
-        <v>0.90334</v>
+        <v>0.8986</v>
       </c>
       <c r="AB13" s="3" t="n">
-        <v>1.00903</v>
+        <v>0.9986</v>
       </c>
       <c r="AC13" s="1" t="n">
-        <v>0.47244</v>
+        <v>0.48039</v>
       </c>
       <c r="AD13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AE13" t="n">
         <v>6</v>
       </c>
       <c r="AF13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG13" t="n">
         <v>0</v>
       </c>
       <c r="AH13" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="AI13" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="AJ13" t="n">
         <v>7</v>
@@ -2642,28 +2642,28 @@
         <v>26</v>
       </c>
       <c r="AP13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AQ13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR13" t="n">
         <v>1</v>
       </c>
       <c r="AS13" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AT13" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -2743,13 +2743,13 @@
         <v>0.511475</v>
       </c>
       <c r="W14" s="1" t="n">
-        <v>0.59774</v>
+        <v>0.59736</v>
       </c>
       <c r="X14" s="1" t="n">
-        <v>0.59491</v>
+        <v>0.59437</v>
       </c>
       <c r="Y14" s="1" t="n">
-        <v>0.60273</v>
+        <v>0.60205</v>
       </c>
       <c r="Z14" s="1" t="n">
         <v>0.07692</v>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3044,7 @@
         <v>3</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>28.5</v>
+        <v>28.58333</v>
       </c>
       <c r="S16" s="2" t="n">
         <v>24.08333</v>
@@ -3068,13 +3068,13 @@
         <v>0.5837599999999999</v>
       </c>
       <c r="Z16" s="1" t="n">
-        <v>0.07826</v>
+        <v>0.07792</v>
       </c>
       <c r="AA16" s="1" t="n">
         <v>0.88083</v>
       </c>
       <c r="AB16" s="3" t="n">
-        <v>0.95909</v>
+        <v>0.95875</v>
       </c>
       <c r="AC16" s="1" t="n">
         <v>0.57859</v>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
         <v>0.75</v>
       </c>
       <c r="V17" s="1" t="n">
-        <v>0.464285</v>
+        <v>0.462912</v>
       </c>
       <c r="W17" s="1" t="n">
         <v>0.5144300000000001</v>
@@ -3295,42 +3295,42 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>San Jose Sharks</t>
+          <t>Detroit Red Wings</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SJS</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>12</v>
       </c>
       <c r="F18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I18" t="n">
         <v>13</v>
@@ -3339,225 +3339,225 @@
         <v>0.541667</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M18" t="n">
+        <v>33</v>
+      </c>
+      <c r="N18" t="n">
         <v>37</v>
       </c>
-      <c r="N18" t="n">
-        <v>43</v>
-      </c>
       <c r="O18" t="n">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="P18" s="2" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="Q18" s="2" t="n">
         <v>3.0833</v>
       </c>
-      <c r="Q18" s="2" t="n">
-        <v>3.5833</v>
-      </c>
       <c r="R18" s="2" t="n">
-        <v>28.08333</v>
+        <v>29.83333</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>30.33333</v>
+        <v>25.75</v>
       </c>
       <c r="T18" s="1" t="n">
-        <v>0.268292</v>
+        <v>0.214285</v>
       </c>
       <c r="U18" s="1" t="n">
-        <v>0.804879</v>
+        <v>0.658537</v>
       </c>
       <c r="V18" s="1" t="n">
-        <v>0.463748</v>
+        <v>0.505681</v>
       </c>
       <c r="W18" s="1" t="n">
-        <v>0.44931</v>
+        <v>0.5340200000000001</v>
       </c>
       <c r="X18" s="1" t="n">
-        <v>0.45185</v>
+        <v>0.54777</v>
       </c>
       <c r="Y18" s="1" t="n">
-        <v>0.47254</v>
+        <v>0.50995</v>
       </c>
       <c r="Z18" s="1" t="n">
-        <v>0.064</v>
+        <v>0.07462000000000001</v>
       </c>
       <c r="AA18" s="1" t="n">
-        <v>0.89925</v>
+        <v>0.91593</v>
       </c>
       <c r="AB18" s="3" t="n">
-        <v>0.9632500000000001</v>
+        <v>0.99055</v>
       </c>
       <c r="AC18" s="1" t="n">
-        <v>0.45081</v>
+        <v>0.50887</v>
       </c>
       <c r="AD18" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AE18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH18" t="n">
+        <v>20</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>23</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN18" t="n">
         <v>13</v>
       </c>
-      <c r="AI18" t="n">
-        <v>16</v>
-      </c>
-      <c r="AJ18" t="n">
-        <v>8</v>
-      </c>
-      <c r="AK18" t="n">
-        <v>4</v>
-      </c>
-      <c r="AL18" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN18" t="n">
-        <v>24</v>
-      </c>
       <c r="AO18" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="AP18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AQ18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AR18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS18" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="AT18" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Washington Capitals</t>
+          <t>San Jose Sharks</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F19" t="n">
         <v>6</v>
       </c>
       <c r="G19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J19" s="1" t="n">
-        <v>0.6</v>
+        <v>0.541667</v>
       </c>
       <c r="K19" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M19" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N19" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="O19" t="n">
-        <v>2</v>
+        <v>-6</v>
       </c>
       <c r="P19" s="2" t="n">
-        <v>3.4</v>
+        <v>3.0833</v>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>3.2</v>
+        <v>3.5833</v>
       </c>
       <c r="R19" s="2" t="n">
-        <v>27.5</v>
+        <v>28.08333</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>28.4</v>
+        <v>30.33333</v>
       </c>
       <c r="T19" s="1" t="n">
-        <v>0.178571</v>
+        <v>0.268292</v>
       </c>
       <c r="U19" s="1" t="n">
-        <v>0.8125</v>
+        <v>0.804879</v>
       </c>
       <c r="V19" s="1" t="n">
-        <v>0.501773</v>
+        <v>0.463748</v>
       </c>
       <c r="W19" s="1" t="n">
-        <v>0.46959</v>
+        <v>0.45022</v>
       </c>
       <c r="X19" s="1" t="n">
-        <v>0.48387</v>
+        <v>0.45241</v>
       </c>
       <c r="Y19" s="1" t="n">
-        <v>0.47993</v>
+        <v>0.47314</v>
       </c>
       <c r="Z19" s="1" t="n">
-        <v>0.12745</v>
+        <v>0.064</v>
       </c>
       <c r="AA19" s="1" t="n">
-        <v>0.89201</v>
+        <v>0.89925</v>
       </c>
       <c r="AB19" s="3" t="n">
-        <v>1.01946</v>
+        <v>0.9632500000000001</v>
       </c>
       <c r="AC19" s="1" t="n">
-        <v>0.42804</v>
+        <v>0.45081</v>
       </c>
       <c r="AD19" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AE19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AF19" t="n">
         <v>2</v>
@@ -3566,64 +3566,64 @@
         <v>0</v>
       </c>
       <c r="AH19" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="AI19" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="AJ19" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="AK19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AL19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN19" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="AO19" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="AP19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AQ19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS19" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="AT19" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="AU19" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>New York Islanders</t>
+          <t>Washington Capitals</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NYI</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3637,174 +3637,174 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G20" t="n">
         <v>4</v>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
         <v>12</v>
       </c>
       <c r="J20" s="1" t="n">
-        <v>0.545455</v>
+        <v>0.6</v>
       </c>
       <c r="K20" t="n">
         <v>5</v>
       </c>
       <c r="L20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M20" t="n">
+        <v>34</v>
+      </c>
+      <c r="N20" t="n">
         <v>32</v>
       </c>
-      <c r="N20" t="n">
-        <v>29</v>
-      </c>
       <c r="O20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P20" s="2" t="n">
-        <v>2.9091</v>
+        <v>3.4</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>2.6364</v>
+        <v>3.2</v>
       </c>
       <c r="R20" s="2" t="n">
-        <v>26.0909</v>
+        <v>27.5</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>26.63636</v>
+        <v>28.4</v>
       </c>
       <c r="T20" s="1" t="n">
-        <v>0.181818</v>
+        <v>0.178571</v>
       </c>
       <c r="U20" s="1" t="n">
-        <v>0.861112</v>
+        <v>0.8125</v>
       </c>
       <c r="V20" s="1" t="n">
-        <v>0.54578</v>
+        <v>0.501773</v>
       </c>
       <c r="W20" s="1" t="n">
-        <v>0.51789</v>
+        <v>0.46959</v>
       </c>
       <c r="X20" s="1" t="n">
-        <v>0.50589</v>
+        <v>0.48387</v>
       </c>
       <c r="Y20" s="1" t="n">
-        <v>0.54174</v>
+        <v>0.47993</v>
       </c>
       <c r="Z20" s="1" t="n">
-        <v>0.09375</v>
+        <v>0.12745</v>
       </c>
       <c r="AA20" s="1" t="n">
-        <v>0.9276</v>
+        <v>0.89201</v>
       </c>
       <c r="AB20" s="3" t="n">
-        <v>1.02135</v>
+        <v>1.01946</v>
       </c>
       <c r="AC20" s="1" t="n">
-        <v>0.51162</v>
+        <v>0.42804</v>
       </c>
       <c r="AD20" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>26</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>23</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>8</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>9</v>
+      </c>
+      <c r="AP20" t="n">
         <v>6</v>
       </c>
-      <c r="AE20" t="n">
-        <v>4</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH20" t="n">
-        <v>21</v>
-      </c>
-      <c r="AI20" t="n">
-        <v>13</v>
-      </c>
-      <c r="AJ20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>11</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>16</v>
-      </c>
-      <c r="AP20" t="n">
-        <v>5</v>
-      </c>
       <c r="AQ20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS20" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="AT20" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="AU20" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nashville Predators</t>
+          <t>New York Islanders</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NSH</t>
+          <t>NYI</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E21" t="n">
         <v>11</v>
       </c>
       <c r="F21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
         <v>12</v>
@@ -3813,133 +3813,133 @@
         <v>0.545455</v>
       </c>
       <c r="K21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M21" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N21" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="O21" t="n">
-        <v>-4</v>
+        <v>3</v>
       </c>
       <c r="P21" s="2" t="n">
-        <v>2.8182</v>
+        <v>2.9091</v>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>3.1818</v>
+        <v>2.6364</v>
       </c>
       <c r="R21" s="2" t="n">
-        <v>25.81818</v>
+        <v>26</v>
       </c>
       <c r="S21" s="2" t="n">
-        <v>29.27272</v>
+        <v>26.63636</v>
       </c>
       <c r="T21" s="1" t="n">
-        <v>0.333333</v>
+        <v>0.181818</v>
       </c>
       <c r="U21" s="1" t="n">
-        <v>0.857143</v>
+        <v>0.861112</v>
       </c>
       <c r="V21" s="1" t="n">
-        <v>0.505511</v>
+        <v>0.54578</v>
       </c>
       <c r="W21" s="1" t="n">
-        <v>0.44533</v>
+        <v>0.51789</v>
       </c>
       <c r="X21" s="1" t="n">
-        <v>0.45765</v>
+        <v>0.50589</v>
       </c>
       <c r="Y21" s="1" t="n">
-        <v>0.42446</v>
+        <v>0.54174</v>
       </c>
       <c r="Z21" s="1" t="n">
-        <v>0.06829</v>
+        <v>0.09417</v>
       </c>
       <c r="AA21" s="1" t="n">
-        <v>0.91304</v>
+        <v>0.9276</v>
       </c>
       <c r="AB21" s="3" t="n">
-        <v>0.98133</v>
+        <v>1.02177</v>
       </c>
       <c r="AC21" s="1" t="n">
-        <v>0.45859</v>
+        <v>0.51162</v>
       </c>
       <c r="AD21" t="n">
         <v>6</v>
       </c>
       <c r="AE21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG21" t="n">
         <v>1</v>
       </c>
       <c r="AH21" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="AI21" t="n">
+        <v>13</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>11</v>
+      </c>
+      <c r="AO21" t="n">
         <v>16</v>
       </c>
-      <c r="AJ21" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK21" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL21" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM21" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN21" t="n">
-        <v>13</v>
-      </c>
-      <c r="AO21" t="n">
-        <v>19</v>
-      </c>
       <c r="AP21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AQ21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AS21" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AT21" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="AU21" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>St. Louis Blues</t>
+          <t>Nashville Predators</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>NSH</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3956,148 +3956,148 @@
         <v>11</v>
       </c>
       <c r="F22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J22" s="1" t="n">
-        <v>0.5</v>
+        <v>0.545455</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M22" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N22" t="n">
         <v>35</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="P22" s="2" t="n">
-        <v>3.1818</v>
+        <v>2.8182</v>
       </c>
       <c r="Q22" s="2" t="n">
         <v>3.1818</v>
       </c>
       <c r="R22" s="2" t="n">
-        <v>26.45454</v>
+        <v>25.81818</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>28.45454</v>
+        <v>29.27272</v>
       </c>
       <c r="T22" s="1" t="n">
-        <v>0.241379</v>
+        <v>0.333333</v>
       </c>
       <c r="U22" s="1" t="n">
-        <v>0.827587</v>
+        <v>0.857143</v>
       </c>
       <c r="V22" s="1" t="n">
-        <v>0.488549</v>
+        <v>0.507086</v>
       </c>
       <c r="W22" s="1" t="n">
-        <v>0.49284</v>
+        <v>0.44533</v>
       </c>
       <c r="X22" s="1" t="n">
-        <v>0.46704</v>
+        <v>0.45765</v>
       </c>
       <c r="Y22" s="1" t="n">
-        <v>0.49122</v>
+        <v>0.42446</v>
       </c>
       <c r="Z22" s="1" t="n">
-        <v>0.0881</v>
+        <v>0.06829</v>
       </c>
       <c r="AA22" s="1" t="n">
-        <v>0.89583</v>
+        <v>0.91304</v>
       </c>
       <c r="AB22" s="3" t="n">
-        <v>0.98393</v>
+        <v>0.98133</v>
       </c>
       <c r="AC22" s="1" t="n">
-        <v>0.5</v>
+        <v>0.45859</v>
       </c>
       <c r="AD22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE22" t="n">
         <v>3</v>
       </c>
       <c r="AF22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG22" t="n">
         <v>1</v>
       </c>
       <c r="AH22" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="AI22" t="n">
+        <v>16</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN22" t="n">
         <v>13</v>
       </c>
-      <c r="AJ22" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK22" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL22" t="n">
-        <v>4</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN22" t="n">
-        <v>20</v>
-      </c>
       <c r="AO22" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="AP22" t="n">
         <v>4</v>
       </c>
       <c r="AQ22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AR22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AS22" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AT22" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AU22" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Winnipeg Jets</t>
+          <t>St. Louis Blues</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>WPG</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4114,13 +4114,13 @@
         <v>11</v>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I23" t="n">
         <v>11</v>
@@ -4129,70 +4129,70 @@
         <v>0.5</v>
       </c>
       <c r="K23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M23" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="N23" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="O23" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="P23" s="2" t="n">
-        <v>2.4545</v>
+        <v>3.1818</v>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>2.8182</v>
+        <v>3.1818</v>
       </c>
       <c r="R23" s="2" t="n">
-        <v>27.18181</v>
+        <v>26.45454</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>29.18181</v>
+        <v>28.45454</v>
       </c>
       <c r="T23" s="1" t="n">
-        <v>0.193548</v>
+        <v>0.241379</v>
       </c>
       <c r="U23" s="1" t="n">
-        <v>0.807693</v>
+        <v>0.827587</v>
       </c>
       <c r="V23" s="1" t="n">
-        <v>0.454253</v>
+        <v>0.488549</v>
       </c>
       <c r="W23" s="1" t="n">
-        <v>0.47821</v>
+        <v>0.49284</v>
       </c>
       <c r="X23" s="1" t="n">
-        <v>0.47272</v>
+        <v>0.46704</v>
       </c>
       <c r="Y23" s="1" t="n">
-        <v>0.48068</v>
+        <v>0.49122</v>
       </c>
       <c r="Z23" s="1" t="n">
-        <v>0.09012000000000001</v>
+        <v>0.0881</v>
       </c>
       <c r="AA23" s="1" t="n">
-        <v>0.92549</v>
+        <v>0.89583</v>
       </c>
       <c r="AB23" s="3" t="n">
-        <v>1.01561</v>
+        <v>0.98393</v>
       </c>
       <c r="AC23" s="1" t="n">
-        <v>0.46418</v>
+        <v>0.5</v>
       </c>
       <c r="AD23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AE23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AG23" t="n">
         <v>1</v>
@@ -4201,40 +4201,40 @@
         <v>15</v>
       </c>
       <c r="AI23" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="AJ23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK23" t="n">
         <v>2</v>
       </c>
       <c r="AL23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AM23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AN23" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="AO23" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AP23" t="n">
         <v>4</v>
       </c>
       <c r="AQ23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS23" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="AT23" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="AU23" t="inlineStr">
         <is>
@@ -4243,29 +4243,29 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Detroit Red Wings</t>
+          <t>Winnipeg Jets</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -4287,67 +4287,67 @@
         <v>0.5</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M24" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="N24" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O24" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="P24" s="2" t="n">
-        <v>2.6364</v>
+        <v>2.4545</v>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>3.0909</v>
+        <v>2.8182</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>29.81818</v>
+        <v>27.18181</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>25.54545</v>
+        <v>29.18181</v>
       </c>
       <c r="T24" s="1" t="n">
-        <v>0.210526</v>
+        <v>0.193548</v>
       </c>
       <c r="U24" s="1" t="n">
-        <v>0.657895</v>
+        <v>0.807693</v>
       </c>
       <c r="V24" s="1" t="n">
-        <v>0.500777</v>
+        <v>0.454253</v>
       </c>
       <c r="W24" s="1" t="n">
-        <v>0.53407</v>
+        <v>0.47821</v>
       </c>
       <c r="X24" s="1" t="n">
-        <v>0.5497</v>
+        <v>0.47272</v>
       </c>
       <c r="Y24" s="1" t="n">
-        <v>0.50946</v>
+        <v>0.48068</v>
       </c>
       <c r="Z24" s="1" t="n">
-        <v>0.07722999999999999</v>
+        <v>0.09012000000000001</v>
       </c>
       <c r="AA24" s="1" t="n">
-        <v>0.91866</v>
+        <v>0.92549</v>
       </c>
       <c r="AB24" s="3" t="n">
-        <v>0.9958900000000001</v>
+        <v>1.01561</v>
       </c>
       <c r="AC24" s="1" t="n">
-        <v>0.51935</v>
+        <v>0.46418</v>
       </c>
       <c r="AD24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AE24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF24" t="n">
         <v>3</v>
@@ -4356,16 +4356,16 @@
         <v>1</v>
       </c>
       <c r="AH24" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="AI24" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="AJ24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AK24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL24" t="n">
         <v>1</v>
@@ -4374,25 +4374,25 @@
         <v>2</v>
       </c>
       <c r="AN24" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="AO24" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AP24" t="n">
         <v>4</v>
       </c>
       <c r="AQ24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AS24" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="AT24" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="AU24" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -4717,19 +4717,19 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Anaheim Ducks</t>
+          <t>Calgary Flames</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ANA</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4761,67 +4761,67 @@
         <v>0.454545</v>
       </c>
       <c r="K27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L27" t="n">
         <v>5</v>
       </c>
       <c r="M27" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="N27" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="O27" t="n">
-        <v>-5</v>
+        <v>-13</v>
       </c>
       <c r="P27" s="2" t="n">
-        <v>2.9091</v>
+        <v>2.5455</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>3.3636</v>
+        <v>3.7273</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>23.54545</v>
+        <v>29.18181</v>
       </c>
       <c r="S27" s="2" t="n">
-        <v>27.18181</v>
+        <v>30.36363</v>
       </c>
       <c r="T27" s="1" t="n">
-        <v>0.222222</v>
+        <v>0.3</v>
       </c>
       <c r="U27" s="1" t="n">
-        <v>0.7619050000000001</v>
+        <v>0.857143</v>
       </c>
       <c r="V27" s="1" t="n">
-        <v>0.445151</v>
+        <v>0.487767</v>
       </c>
       <c r="W27" s="1" t="n">
-        <v>0.47628</v>
+        <v>0.51761</v>
       </c>
       <c r="X27" s="1" t="n">
-        <v>0.47949</v>
+        <v>0.5031600000000001</v>
       </c>
       <c r="Y27" s="1" t="n">
-        <v>0.461</v>
+        <v>0.50696</v>
       </c>
       <c r="Z27" s="1" t="n">
-        <v>0.09708</v>
+        <v>0.05791</v>
       </c>
       <c r="AA27" s="1" t="n">
-        <v>0.90517</v>
+        <v>0.8807700000000001</v>
       </c>
       <c r="AB27" s="3" t="n">
-        <v>1.00225</v>
+        <v>0.93868</v>
       </c>
       <c r="AC27" s="1" t="n">
-        <v>0.49834</v>
+        <v>0.50445</v>
       </c>
       <c r="AD27" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AE27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AF27" t="n">
         <v>3</v>
@@ -4830,16 +4830,16 @@
         <v>0</v>
       </c>
       <c r="AH27" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="AI27" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="AJ27" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AK27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AL27" t="n">
         <v>3</v>
@@ -4848,204 +4848,204 @@
         <v>0</v>
       </c>
       <c r="AN27" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="AO27" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="AP27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AQ27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR27" t="n">
         <v>0</v>
       </c>
       <c r="AS27" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AT27" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AU27" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Philadelphia Flyers</t>
+          <t>Anaheim Ducks</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>ANA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G28" t="n">
+        <v>6</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>10</v>
+      </c>
+      <c r="J28" s="1" t="n">
+        <v>0.454545</v>
+      </c>
+      <c r="K28" t="n">
+        <v>4</v>
+      </c>
+      <c r="L28" t="n">
+        <v>5</v>
+      </c>
+      <c r="M28" t="n">
+        <v>32</v>
+      </c>
+      <c r="N28" t="n">
+        <v>37</v>
+      </c>
+      <c r="O28" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>2.9091</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>3.3636</v>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>23.54545</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>27.18181</v>
+      </c>
+      <c r="T28" s="1" t="n">
+        <v>0.222222</v>
+      </c>
+      <c r="U28" s="1" t="n">
+        <v>0.7619050000000001</v>
+      </c>
+      <c r="V28" s="1" t="n">
+        <v>0.445151</v>
+      </c>
+      <c r="W28" s="1" t="n">
+        <v>0.47628</v>
+      </c>
+      <c r="X28" s="1" t="n">
+        <v>0.47949</v>
+      </c>
+      <c r="Y28" s="1" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="Z28" s="1" t="n">
+        <v>0.09708</v>
+      </c>
+      <c r="AA28" s="1" t="n">
+        <v>0.90517</v>
+      </c>
+      <c r="AB28" s="3" t="n">
+        <v>1.00225</v>
+      </c>
+      <c r="AC28" s="1" t="n">
+        <v>0.49834</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>9</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>15</v>
+      </c>
+      <c r="AJ28" t="n">
         <v>7</v>
       </c>
-      <c r="H28" t="n">
-        <v>3</v>
-      </c>
-      <c r="I28" t="n">
-        <v>9</v>
-      </c>
-      <c r="J28" s="1" t="n">
-        <v>0.346154</v>
-      </c>
-      <c r="K28" t="n">
-        <v>3</v>
-      </c>
-      <c r="L28" t="n">
-        <v>3</v>
-      </c>
-      <c r="M28" t="n">
-        <v>24</v>
-      </c>
-      <c r="N28" t="n">
-        <v>42</v>
-      </c>
-      <c r="O28" t="n">
-        <v>-18</v>
-      </c>
-      <c r="P28" s="2" t="n">
-        <v>1.8462</v>
-      </c>
-      <c r="Q28" s="2" t="n">
-        <v>3.2308</v>
-      </c>
-      <c r="R28" s="2" t="n">
-        <v>22.6923</v>
-      </c>
-      <c r="S28" s="2" t="n">
-        <v>31.46153</v>
-      </c>
-      <c r="T28" s="1" t="n">
-        <v>0.16279</v>
-      </c>
-      <c r="U28" s="1" t="n">
-        <v>0.826087</v>
-      </c>
-      <c r="V28" s="1" t="n">
-        <v>0.50717</v>
-      </c>
-      <c r="W28" s="1" t="n">
-        <v>0.42359</v>
-      </c>
-      <c r="X28" s="1" t="n">
-        <v>0.40832</v>
-      </c>
-      <c r="Y28" s="1" t="n">
-        <v>0.41492</v>
-      </c>
-      <c r="Z28" s="1" t="n">
-        <v>0.06074</v>
-      </c>
-      <c r="AA28" s="1" t="n">
-        <v>0.9035300000000001</v>
-      </c>
-      <c r="AB28" s="3" t="n">
-        <v>0.96427</v>
-      </c>
-      <c r="AC28" s="1" t="n">
-        <v>0.41207</v>
-      </c>
-      <c r="AD28" t="n">
-        <v>7</v>
-      </c>
-      <c r="AE28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF28" t="n">
-        <v>3</v>
-      </c>
-      <c r="AG28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH28" t="n">
-        <v>15</v>
-      </c>
-      <c r="AI28" t="n">
-        <v>25</v>
-      </c>
-      <c r="AJ28" t="n">
-        <v>6</v>
-      </c>
       <c r="AK28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AL28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AM28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN28" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="AO28" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="AP28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AQ28" t="n">
         <v>6</v>
       </c>
       <c r="AR28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS28" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="AT28" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="AU28" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Columbus Blue Jackets</t>
+          <t>Philadelphia Flyers</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CBJ</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5059,171 +5059,171 @@
         </is>
       </c>
       <c r="E29" t="n">
+        <v>13</v>
+      </c>
+      <c r="F29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" t="n">
+        <v>7</v>
+      </c>
+      <c r="H29" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" t="n">
         <v>9</v>
       </c>
-      <c r="F29" t="n">
-        <v>4</v>
-      </c>
-      <c r="G29" t="n">
-        <v>5</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" t="n">
-        <v>8</v>
-      </c>
       <c r="J29" s="1" t="n">
-        <v>0.444444</v>
+        <v>0.346154</v>
       </c>
       <c r="K29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L29" t="n">
         <v>3</v>
       </c>
       <c r="M29" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="N29" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="O29" t="n">
-        <v>-8</v>
+        <v>-18</v>
       </c>
       <c r="P29" s="2" t="n">
-        <v>2.4444</v>
+        <v>1.8462</v>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>3.3333</v>
+        <v>3.2308</v>
       </c>
       <c r="R29" s="2" t="n">
-        <v>26.77777</v>
+        <v>22.6923</v>
       </c>
       <c r="S29" s="2" t="n">
-        <v>27.66666</v>
+        <v>31.46153</v>
       </c>
       <c r="T29" s="1" t="n">
-        <v>0.115384</v>
+        <v>0.16279</v>
       </c>
       <c r="U29" s="1" t="n">
-        <v>0.709678</v>
+        <v>0.826087</v>
       </c>
       <c r="V29" s="1" t="n">
-        <v>0.546816</v>
+        <v>0.50717</v>
       </c>
       <c r="W29" s="1" t="n">
-        <v>0.48877</v>
+        <v>0.42359</v>
       </c>
       <c r="X29" s="1" t="n">
-        <v>0.48076</v>
+        <v>0.40832</v>
       </c>
       <c r="Y29" s="1" t="n">
-        <v>0.46048</v>
+        <v>0.41492</v>
       </c>
       <c r="Z29" s="1" t="n">
-        <v>0.08379</v>
+        <v>0.06074</v>
       </c>
       <c r="AA29" s="1" t="n">
-        <v>0.91709</v>
+        <v>0.9035300000000001</v>
       </c>
       <c r="AB29" s="3" t="n">
-        <v>1.00088</v>
+        <v>0.96427</v>
       </c>
       <c r="AC29" s="1" t="n">
-        <v>0.49629</v>
+        <v>0.41207</v>
       </c>
       <c r="AD29" t="n">
         <v>7</v>
       </c>
       <c r="AE29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AF29" t="n">
         <v>3</v>
       </c>
       <c r="AG29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AH29" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AI29" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="AJ29" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AK29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AM29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN29" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AO29" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="AP29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AQ29" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AR29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS29" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="AT29" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AU29" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Calgary Flames</t>
+          <t>Columbus Blue Jackets</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F30" t="n">
         <v>4</v>
       </c>
       <c r="G30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -5232,70 +5232,70 @@
         <v>8</v>
       </c>
       <c r="J30" s="1" t="n">
-        <v>0.4</v>
+        <v>0.444444</v>
       </c>
       <c r="K30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M30" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N30" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="O30" t="n">
-        <v>-16</v>
+        <v>-8</v>
       </c>
       <c r="P30" s="2" t="n">
-        <v>2.3</v>
+        <v>2.4444</v>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>3.9</v>
+        <v>3.3333</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>28.7</v>
+        <v>26.77777</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>30.5</v>
+        <v>27.66666</v>
       </c>
       <c r="T30" s="1" t="n">
-        <v>0.32</v>
+        <v>0.115384</v>
       </c>
       <c r="U30" s="1" t="n">
-        <v>0.848485</v>
+        <v>0.709678</v>
       </c>
       <c r="V30" s="1" t="n">
-        <v>0.494966</v>
+        <v>0.546816</v>
       </c>
       <c r="W30" s="1" t="n">
-        <v>0.5097</v>
+        <v>0.48813</v>
       </c>
       <c r="X30" s="1" t="n">
-        <v>0.49587</v>
+        <v>0.47985</v>
       </c>
       <c r="Y30" s="1" t="n">
-        <v>0.50632</v>
+        <v>0.45955</v>
       </c>
       <c r="Z30" s="1" t="n">
-        <v>0.05531</v>
+        <v>0.08379</v>
       </c>
       <c r="AA30" s="1" t="n">
-        <v>0.8801600000000001</v>
+        <v>0.91709</v>
       </c>
       <c r="AB30" s="3" t="n">
-        <v>0.93547</v>
+        <v>1.00088</v>
       </c>
       <c r="AC30" s="1" t="n">
-        <v>0.49363</v>
+        <v>0.49629</v>
       </c>
       <c r="AD30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AE30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF30" t="n">
         <v>3</v>
@@ -5304,52 +5304,52 @@
         <v>0</v>
       </c>
       <c r="AH30" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="AI30" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="AJ30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AK30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AM30" t="n">
         <v>0</v>
       </c>
       <c r="AN30" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AO30" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="AP30" t="n">
         <v>4</v>
       </c>
       <c r="AQ30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR30" t="n">
         <v>0</v>
       </c>
       <c r="AS30" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="AT30" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="AU30" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -5375,10 +5375,10 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G31" t="n">
         <v>5</v>
@@ -5387,67 +5387,67 @@
         <v>2</v>
       </c>
       <c r="I31" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J31" s="1" t="n">
-        <v>0.333333</v>
+        <v>0.4</v>
       </c>
       <c r="K31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M31" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="N31" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="O31" t="n">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="P31" s="2" t="n">
-        <v>2.3333</v>
+        <v>2.7</v>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>3.5556</v>
+        <v>3.5</v>
       </c>
       <c r="R31" s="2" t="n">
-        <v>27.22222</v>
+        <v>27.1</v>
       </c>
       <c r="S31" s="2" t="n">
-        <v>29.11111</v>
+        <v>28.8</v>
       </c>
       <c r="T31" s="1" t="n">
-        <v>0.148148</v>
+        <v>0.166666</v>
       </c>
       <c r="U31" s="1" t="n">
-        <v>0.655173</v>
+        <v>0.633334</v>
       </c>
       <c r="V31" s="1" t="n">
-        <v>0.50996</v>
+        <v>0.499111</v>
       </c>
       <c r="W31" s="1" t="n">
-        <v>0.48339</v>
+        <v>0.48131</v>
       </c>
       <c r="X31" s="1" t="n">
-        <v>0.48969</v>
+        <v>0.48456</v>
       </c>
       <c r="Y31" s="1" t="n">
-        <v>0.44821</v>
+        <v>0.44406</v>
       </c>
       <c r="Z31" s="1" t="n">
-        <v>0.06521</v>
+        <v>0.07462000000000001</v>
       </c>
       <c r="AA31" s="1" t="n">
-        <v>0.91414</v>
+        <v>0.91855</v>
       </c>
       <c r="AB31" s="3" t="n">
-        <v>0.9793500000000001</v>
+        <v>0.99317</v>
       </c>
       <c r="AC31" s="1" t="n">
-        <v>0.45967</v>
+        <v>0.45454</v>
       </c>
       <c r="AD31" t="n">
         <v>3</v>
@@ -5468,10 +5468,10 @@
         <v>10</v>
       </c>
       <c r="AJ31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AK31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL31" t="n">
         <v>2</v>
@@ -5480,13 +5480,13 @@
         <v>2</v>
       </c>
       <c r="AN31" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="AO31" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="AP31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AQ31" t="n">
         <v>5</v>
@@ -5495,19 +5495,19 @@
         <v>2</v>
       </c>
       <c r="AS31" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AT31" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="AU31" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -5575,7 +5575,7 @@
         <v>21.36363</v>
       </c>
       <c r="S32" s="2" t="n">
-        <v>30.54545</v>
+        <v>30.63636</v>
       </c>
       <c r="T32" s="1" t="n">
         <v>0.083333</v>
@@ -5599,10 +5599,10 @@
         <v>0.08938</v>
       </c>
       <c r="AA32" s="1" t="n">
-        <v>0.88973</v>
+        <v>0.89015</v>
       </c>
       <c r="AB32" s="3" t="n">
-        <v>0.97911</v>
+        <v>0.97953</v>
       </c>
       <c r="AC32" s="1" t="n">
         <v>0.45806</v>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
         <v>0.644445</v>
       </c>
       <c r="V33" s="1" t="n">
-        <v>0.477568</v>
+        <v>0.476121</v>
       </c>
       <c r="W33" s="1" t="n">
         <v>0.40949</v>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-26 10:07</t>
+          <t>2026-10-27 02:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-27 08:19 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-27 02:52</t>
+          <t>2026-10-27 08:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-28 08:21 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-28 03:04</t>
+          <t>2026-10-28 08:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-29 03:05 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -835,7 +835,7 @@
         <v>33.64285</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>21.85714</v>
+        <v>21.92857</v>
       </c>
       <c r="T2" s="1" t="n">
         <v>0.235294</v>
@@ -847,22 +847,22 @@
         <v>0.501207</v>
       </c>
       <c r="W2" s="1" t="n">
-        <v>0.59685</v>
+        <v>0.59636</v>
       </c>
       <c r="X2" s="1" t="n">
-        <v>0.61547</v>
+        <v>0.61478</v>
       </c>
       <c r="Y2" s="1" t="n">
-        <v>0.60246</v>
+        <v>0.60172</v>
       </c>
       <c r="Z2" s="1" t="n">
         <v>0.09694999999999999</v>
       </c>
       <c r="AA2" s="1" t="n">
-        <v>0.90308</v>
+        <v>0.9035</v>
       </c>
       <c r="AB2" s="3" t="n">
-        <v>1.00003</v>
+        <v>1.00045</v>
       </c>
       <c r="AC2" s="1" t="n">
         <v>0.625</v>
@@ -925,19 +925,19 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Minnesota Wild</t>
+          <t>Edmonton Oilers</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>EDM</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -947,17 +947,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F3" t="n">
         <v>9</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
         <v>2</v>
@@ -966,100 +966,100 @@
         <v>20</v>
       </c>
       <c r="J3" s="1" t="n">
-        <v>0.714286</v>
+        <v>0.769231</v>
       </c>
       <c r="K3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M3" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="N3" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="O3" t="n">
         <v>13</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>3.1429</v>
+        <v>4.3077</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>2.2143</v>
+        <v>3.3077</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>31.21428</v>
+        <v>26.07692</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>25.07142</v>
+        <v>26.84615</v>
       </c>
       <c r="T3" s="1" t="n">
-        <v>0.265306</v>
+        <v>0.357142</v>
       </c>
       <c r="U3" s="1" t="n">
-        <v>0.822223</v>
+        <v>0.714286</v>
       </c>
       <c r="V3" s="1" t="n">
-        <v>0.496314</v>
+        <v>0.493333</v>
       </c>
       <c r="W3" s="1" t="n">
-        <v>0.5353599999999999</v>
+        <v>0.47652</v>
       </c>
       <c r="X3" s="1" t="n">
-        <v>0.55316</v>
+        <v>0.47699</v>
       </c>
       <c r="Y3" s="1" t="n">
-        <v>0.5281</v>
+        <v>0.51129</v>
       </c>
       <c r="Z3" s="1" t="n">
-        <v>0.08307</v>
+        <v>0.13278</v>
       </c>
       <c r="AA3" s="1" t="n">
-        <v>0.92968</v>
+        <v>0.90391</v>
       </c>
       <c r="AB3" s="3" t="n">
-        <v>1.01275</v>
+        <v>1.03669</v>
       </c>
       <c r="AC3" s="1" t="n">
-        <v>0.5501200000000001</v>
+        <v>0.52722</v>
       </c>
       <c r="AD3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AE3" t="n">
         <v>4</v>
       </c>
       <c r="AF3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>29</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>30</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL3" t="n">
         <v>0</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AM3" t="n">
         <v>0</v>
       </c>
-      <c r="AH3" t="n">
-        <v>15</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>10</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>5</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>2</v>
-      </c>
       <c r="AN3" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="AO3" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="AP3" t="n">
         <v>7</v>
@@ -1071,45 +1071,45 @@
         <v>1</v>
       </c>
       <c r="AS3" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="AT3" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Boston Bruins</t>
+          <t>Minnesota Wild</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4" t="n">
         <v>9</v>
@@ -1118,106 +1118,106 @@
         <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J4" s="1" t="n">
-        <v>0.730769</v>
+        <v>0.714286</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L4" t="n">
         <v>9</v>
       </c>
       <c r="M4" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="N4" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="O4" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>3.7692</v>
+        <v>3.1429</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>2.1538</v>
+        <v>2.2143</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>25.38461</v>
+        <v>31.28571</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>28.07692</v>
+        <v>25.07142</v>
       </c>
       <c r="T4" s="1" t="n">
-        <v>0.219512</v>
+        <v>0.265306</v>
       </c>
       <c r="U4" s="1" t="n">
-        <v>0.804348</v>
+        <v>0.822223</v>
       </c>
       <c r="V4" s="1" t="n">
-        <v>0.53437</v>
+        <v>0.496314</v>
       </c>
       <c r="W4" s="1" t="n">
-        <v>0.48453</v>
+        <v>0.5358000000000001</v>
       </c>
       <c r="X4" s="1" t="n">
-        <v>0.48989</v>
+        <v>0.55316</v>
       </c>
       <c r="Y4" s="1" t="n">
-        <v>0.48133</v>
+        <v>0.5281</v>
       </c>
       <c r="Z4" s="1" t="n">
-        <v>0.12222</v>
+        <v>0.08282</v>
       </c>
       <c r="AA4" s="1" t="n">
-        <v>0.94736</v>
+        <v>0.92968</v>
       </c>
       <c r="AB4" s="3" t="n">
-        <v>1.06958</v>
+        <v>1.0125</v>
       </c>
       <c r="AC4" s="1" t="n">
-        <v>0.48175</v>
+        <v>0.5501200000000001</v>
       </c>
       <c r="AD4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AE4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG4" t="n">
         <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="AI4" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ4" t="n">
         <v>10</v>
       </c>
-      <c r="AJ4" t="n">
-        <v>7</v>
-      </c>
       <c r="AK4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AL4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN4" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="AO4" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="AP4" t="n">
         <v>7</v>
@@ -1229,51 +1229,51 @@
         <v>1</v>
       </c>
       <c r="AS4" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="AT4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Vegas Golden Knights</t>
+          <t>Boston Bruins</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>VGK</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F5" t="n">
         <v>9</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
@@ -1282,88 +1282,88 @@
         <v>19</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>0.678571</v>
+        <v>0.730769</v>
       </c>
       <c r="K5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M5" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="N5" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="O5" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>3.6429</v>
+        <v>3.7692</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>2.7857</v>
+        <v>2.1538</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>29.71428</v>
+        <v>25.46153</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>25.14285</v>
+        <v>28.07692</v>
       </c>
       <c r="T5" s="1" t="n">
-        <v>0.255813</v>
+        <v>0.219512</v>
       </c>
       <c r="U5" s="1" t="n">
-        <v>0.676471</v>
+        <v>0.804348</v>
       </c>
       <c r="V5" s="1" t="n">
-        <v>0.503768</v>
+        <v>0.53437</v>
       </c>
       <c r="W5" s="1" t="n">
-        <v>0.52421</v>
+        <v>0.48497</v>
       </c>
       <c r="X5" s="1" t="n">
-        <v>0.54051</v>
+        <v>0.49049</v>
       </c>
       <c r="Y5" s="1" t="n">
-        <v>0.53692</v>
+        <v>0.482</v>
       </c>
       <c r="Z5" s="1" t="n">
-        <v>0.09393</v>
+        <v>0.12177</v>
       </c>
       <c r="AA5" s="1" t="n">
-        <v>0.90942</v>
+        <v>0.94736</v>
       </c>
       <c r="AB5" s="3" t="n">
-        <v>1.00335</v>
+        <v>1.06913</v>
       </c>
       <c r="AC5" s="1" t="n">
-        <v>0.51927</v>
+        <v>0.48175</v>
       </c>
       <c r="AD5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AE5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AF5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG5" t="n">
         <v>0</v>
       </c>
       <c r="AH5" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="AI5" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="AJ5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AK5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AL5" t="n">
         <v>2</v>
@@ -1372,46 +1372,46 @@
         <v>1</v>
       </c>
       <c r="AN5" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="AO5" t="n">
         <v>18</v>
       </c>
       <c r="AP5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AQ5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AR5" t="n">
         <v>1</v>
       </c>
       <c r="AS5" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="AT5" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Edmonton Oilers</t>
+          <t>Vegas Golden Knights</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>VGK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1425,165 +1425,165 @@
         </is>
       </c>
       <c r="E6" t="n">
+        <v>14</v>
+      </c>
+      <c r="F6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>19</v>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>0.678571</v>
+      </c>
+      <c r="K6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M6" t="n">
+        <v>51</v>
+      </c>
+      <c r="N6" t="n">
+        <v>39</v>
+      </c>
+      <c r="O6" t="n">
         <v>12</v>
       </c>
-      <c r="F6" t="n">
+      <c r="P6" s="2" t="n">
+        <v>3.6429</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>2.7857</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>29.71428</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>25.14285</v>
+      </c>
+      <c r="T6" s="1" t="n">
+        <v>0.255813</v>
+      </c>
+      <c r="U6" s="1" t="n">
+        <v>0.676471</v>
+      </c>
+      <c r="V6" s="1" t="n">
+        <v>0.503768</v>
+      </c>
+      <c r="W6" s="1" t="n">
+        <v>0.52384</v>
+      </c>
+      <c r="X6" s="1" t="n">
+        <v>0.5400199999999999</v>
+      </c>
+      <c r="Y6" s="1" t="n">
+        <v>0.5362</v>
+      </c>
+      <c r="Z6" s="1" t="n">
+        <v>0.09393</v>
+      </c>
+      <c r="AA6" s="1" t="n">
+        <v>0.90942</v>
+      </c>
+      <c r="AB6" s="3" t="n">
+        <v>1.00335</v>
+      </c>
+      <c r="AC6" s="1" t="n">
+        <v>0.51927</v>
+      </c>
+      <c r="AD6" t="n">
         <v>8</v>
       </c>
-      <c r="G6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" t="n">
+      <c r="AE6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>32</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>21</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>19</v>
+      </c>
+      <c r="AO6" t="n">
         <v>18</v>
       </c>
-      <c r="J6" s="1" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="K6" t="n">
+      <c r="AP6" t="n">
         <v>6</v>
       </c>
-      <c r="L6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M6" t="n">
-        <v>52</v>
-      </c>
-      <c r="N6" t="n">
-        <v>43</v>
-      </c>
-      <c r="O6" t="n">
-        <v>9</v>
-      </c>
-      <c r="P6" s="2" t="n">
-        <v>4.3333</v>
-      </c>
-      <c r="Q6" s="2" t="n">
-        <v>3.5833</v>
-      </c>
-      <c r="R6" s="2" t="n">
-        <v>25.58333</v>
-      </c>
-      <c r="S6" s="2" t="n">
-        <v>27.08333</v>
-      </c>
-      <c r="T6" s="1" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="U6" s="1" t="n">
-        <v>0.705883</v>
-      </c>
-      <c r="V6" s="1" t="n">
-        <v>0.496413</v>
-      </c>
-      <c r="W6" s="1" t="n">
-        <v>0.47558</v>
-      </c>
-      <c r="X6" s="1" t="n">
-        <v>0.47375</v>
-      </c>
-      <c r="Y6" s="1" t="n">
-        <v>0.51202</v>
-      </c>
-      <c r="Z6" s="1" t="n">
-        <v>0.13425</v>
-      </c>
-      <c r="AA6" s="1" t="n">
-        <v>0.89494</v>
-      </c>
-      <c r="AB6" s="3" t="n">
-        <v>1.02919</v>
-      </c>
-      <c r="AC6" s="1" t="n">
-        <v>0.52076</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>7</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>25</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>30</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>5</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>5</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>27</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>13</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>7</v>
-      </c>
       <c r="AQ6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR6" t="n">
         <v>1</v>
       </c>
       <c r="AS6" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="AT6" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>New Jersey Devils</t>
+          <t>Seattle Kraken</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NJD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
         <v>8</v>
@@ -1592,76 +1592,76 @@
         <v>4</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J7" s="1" t="n">
-        <v>0.666667</v>
+        <v>0.653846</v>
       </c>
       <c r="K7" t="n">
         <v>6</v>
       </c>
       <c r="L7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M7" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="N7" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="O7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>3.4167</v>
+        <v>3.8462</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>2.75</v>
+        <v>3.5385</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>33.5</v>
+        <v>25.46153</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>23.41666</v>
+        <v>31</v>
       </c>
       <c r="T7" s="1" t="n">
-        <v>0.189189</v>
+        <v>0.227272</v>
       </c>
       <c r="U7" s="1" t="n">
-        <v>0.740741</v>
+        <v>0.6756760000000001</v>
       </c>
       <c r="V7" s="1" t="n">
-        <v>0.507552</v>
+        <v>0.513108</v>
       </c>
       <c r="W7" s="1" t="n">
-        <v>0.59388</v>
+        <v>0.43056</v>
       </c>
       <c r="X7" s="1" t="n">
-        <v>0.59226</v>
+        <v>0.43019</v>
       </c>
       <c r="Y7" s="1" t="n">
-        <v>0.60358</v>
+        <v>0.48494</v>
       </c>
       <c r="Z7" s="1" t="n">
-        <v>0.08777</v>
+        <v>0.14176</v>
       </c>
       <c r="AA7" s="1" t="n">
-        <v>0.90265</v>
+        <v>0.91401</v>
       </c>
       <c r="AB7" s="3" t="n">
-        <v>0.99042</v>
+        <v>1.05577</v>
       </c>
       <c r="AC7" s="1" t="n">
-        <v>0.54466</v>
+        <v>0.43325</v>
       </c>
       <c r="AD7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AE7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AF7" t="n">
         <v>2</v>
@@ -1670,52 +1670,52 @@
         <v>0</v>
       </c>
       <c r="AH7" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="AI7" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="AJ7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AK7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL7" t="n">
         <v>2</v>
       </c>
       <c r="AM7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN7" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="AO7" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="AP7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AQ7" t="n">
         <v>3</v>
       </c>
       <c r="AR7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS7" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="AT7" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="AU7" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1780,7 @@
         <v>3</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>28</v>
+        <v>28.08333</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>28.16666</v>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
         <v>30.15384</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>24</v>
+        <v>24.07692</v>
       </c>
       <c r="T9" s="1" t="n">
         <v>0.347826</v>
@@ -1953,7 +1953,7 @@
         <v>0.548185</v>
       </c>
       <c r="W9" s="1" t="n">
-        <v>0.56311</v>
+        <v>0.56275</v>
       </c>
       <c r="X9" s="1" t="n">
         <v>0.56798</v>
@@ -1965,10 +1965,10 @@
         <v>0.08934</v>
       </c>
       <c r="AA9" s="1" t="n">
-        <v>0.89873</v>
+        <v>0.89916</v>
       </c>
       <c r="AB9" s="3" t="n">
-        <v>0.98807</v>
+        <v>0.9885</v>
       </c>
       <c r="AC9" s="1" t="n">
         <v>0.51231</v>
@@ -2031,19 +2031,19 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ottawa Senators</t>
+          <t>New Jersey Devils</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>OTT</t>
+          <t>NJD</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -2078,64 +2078,64 @@
         <v>6</v>
       </c>
       <c r="L10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M10" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="N10" t="n">
         <v>38</v>
       </c>
       <c r="O10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>3</v>
+        <v>3.3077</v>
       </c>
       <c r="Q10" s="2" t="n">
         <v>2.9231</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>25.46153</v>
+        <v>32.61538</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>26.23076</v>
+        <v>25</v>
       </c>
       <c r="T10" s="1" t="n">
-        <v>0.127272</v>
+        <v>0.175</v>
       </c>
       <c r="U10" s="1" t="n">
-        <v>0.777778</v>
+        <v>0.7241379999999999</v>
       </c>
       <c r="V10" s="1" t="n">
-        <v>0.524438</v>
+        <v>0.503429</v>
       </c>
       <c r="W10" s="1" t="n">
-        <v>0.46788</v>
+        <v>0.57485</v>
       </c>
       <c r="X10" s="1" t="n">
-        <v>0.46941</v>
+        <v>0.56753</v>
       </c>
       <c r="Y10" s="1" t="n">
-        <v>0.44045</v>
+        <v>0.57437</v>
       </c>
       <c r="Z10" s="1" t="n">
-        <v>0.103</v>
+        <v>0.08605</v>
       </c>
       <c r="AA10" s="1" t="n">
-        <v>0.92244</v>
+        <v>0.9011400000000001</v>
       </c>
       <c r="AB10" s="3" t="n">
-        <v>1.02544</v>
+        <v>0.98719</v>
       </c>
       <c r="AC10" s="1" t="n">
-        <v>0.48618</v>
+        <v>0.52699</v>
       </c>
       <c r="AD10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AE10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AF10" t="n">
         <v>2</v>
@@ -2144,16 +2144,16 @@
         <v>0</v>
       </c>
       <c r="AH10" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="AI10" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="AJ10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AK10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AL10" t="n">
         <v>3</v>
@@ -2162,25 +2162,25 @@
         <v>0</v>
       </c>
       <c r="AN10" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AO10" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AP10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AQ10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR10" t="n">
         <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="AT10" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="AU10" t="inlineStr">
         <is>
@@ -2189,19 +2189,19 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Florida Panthers</t>
+          <t>Ottawa Senators</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>OTT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2218,13 +2218,13 @@
         <v>13</v>
       </c>
       <c r="F11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>16</v>
@@ -2233,97 +2233,97 @@
         <v>0.615385</v>
       </c>
       <c r="K11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M11" t="n">
         <v>39</v>
       </c>
       <c r="N11" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P11" s="2" t="n">
         <v>3</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>2.8462</v>
+        <v>2.9231</v>
       </c>
       <c r="R11" s="2" t="n">
-        <v>28.23076</v>
+        <v>25.46153</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>24.15384</v>
+        <v>26.23076</v>
       </c>
       <c r="T11" s="1" t="n">
-        <v>0.229508</v>
+        <v>0.127272</v>
       </c>
       <c r="U11" s="1" t="n">
-        <v>0.854546</v>
+        <v>0.777778</v>
       </c>
       <c r="V11" s="1" t="n">
-        <v>0.469816</v>
+        <v>0.524438</v>
       </c>
       <c r="W11" s="1" t="n">
-        <v>0.54935</v>
+        <v>0.46831</v>
       </c>
       <c r="X11" s="1" t="n">
-        <v>0.53645</v>
+        <v>0.47003</v>
       </c>
       <c r="Y11" s="1" t="n">
-        <v>0.57724</v>
+        <v>0.44117</v>
       </c>
       <c r="Z11" s="1" t="n">
-        <v>0.08162999999999999</v>
+        <v>0.103</v>
       </c>
       <c r="AA11" s="1" t="n">
-        <v>0.89201</v>
+        <v>0.92244</v>
       </c>
       <c r="AB11" s="3" t="n">
-        <v>0.9736399999999999</v>
+        <v>1.02544</v>
       </c>
       <c r="AC11" s="1" t="n">
-        <v>0.56346</v>
+        <v>0.48618</v>
       </c>
       <c r="AD11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AE11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AF11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG11" t="n">
         <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="AI11" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="AJ11" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="AK11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AL11" t="n">
         <v>3</v>
       </c>
       <c r="AM11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AN11" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="AO11" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="AP11" t="n">
         <v>6</v>
@@ -2335,31 +2335,31 @@
         <v>0</v>
       </c>
       <c r="AS11" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="AT11" t="n">
         <v>30</v>
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Toronto Maple Leafs</t>
+          <t>Florida Panthers</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2373,13 +2373,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F12" t="n">
         <v>7</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
@@ -2388,136 +2388,136 @@
         <v>16</v>
       </c>
       <c r="J12" s="1" t="n">
-        <v>0.571429</v>
+        <v>0.615385</v>
       </c>
       <c r="K12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L12" t="n">
         <v>7</v>
       </c>
       <c r="M12" t="n">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="N12" t="n">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="O12" t="n">
+        <v>2</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>2.8462</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>28.23076</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>24.15384</v>
+      </c>
+      <c r="T12" s="1" t="n">
+        <v>0.229508</v>
+      </c>
+      <c r="U12" s="1" t="n">
+        <v>0.854546</v>
+      </c>
+      <c r="V12" s="1" t="n">
+        <v>0.469816</v>
+      </c>
+      <c r="W12" s="1" t="n">
+        <v>0.5488</v>
+      </c>
+      <c r="X12" s="1" t="n">
+        <v>0.53645</v>
+      </c>
+      <c r="Y12" s="1" t="n">
+        <v>0.57724</v>
+      </c>
+      <c r="Z12" s="1" t="n">
+        <v>0.08162999999999999</v>
+      </c>
+      <c r="AA12" s="1" t="n">
+        <v>0.89201</v>
+      </c>
+      <c r="AB12" s="3" t="n">
+        <v>0.9736399999999999</v>
+      </c>
+      <c r="AC12" s="1" t="n">
+        <v>0.56346</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>12</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>27</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>28</v>
+      </c>
+      <c r="AP12" t="n">
         <v>6</v>
       </c>
-      <c r="P12" s="2" t="n">
-        <v>3.7143</v>
-      </c>
-      <c r="Q12" s="2" t="n">
-        <v>3.2857</v>
-      </c>
-      <c r="R12" s="2" t="n">
-        <v>28.57142</v>
-      </c>
-      <c r="S12" s="2" t="n">
-        <v>30.28571</v>
-      </c>
-      <c r="T12" s="1" t="n">
-        <v>0.288888</v>
-      </c>
-      <c r="U12" s="1" t="n">
-        <v>0.936171</v>
-      </c>
-      <c r="V12" s="1" t="n">
-        <v>0.523096</v>
-      </c>
-      <c r="W12" s="1" t="n">
-        <v>0.46448</v>
-      </c>
-      <c r="X12" s="1" t="n">
-        <v>0.47634</v>
-      </c>
-      <c r="Y12" s="1" t="n">
-        <v>0.49322</v>
-      </c>
-      <c r="Z12" s="1" t="n">
-        <v>0.11111</v>
-      </c>
-      <c r="AA12" s="1" t="n">
-        <v>0.89341</v>
-      </c>
-      <c r="AB12" s="3" t="n">
-        <v>1.00452</v>
-      </c>
-      <c r="AC12" s="1" t="n">
-        <v>0.49175</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>8</v>
-      </c>
-      <c r="AE12" t="n">
-        <v>4</v>
-      </c>
-      <c r="AF12" t="n">
-        <v>3</v>
-      </c>
-      <c r="AG12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH12" t="n">
-        <v>24</v>
-      </c>
-      <c r="AI12" t="n">
-        <v>25</v>
-      </c>
-      <c r="AJ12" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK12" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL12" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>28</v>
-      </c>
-      <c r="AO12" t="n">
-        <v>21</v>
-      </c>
-      <c r="AP12" t="n">
-        <v>5</v>
-      </c>
       <c r="AQ12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS12" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="AT12" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tampa Bay Lightning</t>
+          <t>Toronto Maple Leafs</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TBL</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2531,22 +2531,22 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F13" t="n">
         <v>7</v>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J13" s="1" t="n">
-        <v>0.681818</v>
+        <v>0.5333329999999999</v>
       </c>
       <c r="K13" t="n">
         <v>6</v>
@@ -2555,79 +2555,79 @@
         <v>7</v>
       </c>
       <c r="M13" t="n">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="N13" t="n">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="O13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P13" s="2" t="n">
-        <v>3.4545</v>
+        <v>3.7333</v>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>3.0909</v>
+        <v>3.4</v>
       </c>
       <c r="R13" s="2" t="n">
-        <v>30.36363</v>
+        <v>28.06666</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>24.54545</v>
+        <v>29.4</v>
       </c>
       <c r="T13" s="1" t="n">
-        <v>0.15</v>
+        <v>0.3125</v>
       </c>
       <c r="U13" s="1" t="n">
-        <v>0.766667</v>
+        <v>0.923077</v>
       </c>
       <c r="V13" s="1" t="n">
-        <v>0.484992</v>
+        <v>0.523255</v>
       </c>
       <c r="W13" s="1" t="n">
-        <v>0.5527300000000001</v>
+        <v>0.47067</v>
       </c>
       <c r="X13" s="1" t="n">
-        <v>0.55445</v>
+        <v>0.48163</v>
       </c>
       <c r="Y13" s="1" t="n">
-        <v>0.55047</v>
+        <v>0.4968</v>
       </c>
       <c r="Z13" s="1" t="n">
-        <v>0.10852</v>
+        <v>0.10645</v>
       </c>
       <c r="AA13" s="1" t="n">
-        <v>0.89162</v>
+        <v>0.88554</v>
       </c>
       <c r="AB13" s="3" t="n">
-        <v>1.00014</v>
+        <v>0.99199</v>
       </c>
       <c r="AC13" s="1" t="n">
-        <v>0.5817600000000001</v>
+        <v>0.5</v>
       </c>
       <c r="AD13" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AE13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH13" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="AI13" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="AJ13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AK13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL13" t="n">
         <v>3</v>
@@ -2636,66 +2636,66 @@
         <v>1</v>
       </c>
       <c r="AN13" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="AO13" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AP13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AQ13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AR13" t="n">
         <v>1</v>
       </c>
       <c r="AS13" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="AT13" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Seattle Kraken</t>
+          <t>Tampa Bay Lightning</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>TBL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
         <v>7</v>
       </c>
       <c r="G14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H14" t="n">
         <v>1</v>
@@ -2704,73 +2704,73 @@
         <v>15</v>
       </c>
       <c r="J14" s="1" t="n">
-        <v>0.625</v>
+        <v>0.681818</v>
       </c>
       <c r="K14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L14" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M14" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N14" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="O14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P14" s="2" t="n">
-        <v>3.75</v>
+        <v>3.4545</v>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>3.5</v>
+        <v>3.0909</v>
       </c>
       <c r="R14" s="2" t="n">
-        <v>26.16666</v>
+        <v>30.36363</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>31.83333</v>
+        <v>24.54545</v>
       </c>
       <c r="T14" s="1" t="n">
-        <v>0.230769</v>
+        <v>0.15</v>
       </c>
       <c r="U14" s="1" t="n">
-        <v>0.705883</v>
+        <v>0.766667</v>
       </c>
       <c r="V14" s="1" t="n">
-        <v>0.516172</v>
+        <v>0.484992</v>
       </c>
       <c r="W14" s="1" t="n">
-        <v>0.43106</v>
+        <v>0.5527300000000001</v>
       </c>
       <c r="X14" s="1" t="n">
-        <v>0.4308</v>
+        <v>0.55445</v>
       </c>
       <c r="Y14" s="1" t="n">
-        <v>0.48824</v>
+        <v>0.55047</v>
       </c>
       <c r="Z14" s="1" t="n">
-        <v>0.13306</v>
+        <v>0.10852</v>
       </c>
       <c r="AA14" s="1" t="n">
-        <v>0.9103</v>
+        <v>0.89162</v>
       </c>
       <c r="AB14" s="3" t="n">
-        <v>1.04336</v>
+        <v>1.00014</v>
       </c>
       <c r="AC14" s="1" t="n">
-        <v>0.43576</v>
+        <v>0.5817600000000001</v>
       </c>
       <c r="AD14" t="n">
         <v>5</v>
       </c>
       <c r="AE14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AF14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AG14" t="n">
         <v>0</v>
@@ -2779,49 +2779,49 @@
         <v>18</v>
       </c>
       <c r="AI14" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="AJ14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>20</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>25</v>
+      </c>
+      <c r="AP14" t="n">
         <v>7</v>
       </c>
-      <c r="AK14" t="n">
-        <v>4</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>27</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>24</v>
-      </c>
-      <c r="AP14" t="n">
-        <v>6</v>
-      </c>
       <c r="AQ14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AR14" t="n">
         <v>1</v>
       </c>
       <c r="AS14" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="AT14" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>OT1</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -2901,13 +2901,13 @@
         <v>0.560862</v>
       </c>
       <c r="W15" s="1" t="n">
-        <v>0.52225</v>
+        <v>0.5212599999999999</v>
       </c>
       <c r="X15" s="1" t="n">
         <v>0.5351900000000001</v>
       </c>
       <c r="Y15" s="1" t="n">
-        <v>0.52481</v>
+        <v>0.5233</v>
       </c>
       <c r="Z15" s="1" t="n">
         <v>0.08898</v>
@@ -2979,39 +2979,39 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>New York Rangers</t>
+          <t>Colorado Avalanche</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NYR</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F16" t="n">
         <v>7</v>
       </c>
       <c r="G16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H16" t="n">
         <v>1</v>
@@ -3020,7 +3020,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="1" t="n">
-        <v>0.535714</v>
+        <v>0.576923</v>
       </c>
       <c r="K16" t="n">
         <v>7</v>
@@ -3029,127 +3029,127 @@
         <v>7</v>
       </c>
       <c r="M16" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="N16" t="n">
         <v>42</v>
       </c>
       <c r="O16" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="P16" s="2" t="n">
-        <v>3.1429</v>
+        <v>4.1538</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>3</v>
+        <v>3.2308</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>24.71428</v>
+        <v>30.38461</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>26.28571</v>
+        <v>28</v>
       </c>
       <c r="T16" s="1" t="n">
-        <v>0.210526</v>
+        <v>0.195121</v>
       </c>
       <c r="U16" s="1" t="n">
-        <v>0.904762</v>
+        <v>0.769231</v>
       </c>
       <c r="V16" s="1" t="n">
-        <v>0.538274</v>
+        <v>0.469182</v>
       </c>
       <c r="W16" s="1" t="n">
-        <v>0.48097</v>
+        <v>0.52496</v>
       </c>
       <c r="X16" s="1" t="n">
-        <v>0.47228</v>
+        <v>0.5245300000000001</v>
       </c>
       <c r="Y16" s="1" t="n">
-        <v>0.47249</v>
+        <v>0.5428500000000001</v>
       </c>
       <c r="Z16" s="1" t="n">
-        <v>0.1</v>
+        <v>0.13826</v>
       </c>
       <c r="AA16" s="1" t="n">
-        <v>0.8986</v>
+        <v>0.91409</v>
       </c>
       <c r="AB16" s="3" t="n">
-        <v>0.9986</v>
+        <v>1.05235</v>
       </c>
       <c r="AC16" s="1" t="n">
-        <v>0.48039</v>
+        <v>0.51732</v>
       </c>
       <c r="AD16" t="n">
         <v>7</v>
       </c>
       <c r="AE16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>35</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>21</v>
+      </c>
+      <c r="AJ16" t="n">
         <v>6</v>
       </c>
-      <c r="AF16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG16" t="n">
+      <c r="AK16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM16" t="n">
         <v>0</v>
       </c>
-      <c r="AH16" t="n">
-        <v>32</v>
-      </c>
-      <c r="AI16" t="n">
-        <v>16</v>
-      </c>
-      <c r="AJ16" t="n">
-        <v>7</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL16" t="n">
-        <v>5</v>
-      </c>
-      <c r="AM16" t="n">
-        <v>1</v>
-      </c>
       <c r="AN16" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="AO16" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="AP16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AQ16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AR16" t="n">
         <v>1</v>
       </c>
       <c r="AS16" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="AT16" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>New York Islanders</t>
+          <t>New York Rangers</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NYI</t>
+          <t>NYR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3163,490 +3163,490 @@
         </is>
       </c>
       <c r="E17" t="n">
+        <v>14</v>
+      </c>
+      <c r="F17" t="n">
+        <v>7</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>15</v>
+      </c>
+      <c r="J17" s="1" t="n">
+        <v>0.535714</v>
+      </c>
+      <c r="K17" t="n">
+        <v>7</v>
+      </c>
+      <c r="L17" t="n">
+        <v>7</v>
+      </c>
+      <c r="M17" t="n">
+        <v>44</v>
+      </c>
+      <c r="N17" t="n">
+        <v>42</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>3.1429</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>24.71428</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>26.28571</v>
+      </c>
+      <c r="T17" s="1" t="n">
+        <v>0.210526</v>
+      </c>
+      <c r="U17" s="1" t="n">
+        <v>0.904762</v>
+      </c>
+      <c r="V17" s="1" t="n">
+        <v>0.538274</v>
+      </c>
+      <c r="W17" s="1" t="n">
+        <v>0.48097</v>
+      </c>
+      <c r="X17" s="1" t="n">
+        <v>0.47228</v>
+      </c>
+      <c r="Y17" s="1" t="n">
+        <v>0.47249</v>
+      </c>
+      <c r="Z17" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AA17" s="1" t="n">
+        <v>0.8986</v>
+      </c>
+      <c r="AB17" s="3" t="n">
+        <v>0.9986</v>
+      </c>
+      <c r="AC17" s="1" t="n">
+        <v>0.48039</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>32</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>16</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN17" t="n">
         <v>12</v>
       </c>
-      <c r="F17" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" t="n">
-        <v>4</v>
-      </c>
-      <c r="H17" t="n">
-        <v>2</v>
-      </c>
-      <c r="I17" t="n">
-        <v>14</v>
-      </c>
-      <c r="J17" s="1" t="n">
-        <v>0.583333</v>
-      </c>
-      <c r="K17" t="n">
-        <v>5</v>
-      </c>
-      <c r="L17" t="n">
-        <v>5</v>
-      </c>
-      <c r="M17" t="n">
+      <c r="AO17" t="n">
+        <v>26</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>33</v>
+      </c>
+      <c r="AT17" t="n">
         <v>36</v>
       </c>
-      <c r="N17" t="n">
-        <v>32</v>
-      </c>
-      <c r="O17" t="n">
-        <v>4</v>
-      </c>
-      <c r="P17" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q17" s="2" t="n">
-        <v>2.6667</v>
-      </c>
-      <c r="R17" s="2" t="n">
-        <v>26.16666</v>
-      </c>
-      <c r="S17" s="2" t="n">
-        <v>26.33333</v>
-      </c>
-      <c r="T17" s="1" t="n">
-        <v>0.157894</v>
-      </c>
-      <c r="U17" s="1" t="n">
-        <v>0.8536589999999999</v>
-      </c>
-      <c r="V17" s="1" t="n">
-        <v>0.549755</v>
-      </c>
-      <c r="W17" s="1" t="n">
-        <v>0.51631</v>
-      </c>
-      <c r="X17" s="1" t="n">
-        <v>0.50874</v>
-      </c>
-      <c r="Y17" s="1" t="n">
-        <v>0.53565</v>
-      </c>
-      <c r="Z17" s="1" t="n">
-        <v>0.09349</v>
-      </c>
-      <c r="AA17" s="1" t="n">
-        <v>0.92405</v>
-      </c>
-      <c r="AB17" s="3" t="n">
-        <v>1.01754</v>
-      </c>
-      <c r="AC17" s="1" t="n">
-        <v>0.52669</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>4</v>
-      </c>
-      <c r="AF17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH17" t="n">
-        <v>21</v>
-      </c>
-      <c r="AI17" t="n">
-        <v>13</v>
-      </c>
-      <c r="AJ17" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN17" t="n">
-        <v>15</v>
-      </c>
-      <c r="AO17" t="n">
-        <v>19</v>
-      </c>
-      <c r="AP17" t="n">
-        <v>5</v>
-      </c>
-      <c r="AQ17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AR17" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS17" t="n">
-        <v>29</v>
-      </c>
-      <c r="AT17" t="n">
-        <v>30</v>
-      </c>
       <c r="AU17" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Colorado Avalanche</t>
+          <t>Washington Capitals</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J18" s="1" t="n">
-        <v>0.541667</v>
+        <v>0.636364</v>
       </c>
       <c r="K18" t="n">
         <v>6</v>
       </c>
       <c r="L18" t="n">
+        <v>7</v>
+      </c>
+      <c r="M18" t="n">
+        <v>39</v>
+      </c>
+      <c r="N18" t="n">
+        <v>34</v>
+      </c>
+      <c r="O18" t="n">
+        <v>5</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>3.5455</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>3.0909</v>
+      </c>
+      <c r="R18" s="2" t="n">
+        <v>27.72727</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>28.0909</v>
+      </c>
+      <c r="T18" s="1" t="n">
+        <v>0.193548</v>
+      </c>
+      <c r="U18" s="1" t="n">
+        <v>0.805556</v>
+      </c>
+      <c r="V18" s="1" t="n">
+        <v>0.495129</v>
+      </c>
+      <c r="W18" s="1" t="n">
+        <v>0.47464</v>
+      </c>
+      <c r="X18" s="1" t="n">
+        <v>0.49159</v>
+      </c>
+      <c r="Y18" s="1" t="n">
+        <v>0.48254</v>
+      </c>
+      <c r="Z18" s="1" t="n">
+        <v>0.12663</v>
+      </c>
+      <c r="AA18" s="1" t="n">
+        <v>0.8974299999999999</v>
+      </c>
+      <c r="AB18" s="3" t="n">
+        <v>1.02406</v>
+      </c>
+      <c r="AC18" s="1" t="n">
+        <v>0.44444</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE18" t="n">
         <v>6</v>
       </c>
-      <c r="M18" t="n">
-        <v>49</v>
-      </c>
-      <c r="N18" t="n">
-        <v>40</v>
-      </c>
-      <c r="O18" t="n">
-        <v>9</v>
-      </c>
-      <c r="P18" s="2" t="n">
-        <v>4.0833</v>
-      </c>
-      <c r="Q18" s="2" t="n">
-        <v>3.3333</v>
-      </c>
-      <c r="R18" s="2" t="n">
-        <v>29.25</v>
-      </c>
-      <c r="S18" s="2" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="T18" s="1" t="n">
-        <v>0.179487</v>
-      </c>
-      <c r="U18" s="1" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="V18" s="1" t="n">
-        <v>0.462912</v>
-      </c>
-      <c r="W18" s="1" t="n">
-        <v>0.5144300000000001</v>
-      </c>
-      <c r="X18" s="1" t="n">
-        <v>0.50954</v>
-      </c>
-      <c r="Y18" s="1" t="n">
-        <v>0.52615</v>
-      </c>
-      <c r="Z18" s="1" t="n">
-        <v>0.14233</v>
-      </c>
-      <c r="AA18" s="1" t="n">
-        <v>0.91208</v>
-      </c>
-      <c r="AB18" s="3" t="n">
-        <v>1.05441</v>
-      </c>
-      <c r="AC18" s="1" t="n">
-        <v>0.50552</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE18" t="n">
-        <v>4</v>
-      </c>
       <c r="AF18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH18" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AI18" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="AJ18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AK18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AL18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AM18" t="n">
         <v>0</v>
       </c>
       <c r="AN18" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="AO18" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="AP18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AQ18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AR18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS18" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AT18" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nashville Predators</t>
+          <t>New York Islanders</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NSH</t>
+          <t>NYI</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E19" t="n">
         <v>12</v>
       </c>
       <c r="F19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J19" s="1" t="n">
-        <v>0.541667</v>
+        <v>0.583333</v>
       </c>
       <c r="K19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M19" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N19" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="O19" t="n">
-        <v>-5</v>
+        <v>4</v>
       </c>
       <c r="P19" s="2" t="n">
-        <v>2.8333</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>3.25</v>
+        <v>2.6667</v>
       </c>
       <c r="R19" s="2" t="n">
-        <v>25.58333</v>
+        <v>26.08333</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>29.16666</v>
+        <v>26.33333</v>
       </c>
       <c r="T19" s="1" t="n">
-        <v>0.317073</v>
+        <v>0.157894</v>
       </c>
       <c r="U19" s="1" t="n">
-        <v>0.875</v>
+        <v>0.8536589999999999</v>
       </c>
       <c r="V19" s="1" t="n">
-        <v>0.499276</v>
+        <v>0.549755</v>
       </c>
       <c r="W19" s="1" t="n">
-        <v>0.44995</v>
+        <v>0.51631</v>
       </c>
       <c r="X19" s="1" t="n">
-        <v>0.45796</v>
+        <v>0.50874</v>
       </c>
       <c r="Y19" s="1" t="n">
-        <v>0.43344</v>
+        <v>0.53565</v>
       </c>
       <c r="Z19" s="1" t="n">
-        <v>0.07239</v>
+        <v>0.09349</v>
       </c>
       <c r="AA19" s="1" t="n">
-        <v>0.91304</v>
+        <v>0.92405</v>
       </c>
       <c r="AB19" s="3" t="n">
-        <v>0.98543</v>
+        <v>1.01754</v>
       </c>
       <c r="AC19" s="1" t="n">
-        <v>0.44807</v>
+        <v>0.52669</v>
       </c>
       <c r="AD19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AE19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH19" t="n">
         <v>21</v>
       </c>
       <c r="AI19" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="AJ19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AM19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AN19" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AO19" t="n">
         <v>19</v>
       </c>
       <c r="AP19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AQ19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AS19" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="AT19" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="AU19" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Buffalo Sabres</t>
+          <t>Nashville Predators</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>NSH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E20" t="n">
         <v>12</v>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I20" t="n">
         <v>13</v>
@@ -3655,133 +3655,133 @@
         <v>0.541667</v>
       </c>
       <c r="K20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M20" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N20" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="O20" t="n">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="P20" s="2" t="n">
-        <v>2.75</v>
+        <v>2.8333</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>3.4167</v>
+        <v>3.25</v>
       </c>
       <c r="R20" s="2" t="n">
-        <v>27.5</v>
+        <v>25.58333</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>26.25</v>
+        <v>29.08333</v>
       </c>
       <c r="T20" s="1" t="n">
-        <v>0.09755999999999999</v>
+        <v>0.317073</v>
       </c>
       <c r="U20" s="1" t="n">
-        <v>0.714286</v>
+        <v>0.875</v>
       </c>
       <c r="V20" s="1" t="n">
-        <v>0.475574</v>
+        <v>0.499276</v>
       </c>
       <c r="W20" s="1" t="n">
-        <v>0.52358</v>
+        <v>0.44995</v>
       </c>
       <c r="X20" s="1" t="n">
-        <v>0.51851</v>
+        <v>0.45796</v>
       </c>
       <c r="Y20" s="1" t="n">
-        <v>0.49862</v>
+        <v>0.43344</v>
       </c>
       <c r="Z20" s="1" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.07239</v>
       </c>
       <c r="AA20" s="1" t="n">
-        <v>0.88687</v>
+        <v>0.91304</v>
       </c>
       <c r="AB20" s="3" t="n">
-        <v>0.97777</v>
+        <v>0.98543</v>
       </c>
       <c r="AC20" s="1" t="n">
-        <v>0.52161</v>
+        <v>0.44807</v>
       </c>
       <c r="AD20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AE20" t="n">
         <v>3</v>
       </c>
       <c r="AF20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AH20" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="AI20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>13</v>
+      </c>
+      <c r="AO20" t="n">
         <v>19</v>
       </c>
-      <c r="AJ20" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>19</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>22</v>
-      </c>
       <c r="AP20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AQ20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AR20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AS20" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="AT20" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="AU20" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>OT1</t>
         </is>
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Detroit Red Wings</t>
+          <t>Buffalo Sabres</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3816,61 +3816,61 @@
         <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M21" t="n">
         <v>33</v>
       </c>
       <c r="N21" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="O21" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="P21" s="2" t="n">
         <v>2.75</v>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>3.0833</v>
+        <v>3.4167</v>
       </c>
       <c r="R21" s="2" t="n">
-        <v>29.75</v>
+        <v>27.58333</v>
       </c>
       <c r="S21" s="2" t="n">
-        <v>25.66666</v>
+        <v>26.25</v>
       </c>
       <c r="T21" s="1" t="n">
-        <v>0.214285</v>
+        <v>0.09755999999999999</v>
       </c>
       <c r="U21" s="1" t="n">
-        <v>0.658537</v>
+        <v>0.714286</v>
       </c>
       <c r="V21" s="1" t="n">
-        <v>0.505681</v>
+        <v>0.475574</v>
       </c>
       <c r="W21" s="1" t="n">
-        <v>0.5340200000000001</v>
+        <v>0.52358</v>
       </c>
       <c r="X21" s="1" t="n">
-        <v>0.54777</v>
+        <v>0.51851</v>
       </c>
       <c r="Y21" s="1" t="n">
-        <v>0.50995</v>
+        <v>0.49862</v>
       </c>
       <c r="Z21" s="1" t="n">
-        <v>0.07462000000000001</v>
+        <v>0.09055000000000001</v>
       </c>
       <c r="AA21" s="1" t="n">
-        <v>0.91555</v>
+        <v>0.88687</v>
       </c>
       <c r="AB21" s="3" t="n">
-        <v>0.99017</v>
+        <v>0.97742</v>
       </c>
       <c r="AC21" s="1" t="n">
-        <v>0.50887</v>
+        <v>0.52161</v>
       </c>
       <c r="AD21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AE21" t="n">
         <v>3</v>
@@ -3879,16 +3879,16 @@
         <v>3</v>
       </c>
       <c r="AG21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH21" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="AI21" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="AJ21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AK21" t="n">
         <v>2</v>
@@ -3897,25 +3897,25 @@
         <v>1</v>
       </c>
       <c r="AM21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AN21" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="AO21" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="AP21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AQ21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR21" t="n">
         <v>3</v>
       </c>
       <c r="AS21" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="AT21" t="n">
         <v>32</v>
@@ -3927,323 +3927,323 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>San Jose Sharks</t>
+          <t>Detroit Red Wings</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SJS</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G22" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
         <v>13</v>
       </c>
       <c r="J22" s="1" t="n">
-        <v>0.5</v>
+        <v>0.541667</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M22" t="n">
+        <v>33</v>
+      </c>
+      <c r="N22" t="n">
         <v>37</v>
       </c>
-      <c r="N22" t="n">
-        <v>45</v>
-      </c>
       <c r="O22" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="P22" s="2" t="n">
-        <v>2.8462</v>
+        <v>2.75</v>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>3.4615</v>
+        <v>3.0833</v>
       </c>
       <c r="R22" s="2" t="n">
-        <v>27.6923</v>
+        <v>29.75</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>31.07692</v>
+        <v>25.66666</v>
       </c>
       <c r="T22" s="1" t="n">
-        <v>0.25</v>
+        <v>0.214285</v>
       </c>
       <c r="U22" s="1" t="n">
-        <v>0.818182</v>
+        <v>0.658537</v>
       </c>
       <c r="V22" s="1" t="n">
-        <v>0.470215</v>
+        <v>0.505681</v>
       </c>
       <c r="W22" s="1" t="n">
-        <v>0.45212</v>
+        <v>0.5340200000000001</v>
       </c>
       <c r="X22" s="1" t="n">
-        <v>0.44983</v>
+        <v>0.54777</v>
       </c>
       <c r="Y22" s="1" t="n">
-        <v>0.47024</v>
+        <v>0.50995</v>
       </c>
       <c r="Z22" s="1" t="n">
-        <v>0.05947</v>
+        <v>0.07462000000000001</v>
       </c>
       <c r="AA22" s="1" t="n">
-        <v>0.90666</v>
+        <v>0.91555</v>
       </c>
       <c r="AB22" s="3" t="n">
-        <v>0.96613</v>
+        <v>0.99017</v>
       </c>
       <c r="AC22" s="1" t="n">
-        <v>0.455</v>
+        <v>0.50887</v>
       </c>
       <c r="AD22" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AE22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF22" t="n">
         <v>3</v>
       </c>
       <c r="AG22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH22" t="n">
+        <v>20</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>23</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN22" t="n">
         <v>13</v>
       </c>
-      <c r="AI22" t="n">
-        <v>18</v>
-      </c>
-      <c r="AJ22" t="n">
-        <v>8</v>
-      </c>
-      <c r="AK22" t="n">
-        <v>4</v>
-      </c>
-      <c r="AL22" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN22" t="n">
-        <v>24</v>
-      </c>
       <c r="AO22" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="AP22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AQ22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AR22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS22" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="AT22" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AU22" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Washington Capitals</t>
+          <t>San Jose Sharks</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F23" t="n">
         <v>6</v>
       </c>
       <c r="G23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J23" s="1" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K23" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M23" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="N23" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="O23" t="n">
-        <v>2</v>
+        <v>-8</v>
       </c>
       <c r="P23" s="2" t="n">
-        <v>3.4</v>
+        <v>2.8462</v>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>3.2</v>
+        <v>3.4615</v>
       </c>
       <c r="R23" s="2" t="n">
-        <v>27.5</v>
+        <v>27.6923</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>28.4</v>
+        <v>31.15384</v>
       </c>
       <c r="T23" s="1" t="n">
-        <v>0.178571</v>
+        <v>0.25</v>
       </c>
       <c r="U23" s="1" t="n">
-        <v>0.8125</v>
+        <v>0.818182</v>
       </c>
       <c r="V23" s="1" t="n">
-        <v>0.501773</v>
+        <v>0.470215</v>
       </c>
       <c r="W23" s="1" t="n">
-        <v>0.46959</v>
+        <v>0.45212</v>
       </c>
       <c r="X23" s="1" t="n">
-        <v>0.48387</v>
+        <v>0.44983</v>
       </c>
       <c r="Y23" s="1" t="n">
-        <v>0.47993</v>
+        <v>0.47024</v>
       </c>
       <c r="Z23" s="1" t="n">
-        <v>0.12745</v>
+        <v>0.05947</v>
       </c>
       <c r="AA23" s="1" t="n">
-        <v>0.89201</v>
+        <v>0.9069700000000001</v>
       </c>
       <c r="AB23" s="3" t="n">
-        <v>1.01946</v>
+        <v>0.96644</v>
       </c>
       <c r="AC23" s="1" t="n">
-        <v>0.42804</v>
+        <v>0.455</v>
       </c>
       <c r="AD23" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AE23" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AF23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG23" t="n">
         <v>0</v>
       </c>
       <c r="AH23" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="AI23" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="AJ23" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="AK23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AL23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN23" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="AO23" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="AP23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AQ23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS23" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="AT23" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="AU23" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
         <v>28.08333</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>27.75</v>
+        <v>27.83333</v>
       </c>
       <c r="T24" s="1" t="n">
         <v>0.21875</v>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -4639,7 +4639,7 @@
         <v>0.452135</v>
       </c>
       <c r="W26" s="1" t="n">
-        <v>0.48594</v>
+        <v>0.48641</v>
       </c>
       <c r="X26" s="1" t="n">
         <v>0.483</v>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4943,7 @@
         <v>25.6</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>28</v>
+        <v>28.1</v>
       </c>
       <c r="T28" s="1" t="n">
         <v>0.111111</v>
@@ -4967,10 +4967,10 @@
         <v>0.08994000000000001</v>
       </c>
       <c r="AA28" s="1" t="n">
-        <v>0.91705</v>
+        <v>0.91743</v>
       </c>
       <c r="AB28" s="3" t="n">
-        <v>1.00699</v>
+        <v>1.00737</v>
       </c>
       <c r="AC28" s="1" t="n">
         <v>0.48299</v>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -5059,13 +5059,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F29" t="n">
         <v>5</v>
       </c>
       <c r="G29" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -5074,7 +5074,7 @@
         <v>10</v>
       </c>
       <c r="J29" s="1" t="n">
-        <v>0.454545</v>
+        <v>0.416667</v>
       </c>
       <c r="K29" t="n">
         <v>5</v>
@@ -5086,52 +5086,52 @@
         <v>28</v>
       </c>
       <c r="N29" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="O29" t="n">
-        <v>-13</v>
+        <v>-17</v>
       </c>
       <c r="P29" s="2" t="n">
-        <v>2.5455</v>
+        <v>2.3333</v>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>3.7273</v>
+        <v>3.75</v>
       </c>
       <c r="R29" s="2" t="n">
-        <v>29.18181</v>
+        <v>28.75</v>
       </c>
       <c r="S29" s="2" t="n">
-        <v>30.36363</v>
+        <v>30.5</v>
       </c>
       <c r="T29" s="1" t="n">
-        <v>0.3</v>
+        <v>0.290322</v>
       </c>
       <c r="U29" s="1" t="n">
-        <v>0.857143</v>
+        <v>0.837838</v>
       </c>
       <c r="V29" s="1" t="n">
-        <v>0.486983</v>
+        <v>0.491501</v>
       </c>
       <c r="W29" s="1" t="n">
-        <v>0.51671</v>
+        <v>0.5165</v>
       </c>
       <c r="X29" s="1" t="n">
-        <v>0.5019</v>
+        <v>0.50114</v>
       </c>
       <c r="Y29" s="1" t="n">
-        <v>0.50522</v>
+        <v>0.5049</v>
       </c>
       <c r="Z29" s="1" t="n">
-        <v>0.05791</v>
+        <v>0.053</v>
       </c>
       <c r="AA29" s="1" t="n">
-        <v>0.8807700000000001</v>
+        <v>0.8807</v>
       </c>
       <c r="AB29" s="3" t="n">
-        <v>0.93868</v>
+        <v>0.9337</v>
       </c>
       <c r="AC29" s="1" t="n">
-        <v>0.50445</v>
+        <v>0.49597</v>
       </c>
       <c r="AD29" t="n">
         <v>7</v>
@@ -5152,13 +5152,13 @@
         <v>23</v>
       </c>
       <c r="AJ29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AK29" t="n">
         <v>1</v>
       </c>
       <c r="AL29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AM29" t="n">
         <v>0</v>
@@ -5167,7 +5167,7 @@
         <v>8</v>
       </c>
       <c r="AO29" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="AP29" t="n">
         <v>5</v>
@@ -5179,19 +5179,19 @@
         <v>0</v>
       </c>
       <c r="AS29" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AT29" t="n">
         <v>35</v>
       </c>
       <c r="AU29" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -5217,13 +5217,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F30" t="n">
         <v>3</v>
       </c>
       <c r="G30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H30" t="n">
         <v>4</v>
@@ -5232,7 +5232,7 @@
         <v>10</v>
       </c>
       <c r="J30" s="1" t="n">
-        <v>0.357143</v>
+        <v>0.333333</v>
       </c>
       <c r="K30" t="n">
         <v>3</v>
@@ -5241,55 +5241,55 @@
         <v>3</v>
       </c>
       <c r="M30" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="N30" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O30" t="n">
-        <v>-19</v>
+        <v>-22</v>
       </c>
       <c r="P30" s="2" t="n">
-        <v>1.9286</v>
+        <v>1.9333</v>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>3.2857</v>
+        <v>3.4</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>23.28571</v>
+        <v>23.46666</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>30.28571</v>
+        <v>30.26666</v>
       </c>
       <c r="T30" s="1" t="n">
-        <v>0.155555</v>
+        <v>0.163265</v>
       </c>
       <c r="U30" s="1" t="n">
-        <v>0.829788</v>
+        <v>0.82</v>
       </c>
       <c r="V30" s="1" t="n">
-        <v>0.503059</v>
+        <v>0.507479</v>
       </c>
       <c r="W30" s="1" t="n">
-        <v>0.43583</v>
+        <v>0.43913</v>
       </c>
       <c r="X30" s="1" t="n">
-        <v>0.42214</v>
+        <v>0.42259</v>
       </c>
       <c r="Y30" s="1" t="n">
-        <v>0.41538</v>
+        <v>0.42092</v>
       </c>
       <c r="Z30" s="1" t="n">
-        <v>0.06302000000000001</v>
+        <v>0.06153</v>
       </c>
       <c r="AA30" s="1" t="n">
-        <v>0.9003100000000001</v>
+        <v>0.89884</v>
       </c>
       <c r="AB30" s="3" t="n">
-        <v>0.96333</v>
+        <v>0.9603699999999999</v>
       </c>
       <c r="AC30" s="1" t="n">
-        <v>0.42716</v>
+        <v>0.42459</v>
       </c>
       <c r="AD30" t="n">
         <v>8</v>
@@ -5310,22 +5310,22 @@
         <v>29</v>
       </c>
       <c r="AJ30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AK30" t="n">
         <v>1</v>
       </c>
       <c r="AL30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AM30" t="n">
         <v>1</v>
       </c>
       <c r="AN30" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AO30" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="AP30" t="n">
         <v>3</v>
@@ -5337,19 +5337,19 @@
         <v>2</v>
       </c>
       <c r="AS30" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="AT30" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="AU30" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -5429,13 +5429,13 @@
         <v>0.506451</v>
       </c>
       <c r="W31" s="1" t="n">
-        <v>0.47778</v>
+        <v>0.47727</v>
       </c>
       <c r="X31" s="1" t="n">
-        <v>0.48214</v>
+        <v>0.48143</v>
       </c>
       <c r="Y31" s="1" t="n">
-        <v>0.44677</v>
+        <v>0.44594</v>
       </c>
       <c r="Z31" s="1" t="n">
         <v>0.07207</v>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -5587,13 +5587,13 @@
         <v>0.426512</v>
       </c>
       <c r="W32" s="1" t="n">
-        <v>0.43878</v>
+        <v>0.43921</v>
       </c>
       <c r="X32" s="1" t="n">
-        <v>0.42327</v>
+        <v>0.42381</v>
       </c>
       <c r="Y32" s="1" t="n">
-        <v>0.43377</v>
+        <v>0.43449</v>
       </c>
       <c r="Z32" s="1" t="n">
         <v>0.08373999999999999</v>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-28 08:21</t>
+          <t>2026-10-29 03:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-29 08:22 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-29 03:05</t>
+          <t>2026-10-29 08:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-30 08:22 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-30 03:05</t>
+          <t>2026-10-30 08:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-31 02:59 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
         <v>2.3333</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>30.86666</v>
+        <v>30.93333</v>
       </c>
       <c r="S3" s="2" t="n">
         <v>25.13333</v>
@@ -1005,13 +1005,13 @@
         <v>0.491972</v>
       </c>
       <c r="W3" s="1" t="n">
-        <v>0.53048</v>
+        <v>0.53012</v>
       </c>
       <c r="X3" s="1" t="n">
         <v>0.54659</v>
       </c>
       <c r="Y3" s="1" t="n">
-        <v>0.5178</v>
+        <v>0.51708</v>
       </c>
       <c r="Z3" s="1" t="n">
         <v>0.08645</v>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1306,7 @@
         <v>2.2857</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>25.92857</v>
+        <v>25.85714</v>
       </c>
       <c r="S5" s="2" t="n">
         <v>27.35714</v>
@@ -1330,13 +1330,13 @@
         <v>0.48733</v>
       </c>
       <c r="Z5" s="1" t="n">
-        <v>0.11333</v>
+        <v>0.11371</v>
       </c>
       <c r="AA5" s="1" t="n">
         <v>0.94333</v>
       </c>
       <c r="AB5" s="3" t="n">
-        <v>1.05666</v>
+        <v>1.05704</v>
       </c>
       <c r="AC5" s="1" t="n">
         <v>0.48883</v>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -1425,13 +1425,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" t="n">
         <v>9</v>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" t="n">
         <v>1</v>
@@ -1440,7 +1440,7 @@
         <v>19</v>
       </c>
       <c r="J6" s="1" t="n">
-        <v>0.678571</v>
+        <v>0.633333</v>
       </c>
       <c r="K6" t="n">
         <v>7</v>
@@ -1449,73 +1449,73 @@
         <v>8</v>
       </c>
       <c r="M6" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="N6" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="O6" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>3.6429</v>
+        <v>3.5333</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>2.7857</v>
+        <v>2.9333</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>29.71428</v>
+        <v>29.13333</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>25.14285</v>
+        <v>25.6</v>
       </c>
       <c r="T6" s="1" t="n">
-        <v>0.255813</v>
+        <v>0.272727</v>
       </c>
       <c r="U6" s="1" t="n">
-        <v>0.676471</v>
+        <v>0.694445</v>
       </c>
       <c r="V6" s="1" t="n">
-        <v>0.503768</v>
+        <v>0.505275</v>
       </c>
       <c r="W6" s="1" t="n">
-        <v>0.52384</v>
+        <v>0.51622</v>
       </c>
       <c r="X6" s="1" t="n">
-        <v>0.5400199999999999</v>
+        <v>0.53187</v>
       </c>
       <c r="Y6" s="1" t="n">
-        <v>0.5362</v>
+        <v>0.52691</v>
       </c>
       <c r="Z6" s="1" t="n">
-        <v>0.09393</v>
+        <v>0.09221</v>
       </c>
       <c r="AA6" s="1" t="n">
-        <v>0.90942</v>
+        <v>0.9039700000000001</v>
       </c>
       <c r="AB6" s="3" t="n">
-        <v>1.00335</v>
+        <v>0.99618</v>
       </c>
       <c r="AC6" s="1" t="n">
-        <v>0.51927</v>
+        <v>0.52127</v>
       </c>
       <c r="AD6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AE6" t="n">
         <v>6</v>
       </c>
       <c r="AF6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG6" t="n">
         <v>0</v>
       </c>
       <c r="AH6" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="AI6" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="AJ6" t="n">
         <v>6</v>
@@ -1536,28 +1536,28 @@
         <v>18</v>
       </c>
       <c r="AP6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AQ6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR6" t="n">
         <v>1</v>
       </c>
       <c r="AS6" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="AT6" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -1715,29 +1715,29 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Utah Mammoth</t>
+          <t>New Jersey Devils</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UTA</t>
+          <t>NJD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1765,61 +1765,61 @@
         <v>9</v>
       </c>
       <c r="M8" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="N8" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="O8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>3.6429</v>
+        <v>3.4286</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>3.2857</v>
+        <v>2.8571</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>30.42857</v>
+        <v>32.57142</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>24.78571</v>
       </c>
       <c r="T8" s="1" t="n">
-        <v>0.340425</v>
+        <v>0.166666</v>
       </c>
       <c r="U8" s="1" t="n">
-        <v>0.673914</v>
+        <v>0.7</v>
       </c>
       <c r="V8" s="1" t="n">
-        <v>0.549065</v>
+        <v>0.5012720000000001</v>
       </c>
       <c r="W8" s="1" t="n">
-        <v>0.55569</v>
+        <v>0.57634</v>
       </c>
       <c r="X8" s="1" t="n">
-        <v>0.56333</v>
+        <v>0.56856</v>
       </c>
       <c r="Y8" s="1" t="n">
-        <v>0.53823</v>
+        <v>0.57394</v>
       </c>
       <c r="Z8" s="1" t="n">
-        <v>0.08782</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="AA8" s="1" t="n">
-        <v>0.90262</v>
+        <v>0.90391</v>
       </c>
       <c r="AB8" s="3" t="n">
-        <v>0.99044</v>
+        <v>0.99481</v>
       </c>
       <c r="AC8" s="1" t="n">
-        <v>0.49885</v>
+        <v>0.52153</v>
       </c>
       <c r="AD8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AE8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AF8" t="n">
         <v>2</v>
@@ -1828,16 +1828,16 @@
         <v>0</v>
       </c>
       <c r="AH8" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="AI8" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="AJ8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AK8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AL8" t="n">
         <v>3</v>
@@ -1846,25 +1846,25 @@
         <v>0</v>
       </c>
       <c r="AN8" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="AO8" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="AP8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AQ8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR8" t="n">
         <v>0</v>
       </c>
       <c r="AS8" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="AT8" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="AU8" t="inlineStr">
         <is>
@@ -1873,114 +1873,114 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tampa Bay Lightning</t>
+          <t>Utah Mammoth</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TBL</t>
+          <t>UTA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J9" s="1" t="n">
-        <v>0.708333</v>
+        <v>0.642857</v>
       </c>
       <c r="K9" t="n">
         <v>7</v>
       </c>
       <c r="L9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M9" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="N9" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="O9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>3.6667</v>
+        <v>3.6429</v>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>3.1667</v>
+        <v>3.2857</v>
       </c>
       <c r="R9" s="2" t="n">
-        <v>30.41666</v>
+        <v>30.5</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>24.25</v>
+        <v>24.71428</v>
       </c>
       <c r="T9" s="1" t="n">
-        <v>0.16279</v>
+        <v>0.340425</v>
       </c>
       <c r="U9" s="1" t="n">
-        <v>0.78125</v>
+        <v>0.673914</v>
       </c>
       <c r="V9" s="1" t="n">
-        <v>0.475106</v>
+        <v>0.549065</v>
       </c>
       <c r="W9" s="1" t="n">
-        <v>0.55004</v>
+        <v>0.55611</v>
       </c>
       <c r="X9" s="1" t="n">
-        <v>0.5496</v>
+        <v>0.56394</v>
       </c>
       <c r="Y9" s="1" t="n">
-        <v>0.55166</v>
+        <v>0.5390200000000001</v>
       </c>
       <c r="Z9" s="1" t="n">
-        <v>0.11469</v>
+        <v>0.08756</v>
       </c>
       <c r="AA9" s="1" t="n">
-        <v>0.88584</v>
+        <v>0.90225</v>
       </c>
       <c r="AB9" s="3" t="n">
-        <v>1.00053</v>
+        <v>0.98981</v>
       </c>
       <c r="AC9" s="1" t="n">
-        <v>0.57507</v>
+        <v>0.49885</v>
       </c>
       <c r="AD9" t="n">
         <v>6</v>
       </c>
       <c r="AE9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AF9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AG9" t="n">
         <v>0</v>
@@ -1989,40 +1989,40 @@
         <v>24</v>
       </c>
       <c r="AI9" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="AJ9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AK9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AL9" t="n">
         <v>3</v>
       </c>
       <c r="AM9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN9" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="AO9" t="n">
         <v>25</v>
       </c>
       <c r="AP9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AQ9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AR9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS9" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="AT9" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="AU9" t="inlineStr">
         <is>
@@ -2031,33 +2031,33 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Seattle Kraken</t>
+          <t>Florida Panthers</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F10" t="n">
         <v>8</v>
@@ -2066,142 +2066,142 @@
         <v>4</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J10" s="1" t="n">
-        <v>0.653846</v>
+        <v>0.642857</v>
       </c>
       <c r="K10" t="n">
         <v>6</v>
       </c>
       <c r="L10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M10" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="N10" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="O10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P10" s="2" t="n">
-        <v>3.8462</v>
+        <v>3.1429</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>3.5385</v>
+        <v>2.7857</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>25.46153</v>
+        <v>28.92857</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>31.07692</v>
+        <v>24.14285</v>
       </c>
       <c r="T10" s="1" t="n">
-        <v>0.227272</v>
+        <v>0.242424</v>
       </c>
       <c r="U10" s="1" t="n">
-        <v>0.6756760000000001</v>
+        <v>0.847458</v>
       </c>
       <c r="V10" s="1" t="n">
-        <v>0.513108</v>
+        <v>0.48112</v>
       </c>
       <c r="W10" s="1" t="n">
-        <v>0.43092</v>
+        <v>0.55627</v>
       </c>
       <c r="X10" s="1" t="n">
-        <v>0.43068</v>
+        <v>0.54428</v>
       </c>
       <c r="Y10" s="1" t="n">
-        <v>0.48576</v>
+        <v>0.58012</v>
       </c>
       <c r="Z10" s="1" t="n">
-        <v>0.14176</v>
+        <v>0.08118</v>
       </c>
       <c r="AA10" s="1" t="n">
-        <v>0.91428</v>
+        <v>0.89473</v>
       </c>
       <c r="AB10" s="3" t="n">
-        <v>1.05604</v>
+        <v>0.9759100000000001</v>
       </c>
       <c r="AC10" s="1" t="n">
-        <v>0.43325</v>
+        <v>0.5698</v>
       </c>
       <c r="AD10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AE10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG10" t="n">
         <v>0</v>
       </c>
       <c r="AH10" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="AI10" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="AJ10" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="AK10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AL10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM10" t="n">
         <v>2</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>1</v>
       </c>
       <c r="AN10" t="n">
         <v>27</v>
       </c>
       <c r="AO10" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="AP10" t="n">
         <v>6</v>
       </c>
       <c r="AQ10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AT10" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="AU10" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ottawa Senators</t>
+          <t>Tampa Bay Lightning</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OTT</t>
+          <t>TBL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2215,13 +2215,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
         <v>8</v>
       </c>
       <c r="G11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
         <v>1</v>
@@ -2230,228 +2230,228 @@
         <v>17</v>
       </c>
       <c r="J11" s="1" t="n">
-        <v>0.607143</v>
+        <v>0.708333</v>
       </c>
       <c r="K11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M11" t="n">
         <v>44</v>
       </c>
       <c r="N11" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="O11" t="n">
+        <v>6</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>3.6667</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>3.1667</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>30.41666</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>24.25</v>
+      </c>
+      <c r="T11" s="1" t="n">
+        <v>0.16279</v>
+      </c>
+      <c r="U11" s="1" t="n">
+        <v>0.78125</v>
+      </c>
+      <c r="V11" s="1" t="n">
+        <v>0.475106</v>
+      </c>
+      <c r="W11" s="1" t="n">
+        <v>0.55004</v>
+      </c>
+      <c r="X11" s="1" t="n">
+        <v>0.5496</v>
+      </c>
+      <c r="Y11" s="1" t="n">
+        <v>0.55166</v>
+      </c>
+      <c r="Z11" s="1" t="n">
+        <v>0.11469</v>
+      </c>
+      <c r="AA11" s="1" t="n">
+        <v>0.88584</v>
+      </c>
+      <c r="AB11" s="3" t="n">
+        <v>1.00053</v>
+      </c>
+      <c r="AC11" s="1" t="n">
+        <v>0.57507</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF11" t="n">
         <v>0</v>
-      </c>
-      <c r="P11" s="2" t="n">
-        <v>3.1429</v>
-      </c>
-      <c r="Q11" s="2" t="n">
-        <v>3.1429</v>
-      </c>
-      <c r="R11" s="2" t="n">
-        <v>25.21428</v>
-      </c>
-      <c r="S11" s="2" t="n">
-        <v>27.07142</v>
-      </c>
-      <c r="T11" s="1" t="n">
-        <v>0.135593</v>
-      </c>
-      <c r="U11" s="1" t="n">
-        <v>0.769231</v>
-      </c>
-      <c r="V11" s="1" t="n">
-        <v>0.521367</v>
-      </c>
-      <c r="W11" s="1" t="n">
-        <v>0.4715</v>
-      </c>
-      <c r="X11" s="1" t="n">
-        <v>0.47434</v>
-      </c>
-      <c r="Y11" s="1" t="n">
-        <v>0.44309</v>
-      </c>
-      <c r="Z11" s="1" t="n">
-        <v>0.108</v>
-      </c>
-      <c r="AA11" s="1" t="n">
-        <v>0.9157</v>
-      </c>
-      <c r="AB11" s="3" t="n">
-        <v>1.0237</v>
-      </c>
-      <c r="AC11" s="1" t="n">
-        <v>0.48825</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>7</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>5</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>2</v>
       </c>
       <c r="AG11" t="n">
         <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AI11" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="AJ11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>20</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>25</v>
+      </c>
+      <c r="AP11" t="n">
         <v>7</v>
       </c>
-      <c r="AK11" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>21</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>22</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>5</v>
-      </c>
       <c r="AQ11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AR11" t="n">
         <v>1</v>
       </c>
       <c r="AS11" t="n">
+        <v>40</v>
+      </c>
+      <c r="AT11" t="n">
         <v>32</v>
       </c>
-      <c r="AT11" t="n">
-        <v>35</v>
-      </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Washington Capitals</t>
+          <t>Seattle Kraken</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F12" t="n">
         <v>8</v>
       </c>
       <c r="G12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>17</v>
+      </c>
+      <c r="J12" s="1" t="n">
+        <v>0.607143</v>
+      </c>
+      <c r="K12" t="n">
+        <v>6</v>
+      </c>
+      <c r="L12" t="n">
+        <v>6</v>
+      </c>
+      <c r="M12" t="n">
+        <v>52</v>
+      </c>
+      <c r="N12" t="n">
+        <v>52</v>
+      </c>
+      <c r="O12" t="n">
         <v>0</v>
       </c>
-      <c r="I12" t="n">
-        <v>16</v>
-      </c>
-      <c r="J12" s="1" t="n">
-        <v>0.666667</v>
-      </c>
-      <c r="K12" t="n">
-        <v>7</v>
-      </c>
-      <c r="L12" t="n">
-        <v>8</v>
-      </c>
-      <c r="M12" t="n">
-        <v>43</v>
-      </c>
-      <c r="N12" t="n">
-        <v>37</v>
-      </c>
-      <c r="O12" t="n">
-        <v>6</v>
-      </c>
       <c r="P12" s="2" t="n">
-        <v>3.5833</v>
+        <v>3.7143</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>3.0833</v>
+        <v>3.7143</v>
       </c>
       <c r="R12" s="2" t="n">
-        <v>27.83333</v>
+        <v>25.21428</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>28</v>
+        <v>30.78571</v>
       </c>
       <c r="T12" s="1" t="n">
-        <v>0.181818</v>
+        <v>0.229166</v>
       </c>
       <c r="U12" s="1" t="n">
-        <v>0.794872</v>
+        <v>0.641026</v>
       </c>
       <c r="V12" s="1" t="n">
-        <v>0.486607</v>
+        <v>0.517919</v>
       </c>
       <c r="W12" s="1" t="n">
-        <v>0.48096</v>
+        <v>0.43055</v>
       </c>
       <c r="X12" s="1" t="n">
-        <v>0.49682</v>
+        <v>0.43312</v>
       </c>
       <c r="Y12" s="1" t="n">
-        <v>0.49175</v>
+        <v>0.48661</v>
       </c>
       <c r="Z12" s="1" t="n">
-        <v>0.12992</v>
+        <v>0.13571</v>
       </c>
       <c r="AA12" s="1" t="n">
-        <v>0.89723</v>
+        <v>0.90801</v>
       </c>
       <c r="AB12" s="3" t="n">
-        <v>1.02715</v>
+        <v>1.04372</v>
       </c>
       <c r="AC12" s="1" t="n">
-        <v>0.43518</v>
+        <v>0.44008</v>
       </c>
       <c r="AD12" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AE12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AF12" t="n">
         <v>2</v>
@@ -2460,64 +2460,64 @@
         <v>0</v>
       </c>
       <c r="AH12" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="AI12" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="AJ12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AK12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AL12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AM12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN12" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="AO12" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="AP12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AQ12" t="n">
         <v>3</v>
       </c>
       <c r="AR12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS12" t="n">
         <v>37</v>
       </c>
       <c r="AT12" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>New Jersey Devils</t>
+          <t>Ottawa Senators</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NJD</t>
+          <t>OTT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2527,11 +2527,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F13" t="n">
         <v>8</v>
@@ -2540,76 +2540,76 @@
         <v>5</v>
       </c>
       <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J13" s="1" t="n">
+        <v>0.607143</v>
+      </c>
+      <c r="K13" t="n">
+        <v>6</v>
+      </c>
+      <c r="L13" t="n">
+        <v>6</v>
+      </c>
+      <c r="M13" t="n">
+        <v>44</v>
+      </c>
+      <c r="N13" t="n">
+        <v>44</v>
+      </c>
+      <c r="O13" t="n">
         <v>0</v>
       </c>
-      <c r="I13" t="n">
-        <v>16</v>
-      </c>
-      <c r="J13" s="1" t="n">
-        <v>0.615385</v>
-      </c>
-      <c r="K13" t="n">
-        <v>6</v>
-      </c>
-      <c r="L13" t="n">
-        <v>8</v>
-      </c>
-      <c r="M13" t="n">
-        <v>43</v>
-      </c>
-      <c r="N13" t="n">
-        <v>38</v>
-      </c>
-      <c r="O13" t="n">
+      <c r="P13" s="2" t="n">
+        <v>3.1429</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>3.1429</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>25.21428</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>27.07142</v>
+      </c>
+      <c r="T13" s="1" t="n">
+        <v>0.135593</v>
+      </c>
+      <c r="U13" s="1" t="n">
+        <v>0.769231</v>
+      </c>
+      <c r="V13" s="1" t="n">
+        <v>0.521367</v>
+      </c>
+      <c r="W13" s="1" t="n">
+        <v>0.4715</v>
+      </c>
+      <c r="X13" s="1" t="n">
+        <v>0.47434</v>
+      </c>
+      <c r="Y13" s="1" t="n">
+        <v>0.44309</v>
+      </c>
+      <c r="Z13" s="1" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="AA13" s="1" t="n">
+        <v>0.9157</v>
+      </c>
+      <c r="AB13" s="3" t="n">
+        <v>1.0237</v>
+      </c>
+      <c r="AC13" s="1" t="n">
+        <v>0.48825</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE13" t="n">
         <v>5</v>
-      </c>
-      <c r="P13" s="2" t="n">
-        <v>3.3077</v>
-      </c>
-      <c r="Q13" s="2" t="n">
-        <v>2.9231</v>
-      </c>
-      <c r="R13" s="2" t="n">
-        <v>32.61538</v>
-      </c>
-      <c r="S13" s="2" t="n">
-        <v>25.07692</v>
-      </c>
-      <c r="T13" s="1" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="U13" s="1" t="n">
-        <v>0.7241379999999999</v>
-      </c>
-      <c r="V13" s="1" t="n">
-        <v>0.503429</v>
-      </c>
-      <c r="W13" s="1" t="n">
-        <v>0.57485</v>
-      </c>
-      <c r="X13" s="1" t="n">
-        <v>0.56753</v>
-      </c>
-      <c r="Y13" s="1" t="n">
-        <v>0.57352</v>
-      </c>
-      <c r="Z13" s="1" t="n">
-        <v>0.08605</v>
-      </c>
-      <c r="AA13" s="1" t="n">
-        <v>0.90151</v>
-      </c>
-      <c r="AB13" s="3" t="n">
-        <v>0.98756</v>
-      </c>
-      <c r="AC13" s="1" t="n">
-        <v>0.52699</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>8</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>6</v>
       </c>
       <c r="AF13" t="n">
         <v>2</v>
@@ -2618,64 +2618,64 @@
         <v>0</v>
       </c>
       <c r="AH13" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="AI13" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="AJ13" t="n">
+        <v>7</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>21</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>22</v>
+      </c>
+      <c r="AP13" t="n">
         <v>5</v>
       </c>
-      <c r="AK13" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>14</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>20</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>7</v>
-      </c>
       <c r="AQ13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS13" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="AT13" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>OT1</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Florida Panthers</t>
+          <t>Washington Capitals</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2685,143 +2685,143 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G14" t="n">
         <v>4</v>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>16</v>
       </c>
       <c r="J14" s="1" t="n">
-        <v>0.615385</v>
+        <v>0.666667</v>
       </c>
       <c r="K14" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M14" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="N14" t="n">
         <v>37</v>
       </c>
       <c r="O14" t="n">
+        <v>6</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>3.5833</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>3.0833</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>27.83333</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>28.08333</v>
+      </c>
+      <c r="T14" s="1" t="n">
+        <v>0.181818</v>
+      </c>
+      <c r="U14" s="1" t="n">
+        <v>0.794872</v>
+      </c>
+      <c r="V14" s="1" t="n">
+        <v>0.486607</v>
+      </c>
+      <c r="W14" s="1" t="n">
+        <v>0.48003</v>
+      </c>
+      <c r="X14" s="1" t="n">
+        <v>0.49682</v>
+      </c>
+      <c r="Y14" s="1" t="n">
+        <v>0.49038</v>
+      </c>
+      <c r="Z14" s="1" t="n">
+        <v>0.12992</v>
+      </c>
+      <c r="AA14" s="1" t="n">
+        <v>0.89763</v>
+      </c>
+      <c r="AB14" s="3" t="n">
+        <v>1.02755</v>
+      </c>
+      <c r="AC14" s="1" t="n">
+        <v>0.43518</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF14" t="n">
         <v>2</v>
-      </c>
-      <c r="P14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q14" s="2" t="n">
-        <v>2.8462</v>
-      </c>
-      <c r="R14" s="2" t="n">
-        <v>28.23076</v>
-      </c>
-      <c r="S14" s="2" t="n">
-        <v>24.15384</v>
-      </c>
-      <c r="T14" s="1" t="n">
-        <v>0.229508</v>
-      </c>
-      <c r="U14" s="1" t="n">
-        <v>0.854546</v>
-      </c>
-      <c r="V14" s="1" t="n">
-        <v>0.469816</v>
-      </c>
-      <c r="W14" s="1" t="n">
-        <v>0.5488</v>
-      </c>
-      <c r="X14" s="1" t="n">
-        <v>0.53645</v>
-      </c>
-      <c r="Y14" s="1" t="n">
-        <v>0.57724</v>
-      </c>
-      <c r="Z14" s="1" t="n">
-        <v>0.08162999999999999</v>
-      </c>
-      <c r="AA14" s="1" t="n">
-        <v>0.89201</v>
-      </c>
-      <c r="AB14" s="3" t="n">
-        <v>0.9736399999999999</v>
-      </c>
-      <c r="AC14" s="1" t="n">
-        <v>0.56346</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>1</v>
       </c>
       <c r="AG14" t="n">
         <v>0</v>
       </c>
       <c r="AH14" t="n">
+        <v>31</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>25</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN14" t="n">
         <v>12</v>
       </c>
-      <c r="AI14" t="n">
-        <v>9</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>10</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>5</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>27</v>
-      </c>
       <c r="AO14" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="AP14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AQ14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR14" t="n">
         <v>0</v>
       </c>
       <c r="AS14" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="AT14" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -2889,7 +2889,7 @@
         <v>26.07692</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>26.23076</v>
+        <v>26.30769</v>
       </c>
       <c r="T15" s="1" t="n">
         <v>0.175</v>
@@ -2901,13 +2901,13 @@
         <v>0.551415</v>
       </c>
       <c r="W15" s="1" t="n">
-        <v>0.51799</v>
+        <v>0.51845</v>
       </c>
       <c r="X15" s="1" t="n">
         <v>0.51105</v>
       </c>
       <c r="Y15" s="1" t="n">
-        <v>0.53776</v>
+        <v>0.53857</v>
       </c>
       <c r="Z15" s="1" t="n">
         <v>0.09293</v>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
         <v>0.509259</v>
       </c>
       <c r="W20" s="1" t="n">
-        <v>0.53385</v>
+        <v>0.53339</v>
       </c>
       <c r="X20" s="1" t="n">
         <v>0.55036</v>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -4153,7 +4153,7 @@
         <v>27.30769</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>28.15384</v>
+        <v>28.07692</v>
       </c>
       <c r="T23" s="1" t="n">
         <v>0.257142</v>
@@ -4177,10 +4177,10 @@
         <v>0.08058</v>
       </c>
       <c r="AA23" s="1" t="n">
-        <v>0.90106</v>
+        <v>0.90071</v>
       </c>
       <c r="AB23" s="3" t="n">
-        <v>0.98164</v>
+        <v>0.98129</v>
       </c>
       <c r="AC23" s="1" t="n">
         <v>0.50497</v>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -4308,7 +4308,7 @@
         <v>3.3077</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>25.6923</v>
+        <v>25.76923</v>
       </c>
       <c r="S24" s="2" t="n">
         <v>29.07692</v>
@@ -4323,22 +4323,22 @@
         <v>0.507362</v>
       </c>
       <c r="W24" s="1" t="n">
-        <v>0.45</v>
+        <v>0.45084</v>
       </c>
       <c r="X24" s="1" t="n">
         <v>0.45747</v>
       </c>
       <c r="Y24" s="1" t="n">
-        <v>0.43211</v>
+        <v>0.43357</v>
       </c>
       <c r="Z24" s="1" t="n">
-        <v>0.075</v>
+        <v>0.07468</v>
       </c>
       <c r="AA24" s="1" t="n">
         <v>0.9069700000000001</v>
       </c>
       <c r="AB24" s="3" t="n">
-        <v>0.98197</v>
+        <v>0.98165</v>
       </c>
       <c r="AC24" s="1" t="n">
         <v>0.46428</v>
@@ -4401,42 +4401,42 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Pittsburgh Penguins</t>
+          <t>Calgary Flames</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E25" t="n">
         <v>13</v>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
         <v>12</v>
@@ -4445,143 +4445,143 @@
         <v>0.461538</v>
       </c>
       <c r="K25" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L25" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M25" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="N25" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="O25" t="n">
-        <v>-1</v>
+        <v>-13</v>
       </c>
       <c r="P25" s="2" t="n">
-        <v>3.3077</v>
+        <v>2.6154</v>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>3.3846</v>
+        <v>3.6154</v>
       </c>
       <c r="R25" s="2" t="n">
-        <v>28.23076</v>
+        <v>28.61538</v>
       </c>
       <c r="S25" s="2" t="n">
-        <v>28</v>
+        <v>29.84615</v>
       </c>
       <c r="T25" s="1" t="n">
-        <v>0.2</v>
+        <v>0.333333</v>
       </c>
       <c r="U25" s="1" t="n">
-        <v>0.84375</v>
+        <v>0.829269</v>
       </c>
       <c r="V25" s="1" t="n">
-        <v>0.454545</v>
+        <v>0.485714</v>
       </c>
       <c r="W25" s="1" t="n">
-        <v>0.51861</v>
+        <v>0.52012</v>
       </c>
       <c r="X25" s="1" t="n">
-        <v>0.51716</v>
+        <v>0.50321</v>
       </c>
       <c r="Y25" s="1" t="n">
-        <v>0.51253</v>
+        <v>0.50461</v>
       </c>
       <c r="Z25" s="1" t="n">
-        <v>0.09764</v>
+        <v>0.06229</v>
       </c>
       <c r="AA25" s="1" t="n">
-        <v>0.89473</v>
+        <v>0.88486</v>
       </c>
       <c r="AB25" s="3" t="n">
-        <v>0.99237</v>
+        <v>0.94715</v>
       </c>
       <c r="AC25" s="1" t="n">
-        <v>0.53708</v>
+        <v>0.49382</v>
       </c>
       <c r="AD25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AE25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AF25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AG25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH25" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="AI25" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="AJ25" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AK25" t="n">
         <v>1</v>
       </c>
       <c r="AL25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AM25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN25" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="AO25" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="AP25" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AQ25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AR25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS25" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="AT25" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="AU25" t="inlineStr">
         <is>
-          <t>OT1</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Anaheim Ducks</t>
+          <t>Pittsburgh Penguins</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ANA</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -4591,82 +4591,82 @@
         <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J26" s="1" t="n">
-        <v>0.423077</v>
+        <v>0.461538</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M26" t="n">
         <v>43</v>
       </c>
       <c r="N26" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="O26" t="n">
-        <v>-7</v>
+        <v>-1</v>
       </c>
       <c r="P26" s="2" t="n">
         <v>3.3077</v>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>3.8462</v>
+        <v>3.3846</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>24.38461</v>
+        <v>28.15384</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>27.92307</v>
+        <v>28.07692</v>
       </c>
       <c r="T26" s="1" t="n">
-        <v>0.285714</v>
+        <v>0.2</v>
       </c>
       <c r="U26" s="1" t="n">
-        <v>0.75</v>
+        <v>0.84375</v>
       </c>
       <c r="V26" s="1" t="n">
-        <v>0.472775</v>
+        <v>0.454545</v>
       </c>
       <c r="W26" s="1" t="n">
-        <v>0.47212</v>
+        <v>0.5182</v>
       </c>
       <c r="X26" s="1" t="n">
-        <v>0.4729</v>
+        <v>0.5165999999999999</v>
       </c>
       <c r="Y26" s="1" t="n">
-        <v>0.45783</v>
+        <v>0.51185</v>
       </c>
       <c r="Z26" s="1" t="n">
-        <v>0.10373</v>
+        <v>0.09797</v>
       </c>
       <c r="AA26" s="1" t="n">
-        <v>0.88888</v>
+        <v>0.8951</v>
       </c>
       <c r="AB26" s="3" t="n">
-        <v>0.99261</v>
+        <v>0.99307</v>
       </c>
       <c r="AC26" s="1" t="n">
-        <v>0.50581</v>
+        <v>0.53708</v>
       </c>
       <c r="AD26" t="n">
         <v>6</v>
       </c>
       <c r="AE26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AF26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AG26" t="n">
         <v>1</v>
@@ -4675,61 +4675,61 @@
         <v>20</v>
       </c>
       <c r="AI26" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="AJ26" t="n">
         <v>7</v>
       </c>
       <c r="AK26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AL26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AM26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN26" t="n">
         <v>23</v>
       </c>
       <c r="AO26" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="AP26" t="n">
         <v>3</v>
       </c>
       <c r="AQ26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS26" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="AT26" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="AU26" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>OT1</t>
         </is>
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Winnipeg Jets</t>
+          <t>Anaheim Ducks</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>WPG</t>
+          <t>ANA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4739,20 +4739,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="E27" t="n">
         <v>13</v>
       </c>
       <c r="F27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
         <v>11</v>
@@ -4764,308 +4764,308 @@
         <v>4</v>
       </c>
       <c r="L27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M27" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N27" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="O27" t="n">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="P27" s="2" t="n">
-        <v>2.4615</v>
+        <v>3.3077</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>3.2308</v>
+        <v>3.8462</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>26.53846</v>
+        <v>24.38461</v>
       </c>
       <c r="S27" s="2" t="n">
-        <v>28.92307</v>
+        <v>27.92307</v>
       </c>
       <c r="T27" s="1" t="n">
-        <v>0.171428</v>
+        <v>0.285714</v>
       </c>
       <c r="U27" s="1" t="n">
-        <v>0.735295</v>
+        <v>0.75</v>
       </c>
       <c r="V27" s="1" t="n">
-        <v>0.467289</v>
+        <v>0.472775</v>
       </c>
       <c r="W27" s="1" t="n">
-        <v>0.48609</v>
+        <v>0.47212</v>
       </c>
       <c r="X27" s="1" t="n">
-        <v>0.48471</v>
+        <v>0.4729</v>
       </c>
       <c r="Y27" s="1" t="n">
-        <v>0.48211</v>
+        <v>0.45783</v>
       </c>
       <c r="Z27" s="1" t="n">
-        <v>0.08921</v>
+        <v>0.10373</v>
       </c>
       <c r="AA27" s="1" t="n">
-        <v>0.91379</v>
+        <v>0.88888</v>
       </c>
       <c r="AB27" s="3" t="n">
-        <v>1.003</v>
+        <v>0.99261</v>
       </c>
       <c r="AC27" s="1" t="n">
-        <v>0.47549</v>
+        <v>0.50581</v>
       </c>
       <c r="AD27" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>20</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>28</v>
+      </c>
+      <c r="AJ27" t="n">
         <v>7</v>
       </c>
-      <c r="AE27" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF27" t="n">
-        <v>4</v>
-      </c>
-      <c r="AG27" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH27" t="n">
-        <v>16</v>
-      </c>
-      <c r="AI27" t="n">
+      <c r="AK27" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN27" t="n">
         <v>23</v>
       </c>
-      <c r="AJ27" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK27" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL27" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM27" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN27" t="n">
-        <v>16</v>
-      </c>
       <c r="AO27" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="AP27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AQ27" t="n">
         <v>6</v>
       </c>
       <c r="AR27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS27" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AT27" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="AU27" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Columbus Blue Jackets</t>
+          <t>Winnipeg Jets</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CBJ</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Western</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Metropolitan</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="E28" t="n">
+        <v>14</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" t="n">
+        <v>7</v>
+      </c>
+      <c r="H28" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" t="n">
         <v>11</v>
       </c>
-      <c r="F28" t="n">
-        <v>5</v>
-      </c>
-      <c r="G28" t="n">
-        <v>6</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>10</v>
-      </c>
       <c r="J28" s="1" t="n">
-        <v>0.454545</v>
+        <v>0.392857</v>
       </c>
       <c r="K28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L28" t="n">
         <v>4</v>
       </c>
       <c r="M28" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="N28" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="O28" t="n">
-        <v>-8</v>
+        <v>-13</v>
       </c>
       <c r="P28" s="2" t="n">
-        <v>2.5455</v>
+        <v>2.4286</v>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>3.2727</v>
+        <v>3.3571</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>25.63636</v>
+        <v>26.35714</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>28</v>
+        <v>29.57142</v>
       </c>
       <c r="T28" s="1" t="n">
-        <v>0.133333</v>
+        <v>0.179487</v>
       </c>
       <c r="U28" s="1" t="n">
-        <v>0.742858</v>
+        <v>0.7179489999999999</v>
       </c>
       <c r="V28" s="1" t="n">
-        <v>0.544615</v>
+        <v>0.460396</v>
       </c>
       <c r="W28" s="1" t="n">
-        <v>0.47938</v>
+        <v>0.4775</v>
       </c>
       <c r="X28" s="1" t="n">
-        <v>0.47238</v>
+        <v>0.477</v>
       </c>
       <c r="Y28" s="1" t="n">
-        <v>0.45692</v>
+        <v>0.47721</v>
       </c>
       <c r="Z28" s="1" t="n">
-        <v>0.08094999999999999</v>
+        <v>0.08802</v>
       </c>
       <c r="AA28" s="1" t="n">
-        <v>0.91213</v>
+        <v>0.91455</v>
       </c>
       <c r="AB28" s="3" t="n">
-        <v>0.99308</v>
+        <v>1.00257</v>
       </c>
       <c r="AC28" s="1" t="n">
-        <v>0.4985</v>
+        <v>0.46788</v>
       </c>
       <c r="AD28" t="n">
         <v>7</v>
       </c>
       <c r="AE28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AF28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH28" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="AI28" t="n">
         <v>23</v>
       </c>
       <c r="AJ28" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AK28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL28" t="n">
         <v>3</v>
       </c>
       <c r="AM28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AN28" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="AO28" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="AP28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AQ28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AR28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS28" t="n">
         <v>22</v>
       </c>
       <c r="AT28" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="AU28" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L4</t>
         </is>
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Calgary Flames</t>
+          <t>Columbus Blue Jackets</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Western</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Metropolitan</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F29" t="n">
         <v>5</v>
       </c>
       <c r="G29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -5074,64 +5074,64 @@
         <v>10</v>
       </c>
       <c r="J29" s="1" t="n">
-        <v>0.416667</v>
+        <v>0.454545</v>
       </c>
       <c r="K29" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M29" t="n">
         <v>28</v>
       </c>
       <c r="N29" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="O29" t="n">
-        <v>-17</v>
+        <v>-8</v>
       </c>
       <c r="P29" s="2" t="n">
-        <v>2.3333</v>
+        <v>2.5455</v>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>3.75</v>
+        <v>3.2727</v>
       </c>
       <c r="R29" s="2" t="n">
-        <v>28.75</v>
+        <v>25.63636</v>
       </c>
       <c r="S29" s="2" t="n">
-        <v>30.5</v>
+        <v>28</v>
       </c>
       <c r="T29" s="1" t="n">
-        <v>0.290322</v>
+        <v>0.133333</v>
       </c>
       <c r="U29" s="1" t="n">
-        <v>0.837838</v>
+        <v>0.742858</v>
       </c>
       <c r="V29" s="1" t="n">
-        <v>0.491501</v>
+        <v>0.544615</v>
       </c>
       <c r="W29" s="1" t="n">
-        <v>0.5165</v>
+        <v>0.47938</v>
       </c>
       <c r="X29" s="1" t="n">
-        <v>0.50114</v>
+        <v>0.47238</v>
       </c>
       <c r="Y29" s="1" t="n">
-        <v>0.5049</v>
+        <v>0.45692</v>
       </c>
       <c r="Z29" s="1" t="n">
-        <v>0.053</v>
+        <v>0.08094999999999999</v>
       </c>
       <c r="AA29" s="1" t="n">
-        <v>0.8807</v>
+        <v>0.91213</v>
       </c>
       <c r="AB29" s="3" t="n">
-        <v>0.9337</v>
+        <v>0.99308</v>
       </c>
       <c r="AC29" s="1" t="n">
-        <v>0.49597</v>
+        <v>0.4985</v>
       </c>
       <c r="AD29" t="n">
         <v>7</v>
@@ -5146,43 +5146,43 @@
         <v>0</v>
       </c>
       <c r="AH29" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="AI29" t="n">
         <v>23</v>
       </c>
       <c r="AJ29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AK29" t="n">
         <v>1</v>
       </c>
       <c r="AL29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AM29" t="n">
         <v>0</v>
       </c>
       <c r="AN29" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AO29" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="AP29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AQ29" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AR29" t="n">
         <v>0</v>
       </c>
       <c r="AS29" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="AT29" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="AU29" t="inlineStr">
         <is>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -5587,7 +5587,7 @@
         <v>0.427613</v>
       </c>
       <c r="W32" s="1" t="n">
-        <v>0.44165</v>
+        <v>0.44215</v>
       </c>
       <c r="X32" s="1" t="n">
         <v>0.4237</v>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-30 08:22</t>
+          <t>2026-10-31 02:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NHL stats 2026-10-31 08:18 ET
</commit_message>
<xml_diff>
--- a/data/nhl_teams.xlsx
+++ b/data/nhl_teams.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2026-10-31 02:59</t>
+          <t>2026-10-31 08:18</t>
         </is>
       </c>
     </row>

</xml_diff>